<commit_message>
Update: Dashboard HTML (13:48:22)
</commit_message>
<xml_diff>
--- a/API데이터_경기_득점_및_도움_기록.xlsx
+++ b/API데이터_경기_득점_및_도움_기록.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F19"/>
+  <dimension ref="A1:F36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -452,7 +452,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-09-23 13:33:47</t>
+          <t>2026-09-24 16:30:57</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -462,29 +462,29 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>셀래스틴</t>
+          <t>UNIT</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2_2</t>
+          <t>3_2</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>무</t>
+          <t>승</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>앙쿠_863246191(2골), 셀래스틴_836158023(2골)</t>
+          <t>앙쿠_848176580(1골), 앙쿠_851194765(1골), 앙쿠_866266039(1골), UNIT_867166676(1골), UNIT_840228251(1골)</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-09-23 13:23:09</t>
+          <t>2026-09-24 16:14:16</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -494,12 +494,12 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>셀래스틴</t>
+          <t>UNIT</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>1_0</t>
+          <t>3_4</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -509,14 +509,14 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>앙쿠_866266039(1골)</t>
+          <t>앙쿠_866266039(1골), 앙쿠_848176580(1골), 앙쿠_863246191(1골), UNIT_867166676(3골), UNIT_848180930(1골)</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-09-23 13:08:58</t>
+          <t>2026-09-24 15:57:54</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -526,12 +526,12 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>ZD장인지참치</t>
+          <t>UNIT</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>3_2</t>
+          <t>4_1</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -541,221 +541,221 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>앙쿠_848176580(1골), 앙쿠_863246191(2골), ZD장인지참치_839200104(1골), ZD장인지참치_840191208(1골)</t>
+          <t>앙쿠_848176580(1골), 앙쿠_863246191(3골), UNIT_848180930(1골)</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-09-23 12:58:26</t>
+          <t>2026-09-24 13:42:25</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>앙쿠</t>
+          <t>UNIT</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>ZD장인지참치</t>
+          <t>셀래스틴</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>2_2</t>
+          <t>4_1</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>무</t>
+          <t>승</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>앙쿠_848176580(1골), 앙쿠_866266039(1골), ZD장인지참치_840191208(2골)</t>
+          <t>UNIT_848180930(2골), UNIT_840228251(1골), UNIT_840192883(1골), 셀래스틴_856277179(1골)</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-09-23 12:28:11</t>
+          <t>2026-09-24 13:30:05</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>0708ManUtd</t>
+          <t>UNIT</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>겐지간지</t>
+          <t>셀래스틴</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>6_2</t>
+          <t>1_3</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>승</t>
+          <t>패</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>0708ManUtd_848183277(1골), 0708ManUtd_863239231(1골), 0708ManUtd_848238794(1골), 0708ManUtd_868001397(2골), 0708ManUtd_848037576(1골), 겐지간지_814231747(2골)</t>
+          <t>UNIT_867166676(1골), 셀래스틴_856277179(1골), 셀래스틴_861005680(1골), 셀래스틴_861142754(1골)</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-09-23 12:19:39</t>
+          <t>2026-09-24 09:29:12</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>아들러</t>
+          <t>여수가스</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>ZD장인지참치</t>
+          <t>ShangHaiPortFC</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>1_5</t>
+          <t>4_2</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>패</t>
+          <t>승</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>아들러_840191208(1골), ZD장인지참치_839200104(2골), ZD장인지참치_840191208(1골), ZD장인지참치_840247263(2골)</t>
+          <t>여수가스_861215732(2골), 여수가스_861162895(2골), ShangHaiPortFC_848031432(1골), ShangHaiPortFC_861051412(1골)</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-09-23 12:19:35</t>
+          <t>2026-09-24 09:16:26</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>경남FC가즈아</t>
+          <t>여수가스</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>콩콩콩룔</t>
+          <t>ShangHaiPortFC</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>2_4</t>
+          <t>4_3</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>패</t>
+          <t>승</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>경남FC가즈아_225238224(2골), 콩콩콩룔_848189505(1골), 콩콩콩룔_866223710(3골)</t>
+          <t>여수가스_861215732(4골), ShangHaiPortFC_845231138(1골), ShangHaiPortFC_848031432(2골)</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-09-23 12:15:41</t>
+          <t>2026-09-24 08:18:47</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>0708ManUtd</t>
+          <t>은안</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>겐지간지</t>
+          <t>방덕</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>4_3</t>
+          <t>2_7</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>승</t>
+          <t>패</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>0708ManUtd_868001397(1골), 0708ManUtd_848037576(2골), 0708ManUtd_848183277(1골), 겐지간지_863256196(1골), 겐지간지_814231747(1골), 겐지간지_845158023(1골)</t>
+          <t>은안_866241236(1골), 은안_848143001(1골), 방덕_868135455(1골), 방덕_868009676(6골)</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-09-23 12:07:26</t>
+          <t>2026-09-24 08:06:58</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>아들러</t>
+          <t>은안</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>ZD장인지참치</t>
+          <t>방덕</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>5_4</t>
+          <t>2_3</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>승</t>
+          <t>패</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>아들러_855232639(1골), 아들러_861000570(1골), 아들러_840191208(2골), 아들러_866251377(1골), ZD장인지참치_839200104(2골), ZD장인지참치_840191208(1골), ZD장인지참치_840256630(1골)</t>
+          <t>은안_856246420(1골), 은안_866241236(1골), 방덕_861077787(1골), 방덕_868009676(1골), 방덕_848007512(1골)</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-09-23 12:05:58</t>
+          <t>2026-09-24 04:51:33</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>경남FC가즈아</t>
+          <t>ZD장인지참치</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>콩콩콩룔</t>
+          <t>용신</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>2_1</t>
+          <t>3_1</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -765,61 +765,61 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>경남FC가즈아_225238224(2골), 콩콩콩룔_867223848(1골)</t>
+          <t>ZD장인지참치_840191208(1골), ZD장인지참치_839200104(2골), 용신_856202126(1골)</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-09-23 11:53:57</t>
+          <t>2026-09-24 04:40:44</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>아들러</t>
+          <t>ZD장인지참치</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>경남FC가즈아</t>
+          <t>용신</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>2_0</t>
+          <t>4_5</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>승</t>
+          <t>패</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>아들러_866251377(1골), 아들러_855232639(1골)</t>
+          <t>ZD장인지참치_840191208(2골), ZD장인지참치_839200104(1골), ZD장인지참치_851240740(1골), 용신_863245367(1골), 용신_820264453(1골), 용신_101173731(1골), 용신_273227535(1골), 용신_856202126(1골)</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-09-23 11:42:25</t>
+          <t>2026-09-24 04:19:09</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>아들러</t>
+          <t>ZD장인지참치</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>경남FC가즈아</t>
+          <t>비주류중독</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>5_0</t>
+          <t>4_4</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -829,29 +829,29 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>아들러_866251377(1골), 아들러_840191208(3골), 아들러_861000570(1골)</t>
+          <t>ZD장인지참치_840191208(2골), ZD장인지참치_839200104(2골), 비주류중독_848006975(1골), 비주류중독_839247699(1골), 비주류중독_825000240(1골), 비주류중독_840052241(1골)</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-09-23 11:29:03</t>
+          <t>2026-09-24 04:02:44</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>앙쿠</t>
+          <t>ZD장인지참치</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>아들러</t>
+          <t>비주류중독</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>1_3</t>
+          <t>0_0</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -859,127 +859,123 @@
           <t>패</t>
         </is>
       </c>
-      <c r="F14" t="inlineStr">
-        <is>
-          <t>앙쿠_851194765(1골), 아들러_840191208(2골), 아들러_852232730(1골)</t>
-        </is>
-      </c>
+      <c r="F14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-09-23 10:27:43</t>
+          <t>2026-09-24 03:45:56</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>아들러</t>
+          <t>UNIT</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>콩콩콩룔</t>
+          <t>ZD장인지참치</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>2_4</t>
+          <t>5_3</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>패</t>
+          <t>승</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>아들러_840191208(2골), 콩콩콩룔_867223848(2골), 콩콩콩룔_866223710(2골)</t>
+          <t>UNIT_867166676(4골), UNIT_848180930(1골), ZD장인지참치_840247263(1골), ZD장인지참치_840191208(2골)</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-09-23 10:15:56</t>
+          <t>2026-09-24 02:48:31</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>아들러</t>
+          <t>여수가스</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>콩콩콩룔</t>
+          <t>방덕</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>2_2</t>
+          <t>3_5</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>무</t>
+          <t>패</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>아들러_840191208(2골), 콩콩콩룔_866223710(1골), 콩콩콩룔_851236496(1골)</t>
+          <t>여수가스_861215732(1골), 여수가스_846188567(1골), 여수가스_828231747(1골), 방덕_827191189(1골), 방덕_101001419(1골), 방덕_861077787(1골), 방덕_848231478(2골)</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-09-23 08:46:09</t>
+          <t>2026-09-23 17:59:32</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>오스트리아</t>
+          <t>0708ManUtd</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>겐지간지</t>
+          <t>여수가스</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>2_1</t>
+          <t>2_3</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>승</t>
+          <t>패</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>오스트리아_291223790(2골), 겐지간지_845158023(1골)</t>
+          <t>0708ManUtd_834239053(1골), 0708ManUtd_851226161(1골), 여수가스_861215732(3골)</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-09-23 08:35:42</t>
+          <t>2026-09-23 17:47:25</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>오스트리아</t>
+          <t>0708ManUtd</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>겐지간지</t>
+          <t>여수가스</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>3_1</t>
+          <t>4_3</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -989,37 +985,581 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>오스트리아_851221671(1골), 오스트리아_864199266(2골), 겐지간지_856237679(1골)</t>
+          <t>0708ManUtd_848037576(1골), 0708ManUtd_868001397(1골), 0708ManUtd_851226161(1골), 0708ManUtd_848238794(1골), 여수가스_861215732(3골)</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
+          <t>2026-09-23 13:33:47</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>앙쿠</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>셀래스틴</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>2_2</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>무</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>앙쿠_863246191(2골), 셀래스틴_836158023(2골)</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>2026-09-23 13:23:09</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>앙쿠</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>셀래스틴</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>1_0</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>승</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>앙쿠_866266039(1골)</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>2026-09-23 13:08:58</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>앙쿠</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>ZD장인지참치</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>3_2</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>승</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>앙쿠_848176580(1골), 앙쿠_863246191(2골), ZD장인지참치_839200104(1골), ZD장인지참치_840191208(1골)</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>2026-09-23 12:58:26</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>앙쿠</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>ZD장인지참치</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>2_2</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>무</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>앙쿠_848176580(1골), 앙쿠_866266039(1골), ZD장인지참치_840191208(2골)</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>2026-09-23 12:28:11</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>0708ManUtd</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>겐지간지</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>6_2</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>승</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>0708ManUtd_848183277(1골), 0708ManUtd_863239231(1골), 0708ManUtd_848238794(1골), 0708ManUtd_868001397(2골), 0708ManUtd_848037576(1골), 겐지간지_814231747(2골)</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>2026-09-23 12:19:39</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>아들러</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>ZD장인지참치</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>1_5</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>패</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>아들러_840191208(1골), ZD장인지참치_839200104(2골), ZD장인지참치_840191208(1골), ZD장인지참치_840247263(2골)</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>2026-09-23 12:19:35</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>경남FC가즈아</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>콩콩콩룔</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>2_4</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>패</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>경남FC가즈아_225238224(2골), 콩콩콩룔_848189505(1골), 콩콩콩룔_866223710(3골)</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>2026-09-23 12:15:41</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>0708ManUtd</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>겐지간지</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>4_3</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>승</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>0708ManUtd_868001397(1골), 0708ManUtd_848037576(2골), 0708ManUtd_848183277(1골), 겐지간지_863256196(1골), 겐지간지_814231747(1골), 겐지간지_845158023(1골)</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>2026-09-23 12:07:26</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>아들러</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>ZD장인지참치</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>5_4</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>승</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>아들러_855232639(1골), 아들러_861000570(1골), 아들러_840191208(2골), 아들러_866251377(1골), ZD장인지참치_839200104(2골), ZD장인지참치_840191208(1골), ZD장인지참치_840256630(1골)</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>2026-09-23 12:05:58</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>경남FC가즈아</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>콩콩콩룔</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>2_1</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>승</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>경남FC가즈아_225238224(2골), 콩콩콩룔_867223848(1골)</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>2026-09-23 11:53:57</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>아들러</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>경남FC가즈아</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>2_0</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>승</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>아들러_866251377(1골), 아들러_855232639(1골)</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>2026-09-23 11:42:25</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>아들러</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>경남FC가즈아</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>5_0</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>승</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>아들러_866251377(1골), 아들러_840191208(3골), 아들러_861000570(1골)</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>2026-09-23 11:29:03</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>앙쿠</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>아들러</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>1_3</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>패</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>앙쿠_851194765(1골), 아들러_840191208(2골), 아들러_852232730(1골)</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>2026-09-23 10:27:43</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>아들러</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>콩콩콩룔</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>2_4</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>패</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>아들러_840191208(2골), 콩콩콩룔_867223848(2골), 콩콩콩룔_866223710(2골)</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>2026-09-23 10:15:56</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>아들러</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>콩콩콩룔</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>2_2</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>무</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>아들러_840191208(2골), 콩콩콩룔_866223710(1골), 콩콩콩룔_851236496(1골)</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>2026-09-23 08:46:09</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>오스트리아</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>겐지간지</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>2_1</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>승</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>오스트리아_291223790(2골), 겐지간지_845158023(1골)</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>2026-09-23 08:35:42</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>오스트리아</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>겐지간지</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>3_1</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>승</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>오스트리아_851221671(1골), 오스트리아_864199266(2골), 겐지간지_856237679(1골)</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
           <t>2026-09-22 14:15:38</t>
         </is>
       </c>
-      <c r="B19" t="inlineStr">
+      <c r="B36" t="inlineStr">
         <is>
           <t>UNIT</t>
         </is>
       </c>
-      <c r="C19" t="inlineStr">
+      <c r="C36" t="inlineStr">
         <is>
           <t>셀래스틴</t>
         </is>
       </c>
-      <c r="D19" t="inlineStr">
+      <c r="D36" t="inlineStr">
         <is>
           <t>1_2</t>
         </is>
       </c>
-      <c r="E19" t="inlineStr">
+      <c r="E36" t="inlineStr">
         <is>
           <t>패</t>
         </is>
       </c>
-      <c r="F19" t="inlineStr">
+      <c r="F36" t="inlineStr">
         <is>
           <t>UNIT_848180930(1골), 셀래스틴_856277179(1골), 셀래스틴_836158023(1골)</t>
         </is>
@@ -1036,7 +1576,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F19"/>
+  <dimension ref="A1:F36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1074,7 +1614,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-09-23 13:33:47</t>
+          <t>2026-09-24 16:30:57</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -1084,29 +1624,29 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>셀래스틴</t>
+          <t>UNIT</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2_2</t>
+          <t>3_2</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>무</t>
+          <t>승</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>앙쿠_856247103(1도움), 앙쿠_814226161(1도움), 셀래스틴_863251854(1도움), 셀래스틴_852241461(1도움)</t>
+          <t>앙쿠_846193747(1도움), 앙쿠_863246191(1도움), 앙쿠_856247103(1도움), UNIT_840192883(1도움), UNIT_840225782(1도움)</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-09-23 13:23:09</t>
+          <t>2026-09-24 16:14:16</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -1116,12 +1656,12 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>셀래스틴</t>
+          <t>UNIT</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>1_0</t>
+          <t>3_4</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -1131,14 +1671,14 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>앙쿠_856247103(1도움)</t>
+          <t>앙쿠_851194765(1도움), 앙쿠_863246191(1도움), 앙쿠_856247103(1도움), UNIT_848135455(1도움), UNIT_863250723(1도움), UNIT_840216150(1도움), UNIT_840210736(1도움)</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-09-23 13:08:58</t>
+          <t>2026-09-24 15:57:54</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -1148,12 +1688,12 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>ZD장인지참치</t>
+          <t>UNIT</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>3_2</t>
+          <t>4_1</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -1163,221 +1703,221 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>앙쿠_851194765(3도움), ZD장인지참치_839200104(1도움), ZD장인지참치_840256630(1도움)</t>
+          <t>앙쿠_851194765(3도움), 앙쿠_848176580(1도움)</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-09-23 12:58:26</t>
+          <t>2026-09-24 13:42:25</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>앙쿠</t>
+          <t>UNIT</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>ZD장인지참치</t>
+          <t>셀래스틴</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>2_2</t>
+          <t>4_1</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>무</t>
+          <t>승</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>앙쿠_856247103(1도움), 앙쿠_814226161(1도움), ZD장인지참치_861182521(1도움), ZD장인지참치_839200104(1도움)</t>
+          <t>UNIT_840210736(1도움), UNIT_840228251(1도움), UNIT_867166676(1도움)</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-09-23 12:28:11</t>
+          <t>2026-09-24 13:30:05</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>0708ManUtd</t>
+          <t>UNIT</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>겐지간지</t>
+          <t>셀래스틴</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>6_2</t>
+          <t>1_3</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>승</t>
+          <t>패</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>0708ManUtd_851226161(2도움), 0708ManUtd_848238794(2도움), 0708ManUtd_868001397(1도움), 겐지간지_856237679(1도움)</t>
+          <t>UNIT_840228251(1도움), 셀래스틴_848230938(1도움), 셀래스틴_863277643(1도움), 셀래스틴_861142754(1도움)</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-09-23 12:19:39</t>
+          <t>2026-09-24 09:29:12</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>아들러</t>
+          <t>여수가스</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>ZD장인지참치</t>
+          <t>ShangHaiPortFC</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>1_5</t>
+          <t>4_2</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>패</t>
+          <t>승</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>아들러_814192318(1도움), ZD장인지참치_861182521(1도움), ZD장인지참치_848210035(1도움), ZD장인지참치_840191208(1도움), ZD장인지참치_840256630(1도움), ZD장인지참치_848199503(1도움)</t>
+          <t>여수가스_845020289(1도움), 여수가스_828231747(1도움), 여수가스_868135455(1도움), 여수가스_846001551(1도움), ShangHaiPortFC_284190813(1도움), ShangHaiPortFC_861051412(1도움)</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-09-23 12:19:35</t>
+          <t>2026-09-24 09:16:26</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>경남FC가즈아</t>
+          <t>여수가스</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>콩콩콩룔</t>
+          <t>ShangHaiPortFC</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>2_4</t>
+          <t>4_3</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>패</t>
+          <t>승</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>경남FC가즈아_853221467(2도움), 콩콩콩룔_867223848(2도움)</t>
+          <t>여수가스_846001551(1도움), 여수가스_828231747(1도움), 여수가스_852274967(1도움), 여수가스_861162895(1도움), ShangHaiPortFC_845231138(1도움), ShangHaiPortFC_861051412(1도움)</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-09-23 12:15:41</t>
+          <t>2026-09-24 08:18:47</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>0708ManUtd</t>
+          <t>은안</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>겐지간지</t>
+          <t>방덕</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>4_3</t>
+          <t>2_7</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>승</t>
+          <t>패</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>0708ManUtd_868001397(2도움), 0708ManUtd_848037576(1도움), 0708ManUtd_851226161(1도움), 겐지간지_861001668(1도움), 겐지간지_826247635(1도움), 겐지간지_852231443(1도움)</t>
+          <t>은안_856251517(1도움), 방덕_868135455(1도움), 방덕_848231478(1도움), 방덕_848007512(1도움), 방덕_861077787(2도움), 방덕_868009676(1도움), 방덕_856226268(1도움)</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-09-23 12:07:26</t>
+          <t>2026-09-24 08:06:58</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>아들러</t>
+          <t>은안</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>ZD장인지참치</t>
+          <t>방덕</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>5_4</t>
+          <t>2_3</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>승</t>
+          <t>패</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>아들러_855232639(2도움), 아들러_861000570(1도움), 아들러_840191208(1도움), ZD장인지참치_839200104(1도움), ZD장인지참치_848199503(1도움), ZD장인지참치_861182521(2도움)</t>
+          <t>은안_856246420(1도움), 은안_848231866(1도움), 방덕_861077787(1도움), 방덕_848007512(1도움)</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-09-23 12:05:58</t>
+          <t>2026-09-24 04:51:33</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>경남FC가즈아</t>
+          <t>ZD장인지참치</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>콩콩콩룔</t>
+          <t>용신</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>2_1</t>
+          <t>3_1</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -1387,61 +1927,61 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>경남FC가즈아_277205156(1도움), 경남FC가즈아_518251161(1도움), 콩콩콩룔_851236496(1도움)</t>
+          <t>ZD장인지참치_848210035(1도움), ZD장인지참치_848199503(1도움), ZD장인지참치_839200104(1도움), 용신_866200104(1도움)</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-09-23 11:53:57</t>
+          <t>2026-09-24 04:40:44</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>아들러</t>
+          <t>ZD장인지참치</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>경남FC가즈아</t>
+          <t>용신</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>2_0</t>
+          <t>4_5</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>승</t>
+          <t>패</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>아들러_861000570(2도움)</t>
+          <t>ZD장인지참치_840191208(2도움), ZD장인지참치_839200104(1도움), ZD장인지참치_851240740(1도움), 용신_863245367(2도움), 용신_273227535(1도움), 용신_848216267(1도움)</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-09-23 11:42:25</t>
+          <t>2026-09-24 04:19:09</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>아들러</t>
+          <t>ZD장인지참치</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>경남FC가즈아</t>
+          <t>비주류중독</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>5_0</t>
+          <t>4_4</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -1451,29 +1991,29 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>아들러_866251377(1도움), 아들러_855232639(1도움), 아들러_840191208(1도움), 아들러_840208574(1도움)</t>
+          <t>ZD장인지참치_861182521(2도움), ZD장인지참치_840256630(1도움), ZD장인지참치_851240740(1도움), 비주류중독_848006975(1도움), 비주류중독_839247699(1도움), 비주류중독_852253149(1도움)</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-09-23 11:29:03</t>
+          <t>2026-09-24 04:02:44</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>앙쿠</t>
+          <t>ZD장인지참치</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>아들러</t>
+          <t>비주류중독</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>1_3</t>
+          <t>0_0</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -1481,127 +2021,123 @@
           <t>패</t>
         </is>
       </c>
-      <c r="F14" t="inlineStr">
-        <is>
-          <t>앙쿠_863246191(1도움), 아들러_840191208(1도움), 아들러_852232730(1도움)</t>
-        </is>
-      </c>
+      <c r="F14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-09-23 10:27:43</t>
+          <t>2026-09-24 03:45:56</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>아들러</t>
+          <t>UNIT</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>콩콩콩룔</t>
+          <t>ZD장인지참치</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>2_4</t>
+          <t>5_3</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>패</t>
+          <t>승</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>아들러_866251377(1도움), 아들러_852232730(1도움), 콩콩콩룔_867220502(1도움), 콩콩콩룔_867223848(1도움), 콩콩콩룔_866223710(1도움), 콩콩콩룔_861006235(1도움)</t>
+          <t>UNIT_840228251(1도움), UNIT_840225782(1도움), UNIT_848135455(1도움), UNIT_848180930(1도움), UNIT_840192883(1도움), ZD장인지참치_848210035(1도움), ZD장인지참치_839200104(2도움)</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-09-23 10:15:56</t>
+          <t>2026-09-24 02:48:31</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>아들러</t>
+          <t>여수가스</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>콩콩콩룔</t>
+          <t>방덕</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>2_2</t>
+          <t>3_5</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>무</t>
+          <t>패</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>아들러_291225126(2도움), 콩콩콩룔_867220502(1도움)</t>
+          <t>여수가스_861162895(1도움), 여수가스_868135455(1도움), 방덕_868009676(1도움), 방덕_101001419(1도움), 방덕_863184200(1도움), 방덕_867001040(1도움)</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-09-23 08:46:09</t>
+          <t>2026-09-23 17:59:32</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>오스트리아</t>
+          <t>0708ManUtd</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>겐지간지</t>
+          <t>여수가스</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>2_1</t>
+          <t>2_3</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>승</t>
+          <t>패</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>오스트리아_864182152(1도움), 겐지간지_826247635(1도움)</t>
+          <t>0708ManUtd_834239053(1도움), 0708ManUtd_868001397(1도움), 여수가스_868135455(1도움), 여수가스_828231747(1도움), 여수가스_845020289(1도움)</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-09-23 08:35:42</t>
+          <t>2026-09-23 17:47:25</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>오스트리아</t>
+          <t>0708ManUtd</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>겐지간지</t>
+          <t>여수가스</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>3_1</t>
+          <t>4_3</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -1611,37 +2147,581 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>오스트리아_864140057(2도움), 겐지간지_814231747(1도움)</t>
+          <t>0708ManUtd_834239053(1도움), 0708ManUtd_868001397(1도움), 0708ManUtd_851226161(1도움), 0708ManUtd_848238794(1도움), 여수가스_861162895(1도움), 여수가스_828231747(1도움)</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
+          <t>2026-09-23 13:33:47</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>앙쿠</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>셀래스틴</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>2_2</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>무</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>앙쿠_856247103(1도움), 앙쿠_814226161(1도움), 셀래스틴_863251854(1도움), 셀래스틴_852241461(1도움)</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>2026-09-23 13:23:09</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>앙쿠</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>셀래스틴</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>1_0</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>승</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>앙쿠_856247103(1도움)</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>2026-09-23 13:08:58</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>앙쿠</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>ZD장인지참치</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>3_2</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>승</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>앙쿠_851194765(3도움), ZD장인지참치_839200104(1도움), ZD장인지참치_840256630(1도움)</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>2026-09-23 12:58:26</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>앙쿠</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>ZD장인지참치</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>2_2</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>무</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>앙쿠_856247103(1도움), 앙쿠_814226161(1도움), ZD장인지참치_861182521(1도움), ZD장인지참치_839200104(1도움)</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>2026-09-23 12:28:11</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>0708ManUtd</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>겐지간지</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>6_2</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>승</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>0708ManUtd_851226161(2도움), 0708ManUtd_848238794(2도움), 0708ManUtd_868001397(1도움), 겐지간지_856237679(1도움)</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>2026-09-23 12:19:39</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>아들러</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>ZD장인지참치</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>1_5</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>패</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>아들러_814192318(1도움), ZD장인지참치_861182521(1도움), ZD장인지참치_848210035(1도움), ZD장인지참치_840191208(1도움), ZD장인지참치_840256630(1도움), ZD장인지참치_848199503(1도움)</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>2026-09-23 12:19:35</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>경남FC가즈아</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>콩콩콩룔</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>2_4</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>패</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>경남FC가즈아_853221467(2도움), 콩콩콩룔_867223848(2도움)</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>2026-09-23 12:15:41</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>0708ManUtd</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>겐지간지</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>4_3</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>승</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>0708ManUtd_868001397(2도움), 0708ManUtd_848037576(1도움), 0708ManUtd_851226161(1도움), 겐지간지_861001668(1도움), 겐지간지_826247635(1도움), 겐지간지_852231443(1도움)</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>2026-09-23 12:07:26</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>아들러</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>ZD장인지참치</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>5_4</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>승</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>아들러_855232639(2도움), 아들러_861000570(1도움), 아들러_840191208(1도움), ZD장인지참치_839200104(1도움), ZD장인지참치_848199503(1도움), ZD장인지참치_861182521(2도움)</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>2026-09-23 12:05:58</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>경남FC가즈아</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>콩콩콩룔</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>2_1</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>승</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>경남FC가즈아_277205156(1도움), 경남FC가즈아_518251161(1도움), 콩콩콩룔_851236496(1도움)</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>2026-09-23 11:53:57</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>아들러</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>경남FC가즈아</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>2_0</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>승</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>아들러_861000570(2도움)</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>2026-09-23 11:42:25</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>아들러</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>경남FC가즈아</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>5_0</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>승</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>아들러_866251377(1도움), 아들러_855232639(1도움), 아들러_840191208(1도움), 아들러_840208574(1도움)</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>2026-09-23 11:29:03</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>앙쿠</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>아들러</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>1_3</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>패</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>앙쿠_863246191(1도움), 아들러_840191208(1도움), 아들러_852232730(1도움)</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>2026-09-23 10:27:43</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>아들러</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>콩콩콩룔</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>2_4</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>패</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>아들러_866251377(1도움), 아들러_852232730(1도움), 콩콩콩룔_867220502(1도움), 콩콩콩룔_867223848(1도움), 콩콩콩룔_866223710(1도움), 콩콩콩룔_861006235(1도움)</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>2026-09-23 10:15:56</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>아들러</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>콩콩콩룔</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>2_2</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>무</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>아들러_291225126(2도움), 콩콩콩룔_867220502(1도움)</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>2026-09-23 08:46:09</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>오스트리아</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>겐지간지</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>2_1</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>승</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>오스트리아_864182152(1도움), 겐지간지_826247635(1도움)</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>2026-09-23 08:35:42</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>오스트리아</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>겐지간지</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>3_1</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>승</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>오스트리아_864140057(2도움), 겐지간지_814231747(1도움)</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
           <t>2026-09-22 14:15:38</t>
         </is>
       </c>
-      <c r="B19" t="inlineStr">
+      <c r="B36" t="inlineStr">
         <is>
           <t>UNIT</t>
         </is>
       </c>
-      <c r="C19" t="inlineStr">
+      <c r="C36" t="inlineStr">
         <is>
           <t>셀래스틴</t>
         </is>
       </c>
-      <c r="D19" t="inlineStr">
+      <c r="D36" t="inlineStr">
         <is>
           <t>1_2</t>
         </is>
       </c>
-      <c r="E19" t="inlineStr">
+      <c r="E36" t="inlineStr">
         <is>
           <t>패</t>
         </is>
       </c>
-      <c r="F19" t="inlineStr">
+      <c r="F36" t="inlineStr">
         <is>
           <t>UNIT_840192883(1도움), 셀래스틴_852277643(1도움), 셀래스틴_852241461(1도움)</t>
         </is>

</xml_diff>

<commit_message>
Update: Dashboard HTML (23:31:43)
</commit_message>
<xml_diff>
--- a/API데이터_경기_득점_및_도움_기록.xlsx
+++ b/API데이터_경기_득점_및_도움_기록.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F36"/>
+  <dimension ref="A1:F46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -452,22 +452,22 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-09-24 16:30:57</t>
+          <t>2026-09-26 12:19:23</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>앙쿠</t>
+          <t>ZD장인지참치</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>UNIT</t>
+          <t>셀래스틴</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>3_2</t>
+          <t>6_4</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -477,29 +477,29 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>앙쿠_848176580(1골), 앙쿠_851194765(1골), 앙쿠_866266039(1골), UNIT_867166676(1골), UNIT_840228251(1골)</t>
+          <t>ZD장인지참치_851240740(1골), ZD장인지참치_840191208(4골), ZD장인지참치_839200104(1골), 셀래스틴_846001551(1골), 셀래스틴_848194765(2골), 셀래스틴_852241461(1골)</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-09-24 16:14:16</t>
+          <t>2026-09-26 12:08:13</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>앙쿠</t>
+          <t>ZD장인지참치</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>UNIT</t>
+          <t>셀래스틴</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>3_4</t>
+          <t>2_1</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -509,78 +509,78 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>앙쿠_866266039(1골), 앙쿠_848176580(1골), 앙쿠_863246191(1골), UNIT_867166676(3골), UNIT_848180930(1골)</t>
+          <t>ZD장인지참치_840191208(2골), 셀래스틴_861005680(1골)</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-09-24 15:57:54</t>
+          <t>2026-09-26 08:26:23</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>앙쿠</t>
+          <t>오스트리아</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>UNIT</t>
+          <t>Special블루</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>4_1</t>
+          <t>1_3</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>승</t>
+          <t>패</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>앙쿠_848176580(1골), 앙쿠_863246191(3골), UNIT_848180930(1골)</t>
+          <t>오스트리아_851221671(1골), Special블루_856246669(1골), Special블루_863248148(1골), Special블루_855241651(1골)</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-09-24 13:42:25</t>
+          <t>2026-09-25 15:57:51</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>UNIT</t>
+          <t>셀래스틴</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>셀래스틴</t>
+          <t>Voor</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>4_1</t>
+          <t>0_3</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>승</t>
+          <t>패</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>UNIT_848180930(2골), UNIT_840228251(1골), UNIT_840192883(1골), 셀래스틴_856277179(1골)</t>
+          <t>Voor_845009676(1골), Voor_845247090(1골), Voor_852233700(1골)</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-09-24 13:30:05</t>
+          <t>2026-09-25 09:45:28</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -590,12 +590,12 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>셀래스틴</t>
+          <t>방덕</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>1_3</t>
+          <t>3_4</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -605,29 +605,29 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>UNIT_867166676(1골), 셀래스틴_856277179(1골), 셀래스틴_861005680(1골), 셀래스틴_861142754(1골)</t>
+          <t>UNIT_848180930(1골), UNIT_840228251(2골), 방덕_848007512(1골), 방덕_868009676(3골)</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-09-24 09:29:12</t>
+          <t>2026-09-25 09:33:41</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>여수가스</t>
+          <t>UNIT</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>ShangHaiPortFC</t>
+          <t>방덕</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>4_2</t>
+          <t>3_2</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -637,51 +637,51 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>여수가스_861215732(2골), 여수가스_861162895(2골), ShangHaiPortFC_848031432(1골), ShangHaiPortFC_861051412(1골)</t>
+          <t>UNIT_848180930(1골), UNIT_840192883(1골), UNIT_867166676(1골), 방덕_861077787(1골), 방덕_868009676(1골)</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-09-24 09:16:26</t>
+          <t>2026-09-25 09:22:20</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>여수가스</t>
+          <t>UNIT</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>ShangHaiPortFC</t>
+          <t>방덕</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>4_3</t>
+          <t>2_3</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>승</t>
+          <t>패</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>여수가스_861215732(4골), ShangHaiPortFC_845231138(1골), ShangHaiPortFC_848031432(2골)</t>
+          <t>UNIT_867166676(1골), UNIT_840192883(1골), 방덕_868009676(1골), 방덕_868135455(1골), 방덕_861077787(1골)</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-09-24 08:18:47</t>
+          <t>2026-09-25 09:10:55</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>은안</t>
+          <t>UNIT</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -691,29 +691,29 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>2_7</t>
+          <t>1_1</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>패</t>
+          <t>무</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>은안_866241236(1골), 은안_848143001(1골), 방덕_868135455(1골), 방덕_868009676(6골)</t>
+          <t>UNIT_840192883(1골), 방덕_868009676(1골)</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-09-24 08:06:58</t>
+          <t>2026-09-25 08:53:47</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>은안</t>
+          <t>UNIT</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -723,103 +723,103 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>2_3</t>
+          <t>2_2</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>패</t>
+          <t>무</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>은안_856246420(1골), 은안_866241236(1골), 방덕_861077787(1골), 방덕_868009676(1골), 방덕_848007512(1골)</t>
+          <t>UNIT_848180930(1골), UNIT_840192883(1골), 방덕_861077787(1골), 방덕_101001419(1골)</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-09-24 04:51:33</t>
+          <t>2026-09-25 08:42:15</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>ZD장인지참치</t>
+          <t>UNIT</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>용신</t>
+          <t>방덕</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>3_1</t>
+          <t>2_3</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>승</t>
+          <t>패</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>ZD장인지참치_840191208(1골), ZD장인지참치_839200104(2골), 용신_856202126(1골)</t>
+          <t>UNIT_867166676(2골), 방덕_868135455(2골), 방덕_856228093(1골)</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-09-24 04:40:44</t>
+          <t>2026-09-24 16:30:57</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>ZD장인지참치</t>
+          <t>앙쿠</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>용신</t>
+          <t>UNIT</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>4_5</t>
+          <t>3_2</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>패</t>
+          <t>승</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>ZD장인지참치_840191208(2골), ZD장인지참치_839200104(1골), ZD장인지참치_851240740(1골), 용신_863245367(1골), 용신_820264453(1골), 용신_101173731(1골), 용신_273227535(1골), 용신_856202126(1골)</t>
+          <t>앙쿠_848176580(1골), 앙쿠_851194765(1골), 앙쿠_866266039(1골), UNIT_867166676(1골), UNIT_840228251(1골)</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-09-24 04:19:09</t>
+          <t>2026-09-24 16:14:16</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>ZD장인지참치</t>
+          <t>앙쿠</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>비주류중독</t>
+          <t>UNIT</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>4_4</t>
+          <t>3_4</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -829,42 +829,46 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>ZD장인지참치_840191208(2골), ZD장인지참치_839200104(2골), 비주류중독_848006975(1골), 비주류중독_839247699(1골), 비주류중독_825000240(1골), 비주류중독_840052241(1골)</t>
+          <t>앙쿠_866266039(1골), 앙쿠_848176580(1골), 앙쿠_863246191(1골), UNIT_867166676(3골), UNIT_848180930(1골)</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-09-24 04:02:44</t>
+          <t>2026-09-24 15:57:54</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>ZD장인지참치</t>
+          <t>앙쿠</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>비주류중독</t>
+          <t>UNIT</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>0_0</t>
+          <t>4_1</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>패</t>
-        </is>
-      </c>
-      <c r="F14" t="inlineStr"/>
+          <t>승</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>앙쿠_848176580(1골), 앙쿠_863246191(3골), UNIT_848180930(1골)</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-09-24 03:45:56</t>
+          <t>2026-09-24 13:42:25</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -874,12 +878,12 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>ZD장인지참치</t>
+          <t>셀래스틴</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>5_3</t>
+          <t>4_1</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -889,29 +893,29 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>UNIT_867166676(4골), UNIT_848180930(1골), ZD장인지참치_840247263(1골), ZD장인지참치_840191208(2골)</t>
+          <t>UNIT_848180930(2골), UNIT_840228251(1골), UNIT_840192883(1골), 셀래스틴_856277179(1골)</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-09-24 02:48:31</t>
+          <t>2026-09-24 13:30:05</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>여수가스</t>
+          <t>UNIT</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>방덕</t>
+          <t>셀래스틴</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>3_5</t>
+          <t>1_3</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -921,56 +925,56 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>여수가스_861215732(1골), 여수가스_846188567(1골), 여수가스_828231747(1골), 방덕_827191189(1골), 방덕_101001419(1골), 방덕_861077787(1골), 방덕_848231478(2골)</t>
+          <t>UNIT_867166676(1골), 셀래스틴_856277179(1골), 셀래스틴_861005680(1골), 셀래스틴_861142754(1골)</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-09-23 17:59:32</t>
+          <t>2026-09-24 09:29:12</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>0708ManUtd</t>
+          <t>여수가스</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>여수가스</t>
+          <t>ShangHaiPortFC</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>2_3</t>
+          <t>4_2</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>패</t>
+          <t>승</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>0708ManUtd_834239053(1골), 0708ManUtd_851226161(1골), 여수가스_861215732(3골)</t>
+          <t>여수가스_861215732(2골), 여수가스_861162895(2골), ShangHaiPortFC_848031432(1골), ShangHaiPortFC_861051412(1골)</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-09-23 17:47:25</t>
+          <t>2026-09-24 09:16:26</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>0708ManUtd</t>
+          <t>여수가스</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>여수가스</t>
+          <t>ShangHaiPortFC</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -985,93 +989,93 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>0708ManUtd_848037576(1골), 0708ManUtd_868001397(1골), 0708ManUtd_851226161(1골), 0708ManUtd_848238794(1골), 여수가스_861215732(3골)</t>
+          <t>여수가스_861215732(4골), ShangHaiPortFC_845231138(1골), ShangHaiPortFC_848031432(2골)</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-09-23 13:33:47</t>
+          <t>2026-09-24 08:18:47</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>앙쿠</t>
+          <t>은안</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>셀래스틴</t>
+          <t>방덕</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>2_2</t>
+          <t>2_7</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>무</t>
+          <t>패</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>앙쿠_863246191(2골), 셀래스틴_836158023(2골)</t>
+          <t>은안_866241236(1골), 은안_848143001(1골), 방덕_868135455(1골), 방덕_868009676(6골)</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-09-23 13:23:09</t>
+          <t>2026-09-24 08:06:58</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>앙쿠</t>
+          <t>은안</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>셀래스틴</t>
+          <t>방덕</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>1_0</t>
+          <t>2_3</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>승</t>
+          <t>패</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>앙쿠_866266039(1골)</t>
+          <t>은안_856246420(1골), 은안_866241236(1골), 방덕_861077787(1골), 방덕_868009676(1골), 방덕_848007512(1골)</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-09-23 13:08:58</t>
+          <t>2026-09-24 04:51:33</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>앙쿠</t>
+          <t>ZD장인지참치</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>ZD장인지참치</t>
+          <t>용신</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>3_2</t>
+          <t>3_1</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -1081,61 +1085,61 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>앙쿠_848176580(1골), 앙쿠_863246191(2골), ZD장인지참치_839200104(1골), ZD장인지참치_840191208(1골)</t>
+          <t>ZD장인지참치_840191208(1골), ZD장인지참치_839200104(2골), 용신_856202126(1골)</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2026-09-23 12:58:26</t>
+          <t>2026-09-24 04:40:44</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>앙쿠</t>
+          <t>ZD장인지참치</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>ZD장인지참치</t>
+          <t>용신</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>2_2</t>
+          <t>4_5</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>무</t>
+          <t>패</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>앙쿠_848176580(1골), 앙쿠_866266039(1골), ZD장인지참치_840191208(2골)</t>
+          <t>ZD장인지참치_840191208(2골), ZD장인지참치_839200104(1골), ZD장인지참치_851240740(1골), 용신_863245367(1골), 용신_820264453(1골), 용신_101173731(1골), 용신_273227535(1골), 용신_856202126(1골)</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-09-23 12:28:11</t>
+          <t>2026-09-24 04:19:09</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>0708ManUtd</t>
+          <t>ZD장인지참치</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>겐지간지</t>
+          <t>비주류중독</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>6_2</t>
+          <t>4_4</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -1145,29 +1149,29 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>0708ManUtd_848183277(1골), 0708ManUtd_863239231(1골), 0708ManUtd_848238794(1골), 0708ManUtd_868001397(2골), 0708ManUtd_848037576(1골), 겐지간지_814231747(2골)</t>
+          <t>ZD장인지참치_840191208(2골), ZD장인지참치_839200104(2골), 비주류중독_848006975(1골), 비주류중독_839247699(1골), 비주류중독_825000240(1골), 비주류중독_840052241(1골)</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>2026-09-23 12:19:39</t>
+          <t>2026-09-24 04:02:44</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>아들러</t>
+          <t>ZD장인지참치</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>ZD장인지참치</t>
+          <t>비주류중독</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>1_5</t>
+          <t>0_0</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -1175,127 +1179,123 @@
           <t>패</t>
         </is>
       </c>
-      <c r="F24" t="inlineStr">
-        <is>
-          <t>아들러_840191208(1골), ZD장인지참치_839200104(2골), ZD장인지참치_840191208(1골), ZD장인지참치_840247263(2골)</t>
-        </is>
-      </c>
+      <c r="F24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-09-23 12:19:35</t>
+          <t>2026-09-24 03:45:56</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>경남FC가즈아</t>
+          <t>UNIT</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>콩콩콩룔</t>
+          <t>ZD장인지참치</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>2_4</t>
+          <t>5_3</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>패</t>
+          <t>승</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>경남FC가즈아_225238224(2골), 콩콩콩룔_848189505(1골), 콩콩콩룔_866223710(3골)</t>
+          <t>UNIT_867166676(4골), UNIT_848180930(1골), ZD장인지참치_840247263(1골), ZD장인지참치_840191208(2골)</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>2026-09-23 12:15:41</t>
+          <t>2026-09-24 02:48:31</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>0708ManUtd</t>
+          <t>여수가스</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>겐지간지</t>
+          <t>방덕</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>4_3</t>
+          <t>3_5</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>승</t>
+          <t>패</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>0708ManUtd_868001397(1골), 0708ManUtd_848037576(2골), 0708ManUtd_848183277(1골), 겐지간지_863256196(1골), 겐지간지_814231747(1골), 겐지간지_845158023(1골)</t>
+          <t>여수가스_861215732(1골), 여수가스_846188567(1골), 여수가스_828231747(1골), 방덕_827191189(1골), 방덕_101001419(1골), 방덕_861077787(1골), 방덕_848231478(2골)</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-09-23 12:07:26</t>
+          <t>2026-09-23 17:59:32</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>아들러</t>
+          <t>0708ManUtd</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>ZD장인지참치</t>
+          <t>여수가스</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>5_4</t>
+          <t>2_3</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>승</t>
+          <t>패</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>아들러_855232639(1골), 아들러_861000570(1골), 아들러_840191208(2골), 아들러_866251377(1골), ZD장인지참치_839200104(2골), ZD장인지참치_840191208(1골), ZD장인지참치_840256630(1골)</t>
+          <t>0708ManUtd_834239053(1골), 0708ManUtd_851226161(1골), 여수가스_861215732(3골)</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>2026-09-23 12:05:58</t>
+          <t>2026-09-23 17:47:25</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>경남FC가즈아</t>
+          <t>0708ManUtd</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>콩콩콩룔</t>
+          <t>여수가스</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>2_1</t>
+          <t>4_3</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
@@ -1305,61 +1305,61 @@
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>경남FC가즈아_225238224(2골), 콩콩콩룔_867223848(1골)</t>
+          <t>0708ManUtd_848037576(1골), 0708ManUtd_868001397(1골), 0708ManUtd_851226161(1골), 0708ManUtd_848238794(1골), 여수가스_861215732(3골)</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-09-23 11:53:57</t>
+          <t>2026-09-23 13:33:47</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>아들러</t>
+          <t>앙쿠</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>경남FC가즈아</t>
+          <t>셀래스틴</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>2_0</t>
+          <t>2_2</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>승</t>
+          <t>무</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>아들러_866251377(1골), 아들러_855232639(1골)</t>
+          <t>앙쿠_863246191(2골), 셀래스틴_836158023(2골)</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>2026-09-23 11:42:25</t>
+          <t>2026-09-23 13:23:09</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>아들러</t>
+          <t>앙쿠</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>경남FC가즈아</t>
+          <t>셀래스틴</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>5_0</t>
+          <t>1_0</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
@@ -1369,14 +1369,14 @@
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>아들러_866251377(1골), 아들러_840191208(3골), 아들러_861000570(1골)</t>
+          <t>앙쿠_866266039(1골)</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-09-23 11:29:03</t>
+          <t>2026-09-23 13:08:58</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -1386,180 +1386,500 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>아들러</t>
+          <t>ZD장인지참치</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>1_3</t>
+          <t>3_2</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>패</t>
+          <t>승</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>앙쿠_851194765(1골), 아들러_840191208(2골), 아들러_852232730(1골)</t>
+          <t>앙쿠_848176580(1골), 앙쿠_863246191(2골), ZD장인지참치_839200104(1골), ZD장인지참치_840191208(1골)</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>2026-09-23 10:27:43</t>
+          <t>2026-09-23 12:58:26</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>아들러</t>
+          <t>앙쿠</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>콩콩콩룔</t>
+          <t>ZD장인지참치</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>2_4</t>
+          <t>2_2</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>패</t>
+          <t>무</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>아들러_840191208(2골), 콩콩콩룔_867223848(2골), 콩콩콩룔_866223710(2골)</t>
+          <t>앙쿠_848176580(1골), 앙쿠_866266039(1골), ZD장인지참치_840191208(2골)</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-09-23 10:15:56</t>
+          <t>2026-09-23 12:28:11</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>아들러</t>
+          <t>0708ManUtd</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>콩콩콩룔</t>
+          <t>겐지간지</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>2_2</t>
+          <t>6_2</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>무</t>
+          <t>승</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>아들러_840191208(2골), 콩콩콩룔_866223710(1골), 콩콩콩룔_851236496(1골)</t>
+          <t>0708ManUtd_848183277(1골), 0708ManUtd_863239231(1골), 0708ManUtd_848238794(1골), 0708ManUtd_868001397(2골), 0708ManUtd_848037576(1골), 겐지간지_814231747(2골)</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>2026-09-23 08:46:09</t>
+          <t>2026-09-23 12:19:39</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>오스트리아</t>
+          <t>아들러</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>겐지간지</t>
+          <t>ZD장인지참치</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>2_1</t>
+          <t>1_5</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>승</t>
+          <t>패</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>오스트리아_291223790(2골), 겐지간지_845158023(1골)</t>
+          <t>아들러_840191208(1골), ZD장인지참치_839200104(2골), ZD장인지참치_840191208(1골), ZD장인지참치_840247263(2골)</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-09-23 08:35:42</t>
+          <t>2026-09-23 12:19:35</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>오스트리아</t>
+          <t>경남FC가즈아</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>겐지간지</t>
+          <t>콩콩콩룔</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>3_1</t>
+          <t>2_4</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>승</t>
+          <t>패</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>오스트리아_851221671(1골), 오스트리아_864199266(2골), 겐지간지_856237679(1골)</t>
+          <t>경남FC가즈아_225238224(2골), 콩콩콩룔_848189505(1골), 콩콩콩룔_866223710(3골)</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
+          <t>2026-09-23 12:15:41</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>0708ManUtd</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>겐지간지</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>4_3</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>승</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>0708ManUtd_868001397(1골), 0708ManUtd_848037576(2골), 0708ManUtd_848183277(1골), 겐지간지_863256196(1골), 겐지간지_814231747(1골), 겐지간지_845158023(1골)</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>2026-09-23 12:07:26</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>아들러</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>ZD장인지참치</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>5_4</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>승</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>아들러_855232639(1골), 아들러_861000570(1골), 아들러_840191208(2골), 아들러_866251377(1골), ZD장인지참치_839200104(2골), ZD장인지참치_840191208(1골), ZD장인지참치_840256630(1골)</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>2026-09-23 12:05:58</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>경남FC가즈아</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>콩콩콩룔</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>2_1</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>승</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>경남FC가즈아_225238224(2골), 콩콩콩룔_867223848(1골)</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>2026-09-23 11:53:57</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>아들러</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>경남FC가즈아</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>2_0</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>승</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>아들러_866251377(1골), 아들러_855232639(1골)</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>2026-09-23 11:42:25</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>아들러</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>경남FC가즈아</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>5_0</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>승</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>아들러_866251377(1골), 아들러_840191208(3골), 아들러_861000570(1골)</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>2026-09-23 11:29:03</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>앙쿠</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>아들러</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>1_3</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>패</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>앙쿠_851194765(1골), 아들러_840191208(2골), 아들러_852232730(1골)</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>2026-09-23 10:27:43</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>아들러</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>콩콩콩룔</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>2_4</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>패</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>아들러_840191208(2골), 콩콩콩룔_867223848(2골), 콩콩콩룔_866223710(2골)</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>2026-09-23 10:15:56</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>아들러</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>콩콩콩룔</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>2_2</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>무</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>아들러_840191208(2골), 콩콩콩룔_866223710(1골), 콩콩콩룔_851236496(1골)</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>2026-09-23 08:46:09</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>오스트리아</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>겐지간지</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>2_1</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>승</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>오스트리아_291223790(2골), 겐지간지_845158023(1골)</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>2026-09-23 08:35:42</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>오스트리아</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>겐지간지</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>3_1</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>승</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>오스트리아_851221671(1골), 오스트리아_864199266(2골), 겐지간지_856237679(1골)</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
           <t>2026-09-22 14:15:38</t>
         </is>
       </c>
-      <c r="B36" t="inlineStr">
+      <c r="B46" t="inlineStr">
         <is>
           <t>UNIT</t>
         </is>
       </c>
-      <c r="C36" t="inlineStr">
+      <c r="C46" t="inlineStr">
         <is>
           <t>셀래스틴</t>
         </is>
       </c>
-      <c r="D36" t="inlineStr">
+      <c r="D46" t="inlineStr">
         <is>
           <t>1_2</t>
         </is>
       </c>
-      <c r="E36" t="inlineStr">
+      <c r="E46" t="inlineStr">
         <is>
           <t>패</t>
         </is>
       </c>
-      <c r="F36" t="inlineStr">
+      <c r="F46" t="inlineStr">
         <is>
           <t>UNIT_848180930(1골), 셀래스틴_856277179(1골), 셀래스틴_836158023(1골)</t>
         </is>
@@ -1576,7 +1896,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F36"/>
+  <dimension ref="A1:F46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1614,22 +1934,22 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-09-24 16:30:57</t>
+          <t>2026-09-26 12:19:23</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>앙쿠</t>
+          <t>ZD장인지참치</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>UNIT</t>
+          <t>셀래스틴</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>3_2</t>
+          <t>6_4</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -1639,29 +1959,29 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>앙쿠_846193747(1도움), 앙쿠_863246191(1도움), 앙쿠_856247103(1도움), UNIT_840192883(1도움), UNIT_840225782(1도움)</t>
+          <t>ZD장인지참치_840191208(1도움), ZD장인지참치_839200104(2도움), ZD장인지참치_840253149(2도움), 셀래스틴_846001551(1도움), 셀래스틴_852259694(1도움), 셀래스틴_852241461(2도움)</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-09-24 16:14:16</t>
+          <t>2026-09-26 12:08:13</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>앙쿠</t>
+          <t>ZD장인지참치</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>UNIT</t>
+          <t>셀래스틴</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>3_4</t>
+          <t>2_1</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -1671,78 +1991,78 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>앙쿠_851194765(1도움), 앙쿠_863246191(1도움), 앙쿠_856247103(1도움), UNIT_848135455(1도움), UNIT_863250723(1도움), UNIT_840216150(1도움), UNIT_840210736(1도움)</t>
+          <t>ZD장인지참치_839200104(1도움), ZD장인지참치_840256630(1도움)</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-09-24 15:57:54</t>
+          <t>2026-09-26 08:26:23</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>앙쿠</t>
+          <t>오스트리아</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>UNIT</t>
+          <t>Special블루</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>4_1</t>
+          <t>1_3</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>승</t>
+          <t>패</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>앙쿠_851194765(3도움), 앙쿠_848176580(1도움)</t>
+          <t>오스트리아_851216275(1도움), Special블루_861001419(2도움)</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-09-24 13:42:25</t>
+          <t>2026-09-25 15:57:51</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>UNIT</t>
+          <t>셀래스틴</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>셀래스틴</t>
+          <t>Voor</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>4_1</t>
+          <t>0_3</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>승</t>
+          <t>패</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>UNIT_840210736(1도움), UNIT_840228251(1도움), UNIT_867166676(1도움)</t>
+          <t>Voor_835183277(1도움), Voor_852233700(1도움), Voor_856256079(1도움)</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-09-24 13:30:05</t>
+          <t>2026-09-25 09:45:28</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -1752,12 +2072,12 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>셀래스틴</t>
+          <t>방덕</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>1_3</t>
+          <t>3_4</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -1767,29 +2087,29 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>UNIT_840228251(1도움), 셀래스틴_848230938(1도움), 셀래스틴_863277643(1도움), 셀래스틴_861142754(1도움)</t>
+          <t>UNIT_840210736(1도움), UNIT_867166676(1도움), UNIT_840192883(1도움), 방덕_861077787(1도움), 방덕_856233096(1도움)</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-09-24 09:29:12</t>
+          <t>2026-09-25 09:33:41</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>여수가스</t>
+          <t>UNIT</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>ShangHaiPortFC</t>
+          <t>방덕</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>4_2</t>
+          <t>3_2</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -1799,51 +2119,51 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>여수가스_845020289(1도움), 여수가스_828231747(1도움), 여수가스_868135455(1도움), 여수가스_846001551(1도움), ShangHaiPortFC_284190813(1도움), ShangHaiPortFC_861051412(1도움)</t>
+          <t>UNIT_848180930(1도움), UNIT_840192883(1도움), UNIT_867166676(1도움), 방덕_848007512(1도움), 방덕_848231478(1도움)</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-09-24 09:16:26</t>
+          <t>2026-09-25 09:22:20</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>여수가스</t>
+          <t>UNIT</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>ShangHaiPortFC</t>
+          <t>방덕</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>4_3</t>
+          <t>2_3</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>승</t>
+          <t>패</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>여수가스_846001551(1도움), 여수가스_828231747(1도움), 여수가스_852274967(1도움), 여수가스_861162895(1도움), ShangHaiPortFC_845231138(1도움), ShangHaiPortFC_861051412(1도움)</t>
+          <t>UNIT_840192883(1도움), 방덕_848231478(2도움), 방덕_868009676(1도움)</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-09-24 08:18:47</t>
+          <t>2026-09-25 09:10:55</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>은안</t>
+          <t>UNIT</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -1853,29 +2173,29 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>2_7</t>
+          <t>1_1</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>패</t>
+          <t>무</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>은안_856251517(1도움), 방덕_868135455(1도움), 방덕_848231478(1도움), 방덕_848007512(1도움), 방덕_861077787(2도움), 방덕_868009676(1도움), 방덕_856226268(1도움)</t>
+          <t>UNIT_840228251(1도움), 방덕_868135455(1도움)</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-09-24 08:06:58</t>
+          <t>2026-09-25 08:53:47</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>은안</t>
+          <t>UNIT</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -1885,103 +2205,103 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>2_3</t>
+          <t>2_2</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>패</t>
+          <t>무</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>은안_856246420(1도움), 은안_848231866(1도움), 방덕_861077787(1도움), 방덕_848007512(1도움)</t>
+          <t>UNIT_867166676(2도움), 방덕_861077787(1도움), 방덕_868135455(1도움)</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-09-24 04:51:33</t>
+          <t>2026-09-25 08:42:15</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>ZD장인지참치</t>
+          <t>UNIT</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>용신</t>
+          <t>방덕</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>3_1</t>
+          <t>2_3</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>승</t>
+          <t>패</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>ZD장인지참치_848210035(1도움), ZD장인지참치_848199503(1도움), ZD장인지참치_839200104(1도움), 용신_866200104(1도움)</t>
+          <t>UNIT_840192883(1도움), UNIT_829274967(1도움), 방덕_848007512(1도움), 방덕_867001040(1도움), 방덕_101001419(1도움)</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-09-24 04:40:44</t>
+          <t>2026-09-24 16:30:57</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>ZD장인지참치</t>
+          <t>앙쿠</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>용신</t>
+          <t>UNIT</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>4_5</t>
+          <t>3_2</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>패</t>
+          <t>승</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>ZD장인지참치_840191208(2도움), ZD장인지참치_839200104(1도움), ZD장인지참치_851240740(1도움), 용신_863245367(2도움), 용신_273227535(1도움), 용신_848216267(1도움)</t>
+          <t>앙쿠_846193747(1도움), 앙쿠_863246191(1도움), 앙쿠_856247103(1도움), UNIT_840192883(1도움), UNIT_840225782(1도움)</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-09-24 04:19:09</t>
+          <t>2026-09-24 16:14:16</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>ZD장인지참치</t>
+          <t>앙쿠</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>비주류중독</t>
+          <t>UNIT</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>4_4</t>
+          <t>3_4</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -1991,42 +2311,46 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>ZD장인지참치_861182521(2도움), ZD장인지참치_840256630(1도움), ZD장인지참치_851240740(1도움), 비주류중독_848006975(1도움), 비주류중독_839247699(1도움), 비주류중독_852253149(1도움)</t>
+          <t>앙쿠_851194765(1도움), 앙쿠_863246191(1도움), 앙쿠_856247103(1도움), UNIT_848135455(1도움), UNIT_863250723(1도움), UNIT_840216150(1도움), UNIT_840210736(1도움)</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-09-24 04:02:44</t>
+          <t>2026-09-24 15:57:54</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>ZD장인지참치</t>
+          <t>앙쿠</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>비주류중독</t>
+          <t>UNIT</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>0_0</t>
+          <t>4_1</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>패</t>
-        </is>
-      </c>
-      <c r="F14" t="inlineStr"/>
+          <t>승</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>앙쿠_851194765(3도움), 앙쿠_848176580(1도움)</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-09-24 03:45:56</t>
+          <t>2026-09-24 13:42:25</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -2036,12 +2360,12 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>ZD장인지참치</t>
+          <t>셀래스틴</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>5_3</t>
+          <t>4_1</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -2051,29 +2375,29 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>UNIT_840228251(1도움), UNIT_840225782(1도움), UNIT_848135455(1도움), UNIT_848180930(1도움), UNIT_840192883(1도움), ZD장인지참치_848210035(1도움), ZD장인지참치_839200104(2도움)</t>
+          <t>UNIT_840210736(1도움), UNIT_840228251(1도움), UNIT_867166676(1도움)</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-09-24 02:48:31</t>
+          <t>2026-09-24 13:30:05</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>여수가스</t>
+          <t>UNIT</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>방덕</t>
+          <t>셀래스틴</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>3_5</t>
+          <t>1_3</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -2083,56 +2407,56 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>여수가스_861162895(1도움), 여수가스_868135455(1도움), 방덕_868009676(1도움), 방덕_101001419(1도움), 방덕_863184200(1도움), 방덕_867001040(1도움)</t>
+          <t>UNIT_840228251(1도움), 셀래스틴_848230938(1도움), 셀래스틴_863277643(1도움), 셀래스틴_861142754(1도움)</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-09-23 17:59:32</t>
+          <t>2026-09-24 09:29:12</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>0708ManUtd</t>
+          <t>여수가스</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>여수가스</t>
+          <t>ShangHaiPortFC</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>2_3</t>
+          <t>4_2</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>패</t>
+          <t>승</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>0708ManUtd_834239053(1도움), 0708ManUtd_868001397(1도움), 여수가스_868135455(1도움), 여수가스_828231747(1도움), 여수가스_845020289(1도움)</t>
+          <t>여수가스_845020289(1도움), 여수가스_828231747(1도움), 여수가스_868135455(1도움), 여수가스_846001551(1도움), ShangHaiPortFC_284190813(1도움), ShangHaiPortFC_861051412(1도움)</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-09-23 17:47:25</t>
+          <t>2026-09-24 09:16:26</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>0708ManUtd</t>
+          <t>여수가스</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>여수가스</t>
+          <t>ShangHaiPortFC</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -2147,93 +2471,93 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>0708ManUtd_834239053(1도움), 0708ManUtd_868001397(1도움), 0708ManUtd_851226161(1도움), 0708ManUtd_848238794(1도움), 여수가스_861162895(1도움), 여수가스_828231747(1도움)</t>
+          <t>여수가스_846001551(1도움), 여수가스_828231747(1도움), 여수가스_852274967(1도움), 여수가스_861162895(1도움), ShangHaiPortFC_845231138(1도움), ShangHaiPortFC_861051412(1도움)</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-09-23 13:33:47</t>
+          <t>2026-09-24 08:18:47</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>앙쿠</t>
+          <t>은안</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>셀래스틴</t>
+          <t>방덕</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>2_2</t>
+          <t>2_7</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>무</t>
+          <t>패</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>앙쿠_856247103(1도움), 앙쿠_814226161(1도움), 셀래스틴_863251854(1도움), 셀래스틴_852241461(1도움)</t>
+          <t>은안_856251517(1도움), 방덕_868135455(1도움), 방덕_848231478(1도움), 방덕_848007512(1도움), 방덕_861077787(2도움), 방덕_868009676(1도움), 방덕_856226268(1도움)</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-09-23 13:23:09</t>
+          <t>2026-09-24 08:06:58</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>앙쿠</t>
+          <t>은안</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>셀래스틴</t>
+          <t>방덕</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>1_0</t>
+          <t>2_3</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>승</t>
+          <t>패</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>앙쿠_856247103(1도움)</t>
+          <t>은안_856246420(1도움), 은안_848231866(1도움), 방덕_861077787(1도움), 방덕_848007512(1도움)</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-09-23 13:08:58</t>
+          <t>2026-09-24 04:51:33</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>앙쿠</t>
+          <t>ZD장인지참치</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>ZD장인지참치</t>
+          <t>용신</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>3_2</t>
+          <t>3_1</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -2243,61 +2567,61 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>앙쿠_851194765(3도움), ZD장인지참치_839200104(1도움), ZD장인지참치_840256630(1도움)</t>
+          <t>ZD장인지참치_848210035(1도움), ZD장인지참치_848199503(1도움), ZD장인지참치_839200104(1도움), 용신_866200104(1도움)</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2026-09-23 12:58:26</t>
+          <t>2026-09-24 04:40:44</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>앙쿠</t>
+          <t>ZD장인지참치</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>ZD장인지참치</t>
+          <t>용신</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>2_2</t>
+          <t>4_5</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>무</t>
+          <t>패</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>앙쿠_856247103(1도움), 앙쿠_814226161(1도움), ZD장인지참치_861182521(1도움), ZD장인지참치_839200104(1도움)</t>
+          <t>ZD장인지참치_840191208(2도움), ZD장인지참치_839200104(1도움), ZD장인지참치_851240740(1도움), 용신_863245367(2도움), 용신_273227535(1도움), 용신_848216267(1도움)</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-09-23 12:28:11</t>
+          <t>2026-09-24 04:19:09</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>0708ManUtd</t>
+          <t>ZD장인지참치</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>겐지간지</t>
+          <t>비주류중독</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>6_2</t>
+          <t>4_4</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -2307,29 +2631,29 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>0708ManUtd_851226161(2도움), 0708ManUtd_848238794(2도움), 0708ManUtd_868001397(1도움), 겐지간지_856237679(1도움)</t>
+          <t>ZD장인지참치_861182521(2도움), ZD장인지참치_840256630(1도움), ZD장인지참치_851240740(1도움), 비주류중독_848006975(1도움), 비주류중독_839247699(1도움), 비주류중독_852253149(1도움)</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>2026-09-23 12:19:39</t>
+          <t>2026-09-24 04:02:44</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>아들러</t>
+          <t>ZD장인지참치</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>ZD장인지참치</t>
+          <t>비주류중독</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>1_5</t>
+          <t>0_0</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -2337,127 +2661,123 @@
           <t>패</t>
         </is>
       </c>
-      <c r="F24" t="inlineStr">
-        <is>
-          <t>아들러_814192318(1도움), ZD장인지참치_861182521(1도움), ZD장인지참치_848210035(1도움), ZD장인지참치_840191208(1도움), ZD장인지참치_840256630(1도움), ZD장인지참치_848199503(1도움)</t>
-        </is>
-      </c>
+      <c r="F24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-09-23 12:19:35</t>
+          <t>2026-09-24 03:45:56</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>경남FC가즈아</t>
+          <t>UNIT</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>콩콩콩룔</t>
+          <t>ZD장인지참치</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>2_4</t>
+          <t>5_3</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>패</t>
+          <t>승</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>경남FC가즈아_853221467(2도움), 콩콩콩룔_867223848(2도움)</t>
+          <t>UNIT_840228251(1도움), UNIT_840225782(1도움), UNIT_848135455(1도움), UNIT_848180930(1도움), UNIT_840192883(1도움), ZD장인지참치_848210035(1도움), ZD장인지참치_839200104(2도움)</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>2026-09-23 12:15:41</t>
+          <t>2026-09-24 02:48:31</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>0708ManUtd</t>
+          <t>여수가스</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>겐지간지</t>
+          <t>방덕</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>4_3</t>
+          <t>3_5</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>승</t>
+          <t>패</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>0708ManUtd_868001397(2도움), 0708ManUtd_848037576(1도움), 0708ManUtd_851226161(1도움), 겐지간지_861001668(1도움), 겐지간지_826247635(1도움), 겐지간지_852231443(1도움)</t>
+          <t>여수가스_861162895(1도움), 여수가스_868135455(1도움), 방덕_868009676(1도움), 방덕_101001419(1도움), 방덕_863184200(1도움), 방덕_867001040(1도움)</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-09-23 12:07:26</t>
+          <t>2026-09-23 17:59:32</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>아들러</t>
+          <t>0708ManUtd</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>ZD장인지참치</t>
+          <t>여수가스</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>5_4</t>
+          <t>2_3</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>승</t>
+          <t>패</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>아들러_855232639(2도움), 아들러_861000570(1도움), 아들러_840191208(1도움), ZD장인지참치_839200104(1도움), ZD장인지참치_848199503(1도움), ZD장인지참치_861182521(2도움)</t>
+          <t>0708ManUtd_834239053(1도움), 0708ManUtd_868001397(1도움), 여수가스_868135455(1도움), 여수가스_828231747(1도움), 여수가스_845020289(1도움)</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>2026-09-23 12:05:58</t>
+          <t>2026-09-23 17:47:25</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>경남FC가즈아</t>
+          <t>0708ManUtd</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>콩콩콩룔</t>
+          <t>여수가스</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>2_1</t>
+          <t>4_3</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
@@ -2467,61 +2787,61 @@
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>경남FC가즈아_277205156(1도움), 경남FC가즈아_518251161(1도움), 콩콩콩룔_851236496(1도움)</t>
+          <t>0708ManUtd_834239053(1도움), 0708ManUtd_868001397(1도움), 0708ManUtd_851226161(1도움), 0708ManUtd_848238794(1도움), 여수가스_861162895(1도움), 여수가스_828231747(1도움)</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-09-23 11:53:57</t>
+          <t>2026-09-23 13:33:47</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>아들러</t>
+          <t>앙쿠</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>경남FC가즈아</t>
+          <t>셀래스틴</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>2_0</t>
+          <t>2_2</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>승</t>
+          <t>무</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>아들러_861000570(2도움)</t>
+          <t>앙쿠_856247103(1도움), 앙쿠_814226161(1도움), 셀래스틴_863251854(1도움), 셀래스틴_852241461(1도움)</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>2026-09-23 11:42:25</t>
+          <t>2026-09-23 13:23:09</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>아들러</t>
+          <t>앙쿠</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>경남FC가즈아</t>
+          <t>셀래스틴</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>5_0</t>
+          <t>1_0</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
@@ -2531,14 +2851,14 @@
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>아들러_866251377(1도움), 아들러_855232639(1도움), 아들러_840191208(1도움), 아들러_840208574(1도움)</t>
+          <t>앙쿠_856247103(1도움)</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-09-23 11:29:03</t>
+          <t>2026-09-23 13:08:58</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -2548,180 +2868,500 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>아들러</t>
+          <t>ZD장인지참치</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>1_3</t>
+          <t>3_2</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>패</t>
+          <t>승</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>앙쿠_863246191(1도움), 아들러_840191208(1도움), 아들러_852232730(1도움)</t>
+          <t>앙쿠_851194765(3도움), ZD장인지참치_839200104(1도움), ZD장인지참치_840256630(1도움)</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>2026-09-23 10:27:43</t>
+          <t>2026-09-23 12:58:26</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>아들러</t>
+          <t>앙쿠</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>콩콩콩룔</t>
+          <t>ZD장인지참치</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>2_4</t>
+          <t>2_2</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>패</t>
+          <t>무</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>아들러_866251377(1도움), 아들러_852232730(1도움), 콩콩콩룔_867220502(1도움), 콩콩콩룔_867223848(1도움), 콩콩콩룔_866223710(1도움), 콩콩콩룔_861006235(1도움)</t>
+          <t>앙쿠_856247103(1도움), 앙쿠_814226161(1도움), ZD장인지참치_861182521(1도움), ZD장인지참치_839200104(1도움)</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-09-23 10:15:56</t>
+          <t>2026-09-23 12:28:11</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>아들러</t>
+          <t>0708ManUtd</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>콩콩콩룔</t>
+          <t>겐지간지</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>2_2</t>
+          <t>6_2</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>무</t>
+          <t>승</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>아들러_291225126(2도움), 콩콩콩룔_867220502(1도움)</t>
+          <t>0708ManUtd_851226161(2도움), 0708ManUtd_848238794(2도움), 0708ManUtd_868001397(1도움), 겐지간지_856237679(1도움)</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>2026-09-23 08:46:09</t>
+          <t>2026-09-23 12:19:39</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>오스트리아</t>
+          <t>아들러</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>겐지간지</t>
+          <t>ZD장인지참치</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>2_1</t>
+          <t>1_5</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>승</t>
+          <t>패</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>오스트리아_864182152(1도움), 겐지간지_826247635(1도움)</t>
+          <t>아들러_814192318(1도움), ZD장인지참치_861182521(1도움), ZD장인지참치_848210035(1도움), ZD장인지참치_840191208(1도움), ZD장인지참치_840256630(1도움), ZD장인지참치_848199503(1도움)</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-09-23 08:35:42</t>
+          <t>2026-09-23 12:19:35</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>오스트리아</t>
+          <t>경남FC가즈아</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>겐지간지</t>
+          <t>콩콩콩룔</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>3_1</t>
+          <t>2_4</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>승</t>
+          <t>패</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>오스트리아_864140057(2도움), 겐지간지_814231747(1도움)</t>
+          <t>경남FC가즈아_853221467(2도움), 콩콩콩룔_867223848(2도움)</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
+          <t>2026-09-23 12:15:41</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>0708ManUtd</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>겐지간지</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>4_3</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>승</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>0708ManUtd_868001397(2도움), 0708ManUtd_848037576(1도움), 0708ManUtd_851226161(1도움), 겐지간지_861001668(1도움), 겐지간지_826247635(1도움), 겐지간지_852231443(1도움)</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>2026-09-23 12:07:26</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>아들러</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>ZD장인지참치</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>5_4</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>승</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>아들러_855232639(2도움), 아들러_861000570(1도움), 아들러_840191208(1도움), ZD장인지참치_839200104(1도움), ZD장인지참치_848199503(1도움), ZD장인지참치_861182521(2도움)</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>2026-09-23 12:05:58</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>경남FC가즈아</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>콩콩콩룔</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>2_1</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>승</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>경남FC가즈아_277205156(1도움), 경남FC가즈아_518251161(1도움), 콩콩콩룔_851236496(1도움)</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>2026-09-23 11:53:57</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>아들러</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>경남FC가즈아</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>2_0</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>승</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>아들러_861000570(2도움)</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>2026-09-23 11:42:25</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>아들러</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>경남FC가즈아</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>5_0</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>승</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>아들러_866251377(1도움), 아들러_855232639(1도움), 아들러_840191208(1도움), 아들러_840208574(1도움)</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>2026-09-23 11:29:03</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>앙쿠</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>아들러</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>1_3</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>패</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>앙쿠_863246191(1도움), 아들러_840191208(1도움), 아들러_852232730(1도움)</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>2026-09-23 10:27:43</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>아들러</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>콩콩콩룔</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>2_4</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>패</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>아들러_866251377(1도움), 아들러_852232730(1도움), 콩콩콩룔_867220502(1도움), 콩콩콩룔_867223848(1도움), 콩콩콩룔_866223710(1도움), 콩콩콩룔_861006235(1도움)</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>2026-09-23 10:15:56</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>아들러</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>콩콩콩룔</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>2_2</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>무</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>아들러_291225126(2도움), 콩콩콩룔_867220502(1도움)</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>2026-09-23 08:46:09</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>오스트리아</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>겐지간지</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>2_1</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>승</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>오스트리아_864182152(1도움), 겐지간지_826247635(1도움)</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>2026-09-23 08:35:42</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>오스트리아</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>겐지간지</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>3_1</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>승</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>오스트리아_864140057(2도움), 겐지간지_814231747(1도움)</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
           <t>2026-09-22 14:15:38</t>
         </is>
       </c>
-      <c r="B36" t="inlineStr">
+      <c r="B46" t="inlineStr">
         <is>
           <t>UNIT</t>
         </is>
       </c>
-      <c r="C36" t="inlineStr">
+      <c r="C46" t="inlineStr">
         <is>
           <t>셀래스틴</t>
         </is>
       </c>
-      <c r="D36" t="inlineStr">
+      <c r="D46" t="inlineStr">
         <is>
           <t>1_2</t>
         </is>
       </c>
-      <c r="E36" t="inlineStr">
+      <c r="E46" t="inlineStr">
         <is>
           <t>패</t>
         </is>
       </c>
-      <c r="F36" t="inlineStr">
+      <c r="F46" t="inlineStr">
         <is>
           <t>UNIT_840192883(1도움), 셀래스틴_852277643(1도움), 셀래스틴_852241461(1도움)</t>
         </is>

</xml_diff>

<commit_message>
Update: Dashboard HTML (20:38:32)
</commit_message>
<xml_diff>
--- a/API데이터_경기_득점_및_도움_기록.xlsx
+++ b/API데이터_경기_득점_및_도움_기록.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F15"/>
+  <dimension ref="A1:F41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -452,22 +452,22 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-09-29 14:16:03</t>
+          <t>2026-10-01 07:54:09</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>개포동덕배</t>
+          <t>호야국2인</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Gucci차붐</t>
+          <t>아들러</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>7_2</t>
+          <t>3_2</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -477,29 +477,29 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>개포동덕배_848206113(1골), 개포동덕배_845208722(1골), 개포동덕배_856202126(1골), 개포동덕배_845190048(4골), Gucci차붐_864247686(1골), Gucci차붐_864176403(1골)</t>
+          <t>호야국2인_851261865(1골), 호야국2인_846192505(1골), 호야국2인_848232293(1골), 아들러_861000570(1골), 아들러_840191208(1골)</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-09-29 14:04:54</t>
+          <t>2026-10-01 07:42:04</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>개포동덕배</t>
+          <t>호야국2인</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Gucci차붐</t>
+          <t>아들러</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>4_2</t>
+          <t>5_2</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -509,61 +509,61 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>개포동덕배_845190048(3골), 개포동덕배_848206113(1골), Gucci차붐_853272733(1골), Gucci차붐_853242004(1골)</t>
+          <t>호야국2인_848227236(2골), 호야국2인_848232293(1골), 호야국2인_848216435(1골), 호야국2인_851216409(1골), 아들러_291225126(1골), 아들러_866251377(1골)</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-09-29 11:20:02</t>
+          <t>2026-10-01 06:47:50</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>UNIT</t>
+          <t>호야국2인</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>콩콩콩룔</t>
+          <t>suma수마</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>1_3</t>
+          <t>4_2</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>패</t>
+          <t>승</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>UNIT_848180930(1골), 콩콩콩룔_867223848(1골), 콩콩콩룔_866223710(2골)</t>
+          <t>호야국2인_845198219(1골), 호야국2인_848232293(2골), 호야국2인_848216435(1골), suma수마_861190046(1골), suma수마_861221162(1골)</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-09-29 11:08:25</t>
+          <t>2026-10-01 06:36:26</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>UNIT</t>
+          <t>호야국2인</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>콩콩콩룔</t>
+          <t>suma수마</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>3_2</t>
+          <t>5_2</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -573,46 +573,46 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>UNIT_848180930(1골), UNIT_848135455(1골), UNIT_867166676(1골), 콩콩콩룔_866223710(1골), 콩콩콩룔_867223848(1골)</t>
+          <t>호야국2인_851216409(1골), 호야국2인_845198219(1골), 호야국2인_846192505(1골), 호야국2인_848227236(1골), 호야국2인_848232293(1골), suma수마_861013383(1골), suma수마_861221162(1골)</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-09-29 10:56:21</t>
+          <t>2026-09-30 17:45:59</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>오스트리아</t>
+          <t>UNIT</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>ShangHaiPortFC</t>
+          <t>Voor</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>7_1</t>
+          <t>2_5</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>승</t>
+          <t>패</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>오스트리아_864199266(3골), 오스트리아_851221671(1골), 오스트리아_864182152(1골), 오스트리아_864140057(1골), 오스트리아_851216275(1골), ShangHaiPortFC_864191910(1골)</t>
+          <t>UNIT_867166676(2골), Voor_845009676(1골), Voor_835183277(1골), Voor_852233700(3골)</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-09-29 10:47:10</t>
+          <t>2026-09-30 17:34:22</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -622,44 +622,44 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>셀래스틴</t>
+          <t>Voor</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>3_2</t>
+          <t>3_4</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>승</t>
+          <t>패</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>UNIT_840228251(1골), UNIT_867166676(2골), 셀래스틴_848231866(1골), 셀래스틴_848230938(1골)</t>
+          <t>UNIT_848180930(2골), UNIT_840192883(1골), Voor_845009676(1골), Voor_856256079(1골), Voor_852233700(2골)</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-09-29 10:45:30</t>
+          <t>2026-09-30 17:17:18</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>오스트리아</t>
+          <t>UNIT</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>ShangHaiPortFC</t>
+          <t>Voor</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>5_1</t>
+          <t>3_2</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -669,14 +669,14 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>오스트리아_864140057(2골), 오스트리아_864182152(1골), 오스트리아_864199266(2골), ShangHaiPortFC_861051412(1골)</t>
+          <t>UNIT_867166676(1골), UNIT_848180930(2골), Voor_852233700(2골)</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-09-29 10:35:32</t>
+          <t>2026-09-30 17:03:54</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -686,29 +686,29 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>셀래스틴</t>
+          <t>Voor</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>1_3</t>
+          <t>5_1</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>패</t>
+          <t>승</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>UNIT_848180930(1골), 셀래스틴_846001551(1골), 셀래스틴_852241461(2골)</t>
+          <t>UNIT_867166676(5골), Voor_845009676(1골)</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-09-29 10:18:25</t>
+          <t>2026-09-30 16:46:35</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -718,34 +718,34 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>셀래스틴</t>
+          <t>Voor</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>2_1</t>
+          <t>2_3</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>승</t>
+          <t>패</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>UNIT_867166676(2골), 셀래스틴_848194765(1골)</t>
+          <t>UNIT_848180930(2골), Voor_845009676(1골), Voor_852233700(2골)</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-09-29 09:24:43</t>
+          <t>2026-09-30 14:01:02</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>오스트리아</t>
+          <t>UNIT</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -755,7 +755,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>2_3</t>
+          <t>2_5</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -765,19 +765,19 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>오스트리아_864199266(1골), 오스트리아_851236636(1골), 셀래스틴_846001551(1골), 셀래스틴_861005680(1골), 셀래스틴_848230938(1골)</t>
+          <t>UNIT_861221162(2골), 셀래스틴_861005680(4골), 셀래스틴_848231866(1골)</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-09-29 09:13:08</t>
+          <t>2026-09-30 13:49:10</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>오스트리아</t>
+          <t>UNIT</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -787,29 +787,29 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>1_1</t>
+          <t>5_3</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>무</t>
+          <t>승</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>오스트리아_864199266(1골), 셀래스틴_861005680(1골)</t>
+          <t>UNIT_867166676(3골), UNIT_861221162(2골), 셀래스틴_846001551(1골), 셀래스틴_852241461(1골), 셀래스틴_861005680(1골)</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-09-29 09:02:47</t>
+          <t>2026-09-30 13:33:10</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>오스트리아</t>
+          <t>UNIT</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -819,79 +819,911 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>3_1</t>
+          <t>1_5</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>승</t>
+          <t>패</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>오스트리아_864140057(1골), 오스트리아_864199266(1골), 오스트리아_864182152(1골), 셀래스틴_861005680(1골)</t>
+          <t>UNIT_848180930(1골), 셀래스틴_848194765(1골), 셀래스틴_861005680(3골), 셀래스틴_852241461(1골)</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-09-29 08:51:25</t>
+          <t>2026-09-30 13:24:44</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>오스트리아</t>
+          <t>Gucci와퍼</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>셀래스틴</t>
+          <t>비주류중독</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>0_2</t>
+          <t>4_3</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>패</t>
+          <t>승</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>셀래스틴_846001551(1골), 셀래스틴_861005680(1골)</t>
+          <t>Gucci와퍼_864200104(4골), 비주류중독_840052241(1골), 비주류중독_825000240(1골), 비주류중독_839247699(1골)</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
+          <t>2026-09-30 13:21:00</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>UNIT</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>셀래스틴</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>2_0</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>승</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>UNIT_848180930(1골), UNIT_867166676(1골)</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-09-30 13:12:24</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Gucci와퍼</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>비주류중독</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>2_3</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>패</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>Gucci와퍼_852028765(1골), Gucci와퍼_852168473(1골), 비주류중독_834239977(1골), 비주류중독_840052241(1골), 비주류중독_839247699(1골)</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2026-09-30 13:10:05</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>UNIT</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>셀래스틴</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>4_3</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>승</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>UNIT_867166676(3골), UNIT_840192883(1골), 셀래스틴_848194765(1골), 셀래스틴_861005680(2골)</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>2026-09-30 12:57:48</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>UNIT</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>셀래스틴</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>3_1</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>승</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>UNIT_867166676(2골), UNIT_848180930(1골), 셀래스틴_846001551(1골)</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>2026-09-30 12:35:39</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>셀래스틴</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>비주류중독</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>2_3</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>패</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>셀래스틴_846001551(1골), 셀래스틴_852241461(1골), 비주류중독_848006975(2골), 비주류중독_839247699(1골)</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>2026-09-30 12:24:21</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>셀래스틴</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>비주류중독</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>2_0</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>승</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>셀래스틴_852241461(1골), 셀래스틴_861005680(1골)</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>2026-09-30 12:00:21</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>UNIT</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>셀래스틴</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>2_3</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>패</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>UNIT_848180930(2골), 셀래스틴_861005680(2골), 셀래스틴_852241461(1골)</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>2026-09-30 09:47:20</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>방덕</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Voor</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>3_4</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>패</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>방덕_848007512(1골), 방덕_856228093(1골), 방덕_863184200(1골), Voor_845247090(2골), Voor_852233700(2골)</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>2026-09-30 09:35:39</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>방덕</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Voor</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>1_6</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>패</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>방덕_101001419(1골), Voor_852233700(3골), Voor_845009676(2골), Voor_845247090(1골)</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>2026-09-30 08:27:58</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Legend독수리</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>syma</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>3_2</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>승</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>Legend독수리_825190048(1골), Legend독수리_861081644(1골), Legend독수리_848188350(1골), syma_863228092(1골), syma_856233848(1골)</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>2026-09-30 08:16:55</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Legend독수리</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>syma</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>1_6</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>패</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>Legend독수리_825190048(1골), syma_866231913(1골), syma_863262863(1골), syma_846001845(3골), syma_852274967(1골)</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>2026-09-30 08:04:48</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Legend독수리</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>syma</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>2_2</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>무</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>Legend독수리_861215732(1골), Legend독수리_852209658(1골), syma_866231913(1골), syma_863228092(1골)</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>2026-09-30 07:53:20</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Legend독수리</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>syma</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>1_2</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>패</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>Legend독수리_861215732(1골), syma_863222665(2골)</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>2026-09-29 14:16:03</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>개포동덕배</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Gucci차붐</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>7_2</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>승</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>개포동덕배_848206113(1골), 개포동덕배_845208722(1골), 개포동덕배_856202126(1골), 개포동덕배_845190048(4골), Gucci차붐_864247686(1골), Gucci차붐_864176403(1골)</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>2026-09-29 14:04:54</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>개포동덕배</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Gucci차붐</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>4_2</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>승</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>개포동덕배_845190048(3골), 개포동덕배_848206113(1골), Gucci차붐_853272733(1골), Gucci차붐_853242004(1골)</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>2026-09-29 11:20:02</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>UNIT</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>콩콩콩룔</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>1_3</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>패</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>UNIT_848180930(1골), 콩콩콩룔_867223848(1골), 콩콩콩룔_866223710(2골)</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>2026-09-29 11:08:25</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>UNIT</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>콩콩콩룔</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>3_2</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>승</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>UNIT_848180930(1골), UNIT_848135455(1골), UNIT_867166676(1골), 콩콩콩룔_866223710(1골), 콩콩콩룔_867223848(1골)</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>2026-09-29 10:56:21</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>오스트리아</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>ShangHaiPortFC</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>7_1</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>승</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>오스트리아_864199266(3골), 오스트리아_851221671(1골), 오스트리아_864182152(1골), 오스트리아_864140057(1골), 오스트리아_851216275(1골), ShangHaiPortFC_864191910(1골)</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>2026-09-29 10:47:10</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>UNIT</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>셀래스틴</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>3_2</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>승</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>UNIT_840228251(1골), UNIT_867166676(2골), 셀래스틴_848231866(1골), 셀래스틴_848230938(1골)</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>2026-09-29 10:45:30</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>오스트리아</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>ShangHaiPortFC</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>5_1</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>승</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>오스트리아_864140057(2골), 오스트리아_864182152(1골), 오스트리아_864199266(2골), ShangHaiPortFC_861051412(1골)</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>2026-09-29 10:35:32</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>UNIT</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>셀래스틴</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>1_3</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>패</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>UNIT_848180930(1골), 셀래스틴_846001551(1골), 셀래스틴_852241461(2골)</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>2026-09-29 10:18:25</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>UNIT</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>셀래스틴</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>2_1</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>승</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>UNIT_867166676(2골), 셀래스틴_848194765(1골)</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>2026-09-29 09:24:43</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>오스트리아</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>셀래스틴</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>2_3</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>패</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>오스트리아_864199266(1골), 오스트리아_851236636(1골), 셀래스틴_846001551(1골), 셀래스틴_861005680(1골), 셀래스틴_848230938(1골)</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>2026-09-29 09:13:08</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>오스트리아</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>셀래스틴</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>1_1</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>무</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>오스트리아_864199266(1골), 셀래스틴_861005680(1골)</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>2026-09-29 09:02:47</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>오스트리아</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>셀래스틴</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>3_1</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>승</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>오스트리아_864140057(1골), 오스트리아_864199266(1골), 오스트리아_864182152(1골), 셀래스틴_861005680(1골)</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>2026-09-29 08:51:25</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>오스트리아</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>셀래스틴</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>0_2</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>패</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>셀래스틴_846001551(1골), 셀래스틴_861005680(1골)</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
           <t>2026-09-29 04:33:11</t>
         </is>
       </c>
-      <c r="B15" t="inlineStr">
+      <c r="B41" t="inlineStr">
         <is>
           <t>여수가스</t>
         </is>
       </c>
-      <c r="C15" t="inlineStr">
+      <c r="C41" t="inlineStr">
         <is>
           <t>오스트리아</t>
         </is>
       </c>
-      <c r="D15" t="inlineStr">
+      <c r="D41" t="inlineStr">
         <is>
           <t>2_3</t>
         </is>
       </c>
-      <c r="E15" t="inlineStr">
-        <is>
-          <t>패</t>
-        </is>
-      </c>
-      <c r="F15" t="inlineStr">
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>패</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
         <is>
           <t>여수가스_828231747(1골), 여수가스_852274967(1골), 오스트리아_864191566(1골), 오스트리아_864199266(2골)</t>
         </is>
@@ -908,7 +1740,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F15"/>
+  <dimension ref="A1:F41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -946,22 +1778,22 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-09-29 14:16:03</t>
+          <t>2026-10-01 07:54:09</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>개포동덕배</t>
+          <t>호야국2인</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Gucci차붐</t>
+          <t>아들러</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>7_2</t>
+          <t>3_2</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -971,29 +1803,29 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>개포동덕배_848206113(1도움), 개포동덕배_845208722(3도움), 개포동덕배_856202126(1도움), 개포동덕배_863212622(2도움), Gucci차붐_853272733(1도움), Gucci차붐_864176403(1도움)</t>
+          <t>호야국2인_848227236(2도움), 호야국2인_848232293(1도움), 아들러_866251377(1도움), 아들러_855232639(1도움)</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-09-29 14:04:54</t>
+          <t>2026-10-01 07:42:04</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>개포동덕배</t>
+          <t>호야국2인</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Gucci차붐</t>
+          <t>아들러</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>4_2</t>
+          <t>5_2</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -1003,61 +1835,61 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>개포동덕배_856202126(1도움), 개포동덕배_863234396(1도움), 개포동덕배_856275298(1도움), 개포동덕배_848206113(1도움), Gucci차붐_864084333(1도움), Gucci차붐_864247686(1도움)</t>
+          <t>호야국2인_848232293(2도움), 호야국2인_848217870(1도움), 호야국2인_851216409(1도움), 아들러_840191208(1도움)</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-09-29 11:20:02</t>
+          <t>2026-10-01 06:47:50</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>UNIT</t>
+          <t>호야국2인</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>콩콩콩룔</t>
+          <t>suma수마</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>1_3</t>
+          <t>4_2</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>패</t>
+          <t>승</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>UNIT_867166676(1도움), 콩콩콩룔_867220502(1도움), 콩콩콩룔_848189505(2도움)</t>
+          <t>호야국2인_848217870(1도움), 호야국2인_848232293(1도움), 호야국2인_852001183(1도움), suma수마_861190046(1도움), suma수마_848225439(1도움)</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-09-29 11:08:25</t>
+          <t>2026-10-01 06:36:26</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>UNIT</t>
+          <t>호야국2인</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>콩콩콩룔</t>
+          <t>suma수마</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>3_2</t>
+          <t>5_2</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -1067,46 +1899,46 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>UNIT_840192883(2도움), UNIT_848265695(1도움), 콩콩콩룔_851236496(1도움)</t>
+          <t>호야국2인_851216409(1도움), 호야국2인_845198219(1도움), 호야국2인_846192505(1도움), 호야국2인_848216435(1도움), suma수마_826223697(1도움)</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-09-29 10:56:21</t>
+          <t>2026-09-30 17:45:59</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>오스트리아</t>
+          <t>UNIT</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>ShangHaiPortFC</t>
+          <t>Voor</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>7_1</t>
+          <t>2_5</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>승</t>
+          <t>패</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>오스트리아_864182152(2도움), 오스트리아_864140057(1도움), 오스트리아_851236636(4도움), ShangHaiPortFC_848031432(1도움)</t>
+          <t>UNIT_840192883(1도움), Voor_856256079(1도움), Voor_861000027(4도움)</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-09-29 10:47:10</t>
+          <t>2026-09-30 17:34:22</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -1116,44 +1948,44 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>셀래스틴</t>
+          <t>Voor</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>3_2</t>
+          <t>3_4</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>승</t>
+          <t>패</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>UNIT_848180930(1도움), UNIT_863250723(1도움), UNIT_840192883(1도움), 셀래스틴_846001551(1도움)</t>
+          <t>UNIT_861221162(1도움), UNIT_866247257(1도움), UNIT_840228251(1도움), Voor_845009676(1도움), Voor_858025420(1도움), Voor_835183277(1도움)</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-09-29 10:45:30</t>
+          <t>2026-09-30 17:17:18</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>오스트리아</t>
+          <t>UNIT</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>ShangHaiPortFC</t>
+          <t>Voor</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>5_1</t>
+          <t>3_2</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -1163,14 +1995,14 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>오스트리아_851221671(1도움), 오스트리아_863223671(1도움), 오스트리아_863240709(1도움), 오스트리아_864140057(1도움), 오스트리아_851216275(1도움), ShangHaiPortFC_827143001(1도움)</t>
+          <t>UNIT_840228251(1도움), UNIT_840192883(1도움), UNIT_848135455(1도움), Voor_845239231(1도움), Voor_845009676(1도움)</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-09-29 10:35:32</t>
+          <t>2026-09-30 17:03:54</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -1180,29 +2012,29 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>셀래스틴</t>
+          <t>Voor</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>1_3</t>
+          <t>5_1</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>패</t>
+          <t>승</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>UNIT_867166676(1도움), 셀래스틴_848231866(2도움), 셀래스틴_852241461(1도움)</t>
+          <t>UNIT_848180930(1도움), UNIT_840192883(1도움), UNIT_848265695(3도움), Voor_852233700(1도움)</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-09-29 10:18:25</t>
+          <t>2026-09-30 16:46:35</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -1212,34 +2044,34 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>셀래스틴</t>
+          <t>Voor</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>2_1</t>
+          <t>2_3</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>승</t>
+          <t>패</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>UNIT_839013383(1도움), UNIT_840192883(1도움), 셀래스틴_846001551(1도움)</t>
+          <t>UNIT_840228251(1도움), UNIT_840192883(1도움), Voor_845009676(1도움), Voor_846184943(1도움), Voor_852233700(1도움)</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-09-29 09:24:43</t>
+          <t>2026-09-30 14:01:02</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>오스트리아</t>
+          <t>UNIT</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -1249,7 +2081,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>2_3</t>
+          <t>2_5</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -1259,19 +2091,19 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>오스트리아_864199266(1도움), 오스트리아_863240709(1도움), 셀래스틴_846001551(1도움), 셀래스틴_848194765(2도움)</t>
+          <t>UNIT_867166676(2도움), 셀래스틴_848194765(1도움), 셀래스틴_848231866(1도움), 셀래스틴_852241461(1도움)</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-09-29 09:13:08</t>
+          <t>2026-09-30 13:49:10</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>오스트리아</t>
+          <t>UNIT</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -1281,29 +2113,29 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>1_1</t>
+          <t>5_3</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>무</t>
+          <t>승</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>오스트리아_851221671(1도움), 셀래스틴_848231866(1도움)</t>
+          <t>UNIT_840210736(2도움), UNIT_867166676(1도움), UNIT_848135455(1도움), UNIT_840192883(1도움), 셀래스틴_863200458(1도움), 셀래스틴_852241461(2도움)</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-09-29 09:02:47</t>
+          <t>2026-09-30 13:33:10</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>오스트리아</t>
+          <t>UNIT</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -1313,79 +2145,911 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>3_1</t>
+          <t>1_5</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>승</t>
+          <t>패</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>오스트리아_864140057(1도움), 오스트리아_864182152(1도움), 오스트리아_851236636(1도움), 셀래스틴_846001551(1도움)</t>
+          <t>UNIT_840192883(1도움), 셀래스틴_863200458(1도움), 셀래스틴_852259694(1도움), 셀래스틴_861005680(1도움)</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-09-29 08:51:25</t>
+          <t>2026-09-30 13:24:44</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>오스트리아</t>
+          <t>Gucci와퍼</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>셀래스틴</t>
+          <t>비주류중독</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>0_2</t>
+          <t>4_3</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>패</t>
+          <t>승</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>셀래스틴_863200458(1도움), 셀래스틴_852241461(1도움)</t>
+          <t>Gucci와퍼_852168473(3도움), Gucci와퍼_852028765(1도움), 비주류중독_840052241(1도움), 비주류중독_862180283(1도움)</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
+          <t>2026-09-30 13:21:00</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>UNIT</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>셀래스틴</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>2_0</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>승</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>UNIT_840192883(1도움), UNIT_840228251(1도움)</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-09-30 13:12:24</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Gucci와퍼</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>비주류중독</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>2_3</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>패</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>Gucci와퍼_852010264(1도움), 비주류중독_834239977(1도움), 비주류중독_848006975(1도움)</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2026-09-30 13:10:05</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>UNIT</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>셀래스틴</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>4_3</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>승</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>UNIT_867166676(1도움), UNIT_840192883(2도움), UNIT_840225782(1도움), 셀래스틴_848194765(1도움), 셀래스틴_863200458(1도움)</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>2026-09-30 12:57:48</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>UNIT</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>셀래스틴</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>3_1</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>승</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>UNIT_863250723(1도움), UNIT_840228251(2도움), 셀래스틴_852241461(1도움)</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>2026-09-30 12:35:39</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>셀래스틴</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>비주류중독</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>2_3</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>패</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>셀래스틴_848231866(1도움), 셀래스틴_852259694(1도움), 비주류중독_839247699(1도움), 비주류중독_834239977(2도움)</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>2026-09-30 12:24:21</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>셀래스틴</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>비주류중독</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>2_0</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>승</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>셀래스틴_852259694(1도움), 셀래스틴_848194765(1도움)</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>2026-09-30 12:00:21</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>UNIT</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>셀래스틴</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>2_3</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>패</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>UNIT_840225782(1도움), UNIT_867166676(1도움), 셀래스틴_848013038(1도움), 셀래스틴_852241461(2도움)</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>2026-09-30 09:47:20</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>방덕</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Voor</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>3_4</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>패</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>방덕_867001040(1도움), 방덕_848231478(2도움), Voor_845009676(1도움), Voor_845239231(1도움), Voor_835183277(1도움), Voor_848216150(1도움)</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>2026-09-30 09:35:39</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>방덕</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Voor</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>1_6</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>패</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>Voor_852233700(2도움), Voor_856256079(1도움), Voor_845009676(2도움), Voor_835183277(1도움)</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>2026-09-30 08:27:58</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Legend독수리</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>syma</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>3_2</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>승</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>Legend독수리_861215732(1도움), Legend독수리_852209658(1도움), syma_852274967(1도움), syma_863228092(1도움)</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>2026-09-30 08:16:55</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Legend독수리</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>syma</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>1_6</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>패</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>Legend독수리_861215732(1도움), syma_866231913(2도움), syma_863222665(4도움)</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>2026-09-30 08:04:48</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Legend독수리</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>syma</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>2_2</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>무</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>Legend독수리_848224425(1도움), Legend독수리_826236703(1도움), syma_856233848(1도움)</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>2026-09-30 07:53:20</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Legend독수리</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>syma</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>1_2</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>패</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>Legend독수리_861081644(1도움), syma_846001845(2도움)</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>2026-09-29 14:16:03</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>개포동덕배</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Gucci차붐</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>7_2</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>승</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>개포동덕배_848206113(1도움), 개포동덕배_845208722(3도움), 개포동덕배_856202126(1도움), 개포동덕배_863212622(2도움), Gucci차붐_853272733(1도움), Gucci차붐_864176403(1도움)</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>2026-09-29 14:04:54</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>개포동덕배</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Gucci차붐</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>4_2</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>승</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>개포동덕배_856202126(1도움), 개포동덕배_863234396(1도움), 개포동덕배_856275298(1도움), 개포동덕배_848206113(1도움), Gucci차붐_864084333(1도움), Gucci차붐_864247686(1도움)</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>2026-09-29 11:20:02</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>UNIT</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>콩콩콩룔</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>1_3</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>패</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>UNIT_867166676(1도움), 콩콩콩룔_867220502(1도움), 콩콩콩룔_848189505(2도움)</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>2026-09-29 11:08:25</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>UNIT</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>콩콩콩룔</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>3_2</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>승</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>UNIT_840192883(2도움), UNIT_848265695(1도움), 콩콩콩룔_851236496(1도움)</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>2026-09-29 10:56:21</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>오스트리아</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>ShangHaiPortFC</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>7_1</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>승</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>오스트리아_864182152(2도움), 오스트리아_864140057(1도움), 오스트리아_851236636(4도움), ShangHaiPortFC_848031432(1도움)</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>2026-09-29 10:47:10</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>UNIT</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>셀래스틴</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>3_2</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>승</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>UNIT_848180930(1도움), UNIT_863250723(1도움), UNIT_840192883(1도움), 셀래스틴_846001551(1도움)</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>2026-09-29 10:45:30</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>오스트리아</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>ShangHaiPortFC</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>5_1</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>승</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>오스트리아_851221671(1도움), 오스트리아_863223671(1도움), 오스트리아_863240709(1도움), 오스트리아_864140057(1도움), 오스트리아_851216275(1도움), ShangHaiPortFC_827143001(1도움)</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>2026-09-29 10:35:32</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>UNIT</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>셀래스틴</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>1_3</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>패</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>UNIT_867166676(1도움), 셀래스틴_848231866(2도움), 셀래스틴_852241461(1도움)</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>2026-09-29 10:18:25</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>UNIT</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>셀래스틴</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>2_1</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>승</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>UNIT_839013383(1도움), UNIT_840192883(1도움), 셀래스틴_846001551(1도움)</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>2026-09-29 09:24:43</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>오스트리아</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>셀래스틴</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>2_3</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>패</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>오스트리아_864199266(1도움), 오스트리아_863240709(1도움), 셀래스틴_846001551(1도움), 셀래스틴_848194765(2도움)</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>2026-09-29 09:13:08</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>오스트리아</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>셀래스틴</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>1_1</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>무</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>오스트리아_851221671(1도움), 셀래스틴_848231866(1도움)</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>2026-09-29 09:02:47</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>오스트리아</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>셀래스틴</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>3_1</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>승</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>오스트리아_864140057(1도움), 오스트리아_864182152(1도움), 오스트리아_851236636(1도움), 셀래스틴_846001551(1도움)</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>2026-09-29 08:51:25</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>오스트리아</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>셀래스틴</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>0_2</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>패</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>셀래스틴_863200458(1도움), 셀래스틴_852241461(1도움)</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
           <t>2026-09-29 04:33:11</t>
         </is>
       </c>
-      <c r="B15" t="inlineStr">
+      <c r="B41" t="inlineStr">
         <is>
           <t>여수가스</t>
         </is>
       </c>
-      <c r="C15" t="inlineStr">
+      <c r="C41" t="inlineStr">
         <is>
           <t>오스트리아</t>
         </is>
       </c>
-      <c r="D15" t="inlineStr">
+      <c r="D41" t="inlineStr">
         <is>
           <t>2_3</t>
         </is>
       </c>
-      <c r="E15" t="inlineStr">
-        <is>
-          <t>패</t>
-        </is>
-      </c>
-      <c r="F15" t="inlineStr">
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>패</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
         <is>
           <t>여수가스_852216393(1도움), 여수가스_861162895(1도움), 오스트리아_864140057(1도움), 오스트리아_851257075(1도움)</t>
         </is>

</xml_diff>

<commit_message>
Update: Dashboard HTML (08:10:55)
</commit_message>
<xml_diff>
--- a/API데이터_경기_득점_및_도움_기록.xlsx
+++ b/API데이터_경기_득점_및_도움_기록.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F41"/>
+  <dimension ref="A1:F64"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -452,86 +452,86 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-10-01 07:54:09</t>
+          <t>2026-10-01 15:50:18</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>호야국2인</t>
+          <t>suma수마</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>아들러</t>
+          <t>피파왕초보구단주</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>3_2</t>
+          <t>1_3</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>승</t>
+          <t>패</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>호야국2인_851261865(1골), 호야국2인_846192505(1골), 호야국2인_848232293(1골), 아들러_861000570(1골), 아들러_840191208(1골)</t>
+          <t>suma수마_861190046(1골), 피파왕초보구단주_861005661(3골)</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-10-01 07:42:04</t>
+          <t>2026-10-01 15:38:48</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>호야국2인</t>
+          <t>suma수마</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>아들러</t>
+          <t>피파왕초보구단주</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>5_2</t>
+          <t>2_2</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>승</t>
+          <t>무</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>호야국2인_848227236(2골), 호야국2인_848232293(1골), 호야국2인_848216435(1골), 호야국2인_851216409(1골), 아들러_291225126(1골), 아들러_866251377(1골)</t>
+          <t>suma수마_861221162(1골), suma수마_861013383(1골), 피파왕초보구단주_846208722(1골), 피파왕초보구단주_856209331(1골)</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-10-01 06:47:50</t>
+          <t>2026-10-01 15:24:08</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>호야국2인</t>
+          <t>피파왕초보구단주</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>suma수마</t>
+          <t>Gucci와퍼</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>4_2</t>
+          <t>5_1</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -541,61 +541,61 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>호야국2인_845198219(1골), 호야국2인_848232293(2골), 호야국2인_848216435(1골), suma수마_861190046(1골), suma수마_861221162(1골)</t>
+          <t>피파왕초보구단주_846208722(2골), 피파왕초보구단주_867000027(2골), 피파왕초보구단주_861005661(1골), Gucci와퍼_852208128(1골)</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-10-01 06:36:26</t>
+          <t>2026-10-01 15:12:09</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>호야국2인</t>
+          <t>피파왕초보구단주</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>suma수마</t>
+          <t>Gucci와퍼</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>5_2</t>
+          <t>3_3</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>승</t>
+          <t>무</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>호야국2인_851216409(1골), 호야국2인_845198219(1골), 호야국2인_846192505(1골), 호야국2인_848227236(1골), 호야국2인_848232293(1골), suma수마_861013383(1골), suma수마_861221162(1골)</t>
+          <t>피파왕초보구단주_848209499(1골), 피파왕초보구단주_861005661(2골), Gucci와퍼_840208574(1골), Gucci와퍼_864200104(2골)</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-09-30 17:45:59</t>
+          <t>2026-10-01 14:56:12</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>UNIT</t>
+          <t>0708ManUtd</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Voor</t>
+          <t>호야국2인</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>2_5</t>
+          <t>1_2</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -605,29 +605,29 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>UNIT_867166676(2골), Voor_845009676(1골), Voor_835183277(1골), Voor_852233700(3골)</t>
+          <t>0708ManUtd_848238794(1골), 호야국2인_848227236(1골), 호야국2인_848232293(1골)</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-09-30 17:34:22</t>
+          <t>2026-10-01 14:51:31</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>UNIT</t>
+          <t>은안</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Voor</t>
+          <t>Gucci와퍼</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>3_4</t>
+          <t>1_4</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -637,61 +637,61 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>UNIT_848180930(2골), UNIT_840192883(1골), Voor_845009676(1골), Voor_856256079(1골), Voor_852233700(2골)</t>
+          <t>은안_852237692(1골), Gucci와퍼_852028765(1골), Gucci와퍼_852010264(1골), Gucci와퍼_864200104(2골)</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-09-30 17:17:18</t>
+          <t>2026-10-01 14:45:02</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>UNIT</t>
+          <t>0708ManUtd</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Voor</t>
+          <t>호야국2인</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>3_2</t>
+          <t>2_3</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>승</t>
+          <t>패</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>UNIT_867166676(1골), UNIT_848180930(2골), Voor_852233700(2골)</t>
+          <t>0708ManUtd_868037576(1골), 0708ManUtd_834239053(1골), 호야국2인_851216409(1골), 호야국2인_848232293(1골), 호야국2인_846192505(1골)</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-09-30 17:03:54</t>
+          <t>2026-10-01 14:39:52</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>UNIT</t>
+          <t>은안</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Voor</t>
+          <t>Gucci와퍼</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>5_1</t>
+          <t>4_1</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -701,61 +701,61 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>UNIT_867166676(5골), Voor_845009676(1골)</t>
+          <t>은안_877143001(3골), 은안_866241236(1골), Gucci와퍼_864200104(1골)</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-09-30 16:46:35</t>
+          <t>2026-10-01 14:31:32</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>UNIT</t>
+          <t>호야국2인</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Voor</t>
+          <t>Special블루</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>2_3</t>
+          <t>3_3</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>패</t>
+          <t>무</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>UNIT_848180930(2골), Voor_845009676(1골), Voor_852233700(2골)</t>
+          <t>호야국2인_848232293(2골), 호야국2인_851216409(1골), Special블루_868001419(1골), Special블루_861047390(1골), Special블루_856246669(1골)</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-09-30 14:01:02</t>
+          <t>2026-10-01 14:21:07</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>UNIT</t>
+          <t>호야국2인</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>셀래스틴</t>
+          <t>Special블루</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>2_5</t>
+          <t>1_3</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -765,29 +765,29 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>UNIT_861221162(2골), 셀래스틴_861005680(4골), 셀래스틴_848231866(1골)</t>
+          <t>호야국2인_848232293(1골), Special블루_851251566(1골), Special블루_877001625(1골), Special블루_868001419(1골)</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-09-30 13:49:10</t>
+          <t>2026-10-01 14:08:57</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>UNIT</t>
+          <t>호야국2인</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>셀래스틴</t>
+          <t>비주류중독</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>5_3</t>
+          <t>3_2</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -797,24 +797,24 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>UNIT_867166676(3골), UNIT_861221162(2골), 셀래스틴_846001551(1골), 셀래스틴_852241461(1골), 셀래스틴_861005680(1골)</t>
+          <t>호야국2인_846192505(3골), 비주류중독_840052241(2골)</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-09-30 13:33:10</t>
+          <t>2026-10-01 13:58:38</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>UNIT</t>
+          <t>호야국2인</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>셀래스틴</t>
+          <t>비주류중독</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -829,19 +829,19 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>UNIT_848180930(1골), 셀래스틴_848194765(1골), 셀래스틴_861005680(3골), 셀래스틴_852241461(1골)</t>
+          <t>호야국2인_848232293(1골), 비주류중독_829203376(1골), 비주류중독_839247699(3골), 비주류중독_840052241(1골)</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-09-30 13:24:44</t>
+          <t>2026-10-01 13:48:03</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Gucci와퍼</t>
+          <t>호야국2인</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -851,66 +851,62 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>4_3</t>
+          <t>0_0</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>승</t>
-        </is>
-      </c>
-      <c r="F14" t="inlineStr">
-        <is>
-          <t>Gucci와퍼_864200104(4골), 비주류중독_840052241(1골), 비주류중독_825000240(1골), 비주류중독_839247699(1골)</t>
-        </is>
-      </c>
+          <t>패</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-09-30 13:21:00</t>
+          <t>2026-10-01 13:34:35</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>UNIT</t>
+          <t>아들러</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>셀래스틴</t>
+          <t>Special블루</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>2_0</t>
+          <t>1_2</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>승</t>
+          <t>패</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>UNIT_848180930(1골), UNIT_867166676(1골)</t>
+          <t>아들러_861000570(1골), Special블루_877001625(1골), Special블루_848230666(1골)</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-09-30 13:12:24</t>
+          <t>2026-10-01 13:24:02</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Gucci와퍼</t>
+          <t>아들러</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>비주류중독</t>
+          <t>Special블루</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -925,29 +921,29 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Gucci와퍼_852028765(1골), Gucci와퍼_852168473(1골), 비주류중독_834239977(1골), 비주류중독_840052241(1골), 비주류중독_839247699(1골)</t>
+          <t>아들러_855232639(2골), Special블루_868001419(1골), Special블루_877001625(2골)</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-09-30 13:10:05</t>
+          <t>2026-10-01 13:13:07</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>UNIT</t>
+          <t>앙쿠</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>셀래스틴</t>
+          <t>syma</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>4_3</t>
+          <t>7_0</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -957,221 +953,213 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>UNIT_867166676(3골), UNIT_840192883(1골), 셀래스틴_848194765(1골), 셀래스틴_861005680(2골)</t>
+          <t>앙쿠_863246191(4골), 앙쿠_851194765(2골), 앙쿠_856247103(1골)</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-09-30 12:57:48</t>
+          <t>2026-10-01 13:02:02</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>UNIT</t>
+          <t>앙쿠</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>셀래스틴</t>
+          <t>syma</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>3_1</t>
+          <t>0_0</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>승</t>
-        </is>
-      </c>
-      <c r="F18" t="inlineStr">
-        <is>
-          <t>UNIT_867166676(2골), UNIT_848180930(1골), 셀래스틴_846001551(1골)</t>
-        </is>
-      </c>
+          <t>패</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-09-30 12:35:39</t>
+          <t>2026-10-01 13:01:02</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>셀래스틴</t>
+          <t>앙쿠</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>비주류중독</t>
+          <t>syma</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>2_3</t>
+          <t>1_1</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>패</t>
+          <t>승</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>셀래스틴_846001551(1골), 셀래스틴_852241461(1골), 비주류중독_848006975(2골), 비주류중독_839247699(1골)</t>
+          <t>앙쿠_848176580(1골), syma_867192629(1골)</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-09-30 12:24:21</t>
+          <t>2026-10-01 12:49:37</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>셀래스틴</t>
+          <t>앙쿠</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>비주류중독</t>
+          <t>syma</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>2_0</t>
+          <t>0_0</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>승</t>
-        </is>
-      </c>
-      <c r="F20" t="inlineStr">
-        <is>
-          <t>셀래스틴_852241461(1골), 셀래스틴_861005680(1골)</t>
-        </is>
-      </c>
+          <t>패</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-09-30 12:00:21</t>
+          <t>2026-10-01 11:22:46</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>UNIT</t>
+          <t>앙쿠</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>셀래스틴</t>
+          <t>Gucci차붐</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>2_3</t>
+          <t>3_0</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>패</t>
+          <t>승</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>UNIT_848180930(2골), 셀래스틴_861005680(2골), 셀래스틴_852241461(1골)</t>
+          <t>앙쿠_851194765(1골), 앙쿠_863246191(2골)</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2026-09-30 09:47:20</t>
+          <t>2026-10-01 11:15:46</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>방덕</t>
+          <t>suma수마</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Voor</t>
+          <t>겐지간지</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>3_4</t>
+          <t>5_1</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>패</t>
+          <t>승</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>방덕_848007512(1골), 방덕_856228093(1골), 방덕_863184200(1골), Voor_845247090(2골), Voor_852233700(2골)</t>
+          <t>suma수마_861190046(1골), suma수마_861221162(3골), suma수마_845192190(1골), 겐지간지_848170890(1골)</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-09-30 09:35:39</t>
+          <t>2026-10-01 11:12:19</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>방덕</t>
+          <t>앙쿠</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Voor</t>
+          <t>Gucci차붐</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>1_6</t>
+          <t>3_1</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>패</t>
+          <t>승</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>방덕_101001419(1골), Voor_852233700(3골), Voor_845009676(2골), Voor_845247090(1골)</t>
+          <t>앙쿠_814226161(1골), 앙쿠_848176580(2골), Gucci차붐_840191208(1골)</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>2026-09-30 08:27:58</t>
+          <t>2026-10-01 11:03:11</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Legend독수리</t>
+          <t>suma수마</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>syma</t>
+          <t>겐지간지</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>3_2</t>
+          <t>5_3</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -1181,125 +1169,125 @@
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>Legend독수리_825190048(1골), Legend독수리_861081644(1골), Legend독수리_848188350(1골), syma_863228092(1골), syma_856233848(1골)</t>
+          <t>suma수마_861190046(2골), suma수마_861221162(1골), suma수마_840001114(2골), 겐지간지_814231747(1골), 겐지간지_852241461(1골), 겐지간지_856237679(1골)</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-09-30 08:16:55</t>
+          <t>2026-10-01 07:54:09</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Legend독수리</t>
+          <t>호야국2인</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>syma</t>
+          <t>아들러</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>1_6</t>
+          <t>3_2</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>패</t>
+          <t>승</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>Legend독수리_825190048(1골), syma_866231913(1골), syma_863262863(1골), syma_846001845(3골), syma_852274967(1골)</t>
+          <t>호야국2인_851261865(1골), 호야국2인_846192505(1골), 호야국2인_848232293(1골), 아들러_861000570(1골), 아들러_840191208(1골)</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>2026-09-30 08:04:48</t>
+          <t>2026-10-01 07:42:04</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Legend독수리</t>
+          <t>호야국2인</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>syma</t>
+          <t>아들러</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>2_2</t>
+          <t>5_2</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>무</t>
+          <t>승</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>Legend독수리_861215732(1골), Legend독수리_852209658(1골), syma_866231913(1골), syma_863228092(1골)</t>
+          <t>호야국2인_848227236(2골), 호야국2인_848232293(1골), 호야국2인_848216435(1골), 호야국2인_851216409(1골), 아들러_291225126(1골), 아들러_866251377(1골)</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-09-30 07:53:20</t>
+          <t>2026-10-01 06:47:50</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Legend독수리</t>
+          <t>호야국2인</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>syma</t>
+          <t>suma수마</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>1_2</t>
+          <t>4_2</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>패</t>
+          <t>승</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>Legend독수리_861215732(1골), syma_863222665(2골)</t>
+          <t>호야국2인_845198219(1골), 호야국2인_848232293(2골), 호야국2인_848216435(1골), suma수마_861190046(1골), suma수마_861221162(1골)</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>2026-09-29 14:16:03</t>
+          <t>2026-10-01 06:36:26</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>개포동덕배</t>
+          <t>호야국2인</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Gucci차붐</t>
+          <t>suma수마</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>7_2</t>
+          <t>5_2</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
@@ -1309,46 +1297,46 @@
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>개포동덕배_848206113(1골), 개포동덕배_845208722(1골), 개포동덕배_856202126(1골), 개포동덕배_845190048(4골), Gucci차붐_864247686(1골), Gucci차붐_864176403(1골)</t>
+          <t>호야국2인_851216409(1골), 호야국2인_845198219(1골), 호야국2인_846192505(1골), 호야국2인_848227236(1골), 호야국2인_848232293(1골), suma수마_861013383(1골), suma수마_861221162(1골)</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-09-29 14:04:54</t>
+          <t>2026-09-30 17:45:59</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>개포동덕배</t>
+          <t>UNIT</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Gucci차붐</t>
+          <t>Voor</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>4_2</t>
+          <t>2_5</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>승</t>
+          <t>패</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>개포동덕배_845190048(3골), 개포동덕배_848206113(1골), Gucci차붐_853272733(1골), Gucci차붐_853242004(1골)</t>
+          <t>UNIT_867166676(2골), Voor_845009676(1골), Voor_835183277(1골), Voor_852233700(3골)</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>2026-09-29 11:20:02</t>
+          <t>2026-09-30 17:34:22</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -1358,12 +1346,12 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>콩콩콩룔</t>
+          <t>Voor</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>1_3</t>
+          <t>3_4</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
@@ -1373,14 +1361,14 @@
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>UNIT_848180930(1골), 콩콩콩룔_867223848(1골), 콩콩콩룔_866223710(2골)</t>
+          <t>UNIT_848180930(2골), UNIT_840192883(1골), Voor_845009676(1골), Voor_856256079(1골), Voor_852233700(2골)</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-09-29 11:08:25</t>
+          <t>2026-09-30 17:17:18</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -1390,7 +1378,7 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>콩콩콩룔</t>
+          <t>Voor</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
@@ -1405,29 +1393,29 @@
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>UNIT_848180930(1골), UNIT_848135455(1골), UNIT_867166676(1골), 콩콩콩룔_866223710(1골), 콩콩콩룔_867223848(1골)</t>
+          <t>UNIT_867166676(1골), UNIT_848180930(2골), Voor_852233700(2골)</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>2026-09-29 10:56:21</t>
+          <t>2026-09-30 17:03:54</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>오스트리아</t>
+          <t>UNIT</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>ShangHaiPortFC</t>
+          <t>Voor</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>7_1</t>
+          <t>5_1</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
@@ -1437,14 +1425,14 @@
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>오스트리아_864199266(3골), 오스트리아_851221671(1골), 오스트리아_864182152(1골), 오스트리아_864140057(1골), 오스트리아_851216275(1골), ShangHaiPortFC_864191910(1골)</t>
+          <t>UNIT_867166676(5골), Voor_845009676(1골)</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-09-29 10:47:10</t>
+          <t>2026-09-30 16:46:35</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -1454,61 +1442,61 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>셀래스틴</t>
+          <t>Voor</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>3_2</t>
+          <t>2_3</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>승</t>
+          <t>패</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>UNIT_840228251(1골), UNIT_867166676(2골), 셀래스틴_848231866(1골), 셀래스틴_848230938(1골)</t>
+          <t>UNIT_848180930(2골), Voor_845009676(1골), Voor_852233700(2골)</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>2026-09-29 10:45:30</t>
+          <t>2026-09-30 14:01:02</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>오스트리아</t>
+          <t>UNIT</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>ShangHaiPortFC</t>
+          <t>셀래스틴</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>5_1</t>
+          <t>2_5</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>승</t>
+          <t>패</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>오스트리아_864140057(2골), 오스트리아_864182152(1골), 오스트리아_864199266(2골), ShangHaiPortFC_861051412(1골)</t>
+          <t>UNIT_861221162(2골), 셀래스틴_861005680(4골), 셀래스틴_848231866(1골)</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-09-29 10:35:32</t>
+          <t>2026-09-30 13:49:10</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -1523,24 +1511,24 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>1_3</t>
+          <t>5_3</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>패</t>
+          <t>승</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>UNIT_848180930(1골), 셀래스틴_846001551(1골), 셀래스틴_852241461(2골)</t>
+          <t>UNIT_867166676(3골), UNIT_861221162(2골), 셀래스틴_846001551(1골), 셀래스틴_852241461(1골), 셀래스틴_861005680(1골)</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>2026-09-29 10:18:25</t>
+          <t>2026-09-30 13:33:10</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -1555,61 +1543,61 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>2_1</t>
+          <t>1_5</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>승</t>
+          <t>패</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>UNIT_867166676(2골), 셀래스틴_848194765(1골)</t>
+          <t>UNIT_848180930(1골), 셀래스틴_848194765(1골), 셀래스틴_861005680(3골), 셀래스틴_852241461(1골)</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2026-09-29 09:24:43</t>
+          <t>2026-09-30 13:24:44</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>오스트리아</t>
+          <t>Gucci와퍼</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>셀래스틴</t>
+          <t>비주류중독</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>2_3</t>
+          <t>4_3</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>패</t>
+          <t>승</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>오스트리아_864199266(1골), 오스트리아_851236636(1골), 셀래스틴_846001551(1골), 셀래스틴_861005680(1골), 셀래스틴_848230938(1골)</t>
+          <t>Gucci와퍼_864200104(4골), 비주류중독_840052241(1골), 비주류중독_825000240(1골), 비주류중독_839247699(1골)</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>2026-09-29 09:13:08</t>
+          <t>2026-09-30 13:21:00</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>오스트리아</t>
+          <t>UNIT</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
@@ -1619,61 +1607,61 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>1_1</t>
+          <t>2_0</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>무</t>
+          <t>승</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>오스트리아_864199266(1골), 셀래스틴_861005680(1골)</t>
+          <t>UNIT_848180930(1골), UNIT_867166676(1골)</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2026-09-29 09:02:47</t>
+          <t>2026-09-30 13:12:24</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>오스트리아</t>
+          <t>Gucci와퍼</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>셀래스틴</t>
+          <t>비주류중독</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>3_1</t>
+          <t>2_3</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>승</t>
+          <t>패</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>오스트리아_864140057(1골), 오스트리아_864199266(1골), 오스트리아_864182152(1골), 셀래스틴_861005680(1골)</t>
+          <t>Gucci와퍼_852028765(1골), Gucci와퍼_852168473(1골), 비주류중독_834239977(1골), 비주류중독_840052241(1골), 비주류중독_839247699(1골)</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>2026-09-29 08:51:25</t>
+          <t>2026-09-30 13:10:05</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>오스트리아</t>
+          <t>UNIT</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
@@ -1683,47 +1671,783 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>0_2</t>
+          <t>4_3</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>패</t>
+          <t>승</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>셀래스틴_846001551(1골), 셀래스틴_861005680(1골)</t>
+          <t>UNIT_867166676(3골), UNIT_840192883(1골), 셀래스틴_848194765(1골), 셀래스틴_861005680(2골)</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
+          <t>2026-09-30 12:57:48</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>UNIT</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>셀래스틴</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>3_1</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>승</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>UNIT_867166676(2골), UNIT_848180930(1골), 셀래스틴_846001551(1골)</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>2026-09-30 12:35:39</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>셀래스틴</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>비주류중독</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>2_3</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>패</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>셀래스틴_846001551(1골), 셀래스틴_852241461(1골), 비주류중독_848006975(2골), 비주류중독_839247699(1골)</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>2026-09-30 12:24:21</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>셀래스틴</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>비주류중독</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>2_0</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>승</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>셀래스틴_852241461(1골), 셀래스틴_861005680(1골)</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>2026-09-30 12:00:21</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>UNIT</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>셀래스틴</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>2_3</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>패</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>UNIT_848180930(2골), 셀래스틴_861005680(2골), 셀래스틴_852241461(1골)</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>2026-09-30 09:47:20</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>방덕</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>Voor</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>3_4</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>패</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>방덕_848007512(1골), 방덕_856228093(1골), 방덕_863184200(1골), Voor_845247090(2골), Voor_852233700(2골)</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>2026-09-30 09:35:39</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>방덕</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>Voor</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>1_6</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>패</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>방덕_101001419(1골), Voor_852233700(3골), Voor_845009676(2골), Voor_845247090(1골)</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>2026-09-30 08:27:58</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>Legend독수리</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>syma</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>3_2</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>승</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>Legend독수리_825190048(1골), Legend독수리_861081644(1골), Legend독수리_848188350(1골), syma_863228092(1골), syma_856233848(1골)</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>2026-09-30 08:16:55</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>Legend독수리</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>syma</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>1_6</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>패</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>Legend독수리_825190048(1골), syma_866231913(1골), syma_863262863(1골), syma_846001845(3골), syma_852274967(1골)</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>2026-09-30 08:04:48</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>Legend독수리</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>syma</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>2_2</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>무</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>Legend독수리_861215732(1골), Legend독수리_852209658(1골), syma_866231913(1골), syma_863228092(1골)</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>2026-09-30 07:53:20</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>Legend독수리</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>syma</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>1_2</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>패</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>Legend독수리_861215732(1골), syma_863222665(2골)</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>2026-09-29 14:16:03</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>개포동덕배</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>Gucci차붐</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>7_2</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>승</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>개포동덕배_848206113(1골), 개포동덕배_845208722(1골), 개포동덕배_856202126(1골), 개포동덕배_845190048(4골), Gucci차붐_864247686(1골), Gucci차붐_864176403(1골)</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>2026-09-29 14:04:54</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>개포동덕배</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>Gucci차붐</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>4_2</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>승</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>개포동덕배_845190048(3골), 개포동덕배_848206113(1골), Gucci차붐_853272733(1골), Gucci차붐_853242004(1골)</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>2026-09-29 11:20:02</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>UNIT</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>콩콩콩룔</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>1_3</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>패</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>UNIT_848180930(1골), 콩콩콩룔_867223848(1골), 콩콩콩룔_866223710(2골)</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>2026-09-29 11:08:25</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>UNIT</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>콩콩콩룔</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>3_2</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>승</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>UNIT_848180930(1골), UNIT_848135455(1골), UNIT_867166676(1골), 콩콩콩룔_866223710(1골), 콩콩콩룔_867223848(1골)</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>2026-09-29 10:56:21</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>오스트리아</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>ShangHaiPortFC</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>7_1</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>승</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>오스트리아_864199266(3골), 오스트리아_851221671(1골), 오스트리아_864182152(1골), 오스트리아_864140057(1골), 오스트리아_851216275(1골), ShangHaiPortFC_864191910(1골)</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>2026-09-29 10:47:10</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>UNIT</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>셀래스틴</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>3_2</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>승</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>UNIT_840228251(1골), UNIT_867166676(2골), 셀래스틴_848231866(1골), 셀래스틴_848230938(1골)</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>2026-09-29 10:45:30</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>오스트리아</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>ShangHaiPortFC</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>5_1</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>승</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>오스트리아_864140057(2골), 오스트리아_864182152(1골), 오스트리아_864199266(2골), ShangHaiPortFC_861051412(1골)</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>2026-09-29 10:35:32</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>UNIT</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>셀래스틴</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>1_3</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>패</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>UNIT_848180930(1골), 셀래스틴_846001551(1골), 셀래스틴_852241461(2골)</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>2026-09-29 10:18:25</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>UNIT</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>셀래스틴</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>2_1</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>승</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>UNIT_867166676(2골), 셀래스틴_848194765(1골)</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>2026-09-29 09:24:43</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>오스트리아</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>셀래스틴</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>2_3</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>패</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>오스트리아_864199266(1골), 오스트리아_851236636(1골), 셀래스틴_846001551(1골), 셀래스틴_861005680(1골), 셀래스틴_848230938(1골)</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>2026-09-29 09:13:08</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>오스트리아</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>셀래스틴</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>1_1</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>무</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>오스트리아_864199266(1골), 셀래스틴_861005680(1골)</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>2026-09-29 09:02:47</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>오스트리아</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>셀래스틴</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>3_1</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>승</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>오스트리아_864140057(1골), 오스트리아_864199266(1골), 오스트리아_864182152(1골), 셀래스틴_861005680(1골)</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>2026-09-29 08:51:25</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>오스트리아</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>셀래스틴</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>0_2</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>패</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>셀래스틴_846001551(1골), 셀래스틴_861005680(1골)</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
           <t>2026-09-29 04:33:11</t>
         </is>
       </c>
-      <c r="B41" t="inlineStr">
+      <c r="B64" t="inlineStr">
         <is>
           <t>여수가스</t>
         </is>
       </c>
-      <c r="C41" t="inlineStr">
+      <c r="C64" t="inlineStr">
         <is>
           <t>오스트리아</t>
         </is>
       </c>
-      <c r="D41" t="inlineStr">
+      <c r="D64" t="inlineStr">
         <is>
           <t>2_3</t>
         </is>
       </c>
-      <c r="E41" t="inlineStr">
-        <is>
-          <t>패</t>
-        </is>
-      </c>
-      <c r="F41" t="inlineStr">
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>패</t>
+        </is>
+      </c>
+      <c r="F64" t="inlineStr">
         <is>
           <t>여수가스_828231747(1골), 여수가스_852274967(1골), 오스트리아_864191566(1골), 오스트리아_864199266(2골)</t>
         </is>
@@ -1740,7 +2464,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F41"/>
+  <dimension ref="A1:F64"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1778,86 +2502,86 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-10-01 07:54:09</t>
+          <t>2026-10-01 15:50:18</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>호야국2인</t>
+          <t>suma수마</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>아들러</t>
+          <t>피파왕초보구단주</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>3_2</t>
+          <t>1_3</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>승</t>
+          <t>패</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>호야국2인_848227236(2도움), 호야국2인_848232293(1도움), 아들러_866251377(1도움), 아들러_855232639(1도움)</t>
+          <t>suma수마_861221162(1도움), 피파왕초보구단주_867000027(1도움), 피파왕초보구단주_851243057(2도움)</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-10-01 07:42:04</t>
+          <t>2026-10-01 15:38:48</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>호야국2인</t>
+          <t>suma수마</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>아들러</t>
+          <t>피파왕초보구단주</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>5_2</t>
+          <t>2_2</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>승</t>
+          <t>무</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>호야국2인_848232293(2도움), 호야국2인_848217870(1도움), 호야국2인_851216409(1도움), 아들러_840191208(1도움)</t>
+          <t>suma수마_845192190(1도움), suma수마_861190046(1도움), 피파왕초보구단주_867000027(1도움)</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-10-01 06:47:50</t>
+          <t>2026-10-01 15:24:08</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>호야국2인</t>
+          <t>피파왕초보구단주</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>suma수마</t>
+          <t>Gucci와퍼</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>4_2</t>
+          <t>5_1</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -1867,61 +2591,61 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>호야국2인_848217870(1도움), 호야국2인_848232293(1도움), 호야국2인_852001183(1도움), suma수마_861190046(1도움), suma수마_848225439(1도움)</t>
+          <t>피파왕초보구단주_846208722(1도움), 피파왕초보구단주_856209331(1도움), 피파왕초보구단주_851243057(1도움), 피파왕초보구단주_867000027(1도움), Gucci와퍼_864200104(1도움)</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-10-01 06:36:26</t>
+          <t>2026-10-01 15:12:09</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>호야국2인</t>
+          <t>피파왕초보구단주</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>suma수마</t>
+          <t>Gucci와퍼</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>5_2</t>
+          <t>3_3</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>승</t>
+          <t>무</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>호야국2인_851216409(1도움), 호야국2인_845198219(1도움), 호야국2인_846192505(1도움), 호야국2인_848216435(1도움), suma수마_826223697(1도움)</t>
+          <t>피파왕초보구단주_846208722(1도움), 피파왕초보구단주_867000027(1도움), Gucci와퍼_852208128(1도움), Gucci와퍼_864200104(1도움), Gucci와퍼_852168473(1도움)</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-09-30 17:45:59</t>
+          <t>2026-10-01 14:56:12</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>UNIT</t>
+          <t>0708ManUtd</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Voor</t>
+          <t>호야국2인</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>2_5</t>
+          <t>1_2</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -1931,29 +2655,29 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>UNIT_840192883(1도움), Voor_856256079(1도움), Voor_861000027(4도움)</t>
+          <t>호야국2인_848232293(1도움), 호야국2인_846192505(1도움)</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-09-30 17:34:22</t>
+          <t>2026-10-01 14:51:31</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>UNIT</t>
+          <t>은안</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Voor</t>
+          <t>Gucci와퍼</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>3_4</t>
+          <t>1_4</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -1963,61 +2687,61 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>UNIT_861221162(1도움), UNIT_866247257(1도움), UNIT_840228251(1도움), Voor_845009676(1도움), Voor_858025420(1도움), Voor_835183277(1도움)</t>
+          <t>은안_866241236(1도움), Gucci와퍼_851210697(1도움), Gucci와퍼_852208128(1도움), Gucci와퍼_840208574(1도움), Gucci와퍼_852010264(1도움)</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-09-30 17:17:18</t>
+          <t>2026-10-01 14:45:02</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>UNIT</t>
+          <t>0708ManUtd</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Voor</t>
+          <t>호야국2인</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>3_2</t>
+          <t>2_3</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>승</t>
+          <t>패</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>UNIT_840228251(1도움), UNIT_840192883(1도움), UNIT_848135455(1도움), Voor_845239231(1도움), Voor_845009676(1도움)</t>
+          <t>0708ManUtd_834239053(1도움), 호야국2인_846192505(1도움)</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-09-30 17:03:54</t>
+          <t>2026-10-01 14:39:52</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>UNIT</t>
+          <t>은안</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Voor</t>
+          <t>Gucci와퍼</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>5_1</t>
+          <t>4_1</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -2027,61 +2751,61 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>UNIT_848180930(1도움), UNIT_840192883(1도움), UNIT_848265695(3도움), Voor_852233700(1도움)</t>
+          <t>은안_848231866(1도움), 은안_856251517(1도움), 은안_856246420(1도움), 은안_866241236(1도움), Gucci와퍼_861139720(1도움)</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-09-30 16:46:35</t>
+          <t>2026-10-01 14:31:32</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>UNIT</t>
+          <t>호야국2인</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Voor</t>
+          <t>Special블루</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>2_3</t>
+          <t>3_3</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>패</t>
+          <t>무</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>UNIT_840228251(1도움), UNIT_840192883(1도움), Voor_845009676(1도움), Voor_846184943(1도움), Voor_852233700(1도움)</t>
+          <t>호야국2인_851216409(1도움), 호야국2인_845198219(1도움), Special블루_877001625(2도움), Special블루_861006975(1도움)</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-09-30 14:01:02</t>
+          <t>2026-10-01 14:21:07</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>UNIT</t>
+          <t>호야국2인</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>셀래스틴</t>
+          <t>Special블루</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>2_5</t>
+          <t>1_3</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -2091,29 +2815,29 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>UNIT_867166676(2도움), 셀래스틴_848194765(1도움), 셀래스틴_848231866(1도움), 셀래스틴_852241461(1도움)</t>
+          <t>호야국2인_846192505(1도움), Special블루_861006975(1도움), Special블루_856246669(2도움)</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-09-30 13:49:10</t>
+          <t>2026-10-01 14:08:57</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>UNIT</t>
+          <t>호야국2인</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>셀래스틴</t>
+          <t>비주류중독</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>5_3</t>
+          <t>3_2</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -2123,24 +2847,24 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>UNIT_840210736(2도움), UNIT_867166676(1도움), UNIT_848135455(1도움), UNIT_840192883(1도움), 셀래스틴_863200458(1도움), 셀래스틴_852241461(2도움)</t>
+          <t>호야국2인_848216435(1도움), 호야국2인_845198219(1도움), 호야국2인_851261865(1도움), 비주류중독_839247699(1도움), 비주류중독_848006975(1도움)</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-09-30 13:33:10</t>
+          <t>2026-10-01 13:58:38</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>UNIT</t>
+          <t>호야국2인</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>셀래스틴</t>
+          <t>비주류중독</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -2155,19 +2879,19 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>UNIT_840192883(1도움), 셀래스틴_863200458(1도움), 셀래스틴_852259694(1도움), 셀래스틴_861005680(1도움)</t>
+          <t>비주류중독_848006975(3도움), 비주류중독_839247699(1도움), 비주류중독_840052241(1도움)</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-09-30 13:24:44</t>
+          <t>2026-10-01 13:48:03</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Gucci와퍼</t>
+          <t>호야국2인</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -2177,66 +2901,62 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>4_3</t>
+          <t>0_0</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>승</t>
-        </is>
-      </c>
-      <c r="F14" t="inlineStr">
-        <is>
-          <t>Gucci와퍼_852168473(3도움), Gucci와퍼_852028765(1도움), 비주류중독_840052241(1도움), 비주류중독_862180283(1도움)</t>
-        </is>
-      </c>
+          <t>패</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-09-30 13:21:00</t>
+          <t>2026-10-01 13:34:35</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>UNIT</t>
+          <t>아들러</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>셀래스틴</t>
+          <t>Special블루</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>2_0</t>
+          <t>1_2</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>승</t>
+          <t>패</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>UNIT_840192883(1도움), UNIT_840228251(1도움)</t>
+          <t>아들러_840191208(1도움), Special블루_877001625(1도움)</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-09-30 13:12:24</t>
+          <t>2026-10-01 13:24:02</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Gucci와퍼</t>
+          <t>아들러</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>비주류중독</t>
+          <t>Special블루</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -2251,29 +2971,29 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Gucci와퍼_852010264(1도움), 비주류중독_834239977(1도움), 비주류중독_848006975(1도움)</t>
+          <t>아들러_866251377(1도움), 아들러_861000570(1도움), Special블루_856246669(1도움), Special블루_848230666(1도움), Special블루_861006975(1도움)</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-09-30 13:10:05</t>
+          <t>2026-10-01 13:13:07</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>UNIT</t>
+          <t>앙쿠</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>셀래스틴</t>
+          <t>syma</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>4_3</t>
+          <t>7_0</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -2283,221 +3003,213 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>UNIT_867166676(1도움), UNIT_840192883(2도움), UNIT_840225782(1도움), 셀래스틴_848194765(1도움), 셀래스틴_863200458(1도움)</t>
+          <t>앙쿠_848176580(5도움)</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-09-30 12:57:48</t>
+          <t>2026-10-01 13:02:02</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>UNIT</t>
+          <t>앙쿠</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>셀래스틴</t>
+          <t>syma</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>3_1</t>
+          <t>0_0</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>승</t>
-        </is>
-      </c>
-      <c r="F18" t="inlineStr">
-        <is>
-          <t>UNIT_863250723(1도움), UNIT_840228251(2도움), 셀래스틴_852241461(1도움)</t>
-        </is>
-      </c>
+          <t>패</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-09-30 12:35:39</t>
+          <t>2026-10-01 13:01:02</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>셀래스틴</t>
+          <t>앙쿠</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>비주류중독</t>
+          <t>syma</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>2_3</t>
+          <t>1_1</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>패</t>
+          <t>승</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>셀래스틴_848231866(1도움), 셀래스틴_852259694(1도움), 비주류중독_839247699(1도움), 비주류중독_834239977(2도움)</t>
+          <t>앙쿠_856247103(1도움), syma_851236295(1도움)</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-09-30 12:24:21</t>
+          <t>2026-10-01 12:49:37</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>셀래스틴</t>
+          <t>앙쿠</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>비주류중독</t>
+          <t>syma</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>2_0</t>
+          <t>0_0</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>승</t>
-        </is>
-      </c>
-      <c r="F20" t="inlineStr">
-        <is>
-          <t>셀래스틴_852259694(1도움), 셀래스틴_848194765(1도움)</t>
-        </is>
-      </c>
+          <t>패</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-09-30 12:00:21</t>
+          <t>2026-10-01 11:22:46</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>UNIT</t>
+          <t>앙쿠</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>셀래스틴</t>
+          <t>Gucci차붐</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>2_3</t>
+          <t>3_0</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>패</t>
+          <t>승</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>UNIT_840225782(1도움), UNIT_867166676(1도움), 셀래스틴_848013038(1도움), 셀래스틴_852241461(2도움)</t>
+          <t>앙쿠_851194765(1도움), 앙쿠_848176580(1도움)</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2026-09-30 09:47:20</t>
+          <t>2026-10-01 11:15:46</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>방덕</t>
+          <t>suma수마</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Voor</t>
+          <t>겐지간지</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>3_4</t>
+          <t>5_1</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>패</t>
+          <t>승</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>방덕_867001040(1도움), 방덕_848231478(2도움), Voor_845009676(1도움), Voor_845239231(1도움), Voor_835183277(1도움), Voor_848216150(1도움)</t>
+          <t>suma수마_851234112(1도움), suma수마_840001114(1도움), suma수마_861190046(1도움), suma수마_848225439(1도움), 겐지간지_845183898(1도움)</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-09-30 09:35:39</t>
+          <t>2026-10-01 11:12:19</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>방덕</t>
+          <t>앙쿠</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Voor</t>
+          <t>Gucci차붐</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>1_6</t>
+          <t>3_1</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>패</t>
+          <t>승</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>Voor_852233700(2도움), Voor_856256079(1도움), Voor_845009676(2도움), Voor_835183277(1도움)</t>
+          <t>앙쿠_851194765(1도움), 앙쿠_848176580(1도움), 앙쿠_863246191(1도움), Gucci차붐_861182521(1도움)</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>2026-09-30 08:27:58</t>
+          <t>2026-10-01 11:03:11</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Legend독수리</t>
+          <t>suma수마</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>syma</t>
+          <t>겐지간지</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>3_2</t>
+          <t>5_3</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -2507,125 +3219,125 @@
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>Legend독수리_861215732(1도움), Legend독수리_852209658(1도움), syma_852274967(1도움), syma_863228092(1도움)</t>
+          <t>suma수마_861013383(2도움), suma수마_826223697(1도움), suma수마_861221162(1도움), suma수마_840001114(1도움), 겐지간지_852231443(1도움), 겐지간지_845158023(2도움)</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-09-30 08:16:55</t>
+          <t>2026-10-01 07:54:09</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Legend독수리</t>
+          <t>호야국2인</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>syma</t>
+          <t>아들러</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>1_6</t>
+          <t>3_2</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>패</t>
+          <t>승</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>Legend독수리_861215732(1도움), syma_866231913(2도움), syma_863222665(4도움)</t>
+          <t>호야국2인_848227236(2도움), 호야국2인_848232293(1도움), 아들러_866251377(1도움), 아들러_855232639(1도움)</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>2026-09-30 08:04:48</t>
+          <t>2026-10-01 07:42:04</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Legend독수리</t>
+          <t>호야국2인</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>syma</t>
+          <t>아들러</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>2_2</t>
+          <t>5_2</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>무</t>
+          <t>승</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>Legend독수리_848224425(1도움), Legend독수리_826236703(1도움), syma_856233848(1도움)</t>
+          <t>호야국2인_848232293(2도움), 호야국2인_848217870(1도움), 호야국2인_851216409(1도움), 아들러_840191208(1도움)</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-09-30 07:53:20</t>
+          <t>2026-10-01 06:47:50</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Legend독수리</t>
+          <t>호야국2인</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>syma</t>
+          <t>suma수마</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>1_2</t>
+          <t>4_2</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>패</t>
+          <t>승</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>Legend독수리_861081644(1도움), syma_846001845(2도움)</t>
+          <t>호야국2인_848217870(1도움), 호야국2인_848232293(1도움), 호야국2인_852001183(1도움), suma수마_861190046(1도움), suma수마_848225439(1도움)</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>2026-09-29 14:16:03</t>
+          <t>2026-10-01 06:36:26</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>개포동덕배</t>
+          <t>호야국2인</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Gucci차붐</t>
+          <t>suma수마</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>7_2</t>
+          <t>5_2</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
@@ -2635,46 +3347,46 @@
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>개포동덕배_848206113(1도움), 개포동덕배_845208722(3도움), 개포동덕배_856202126(1도움), 개포동덕배_863212622(2도움), Gucci차붐_853272733(1도움), Gucci차붐_864176403(1도움)</t>
+          <t>호야국2인_851216409(1도움), 호야국2인_845198219(1도움), 호야국2인_846192505(1도움), 호야국2인_848216435(1도움), suma수마_826223697(1도움)</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-09-29 14:04:54</t>
+          <t>2026-09-30 17:45:59</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>개포동덕배</t>
+          <t>UNIT</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Gucci차붐</t>
+          <t>Voor</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>4_2</t>
+          <t>2_5</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>승</t>
+          <t>패</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>개포동덕배_856202126(1도움), 개포동덕배_863234396(1도움), 개포동덕배_856275298(1도움), 개포동덕배_848206113(1도움), Gucci차붐_864084333(1도움), Gucci차붐_864247686(1도움)</t>
+          <t>UNIT_840192883(1도움), Voor_856256079(1도움), Voor_861000027(4도움)</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>2026-09-29 11:20:02</t>
+          <t>2026-09-30 17:34:22</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -2684,12 +3396,12 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>콩콩콩룔</t>
+          <t>Voor</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>1_3</t>
+          <t>3_4</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
@@ -2699,14 +3411,14 @@
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>UNIT_867166676(1도움), 콩콩콩룔_867220502(1도움), 콩콩콩룔_848189505(2도움)</t>
+          <t>UNIT_861221162(1도움), UNIT_866247257(1도움), UNIT_840228251(1도움), Voor_845009676(1도움), Voor_858025420(1도움), Voor_835183277(1도움)</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-09-29 11:08:25</t>
+          <t>2026-09-30 17:17:18</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -2716,7 +3428,7 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>콩콩콩룔</t>
+          <t>Voor</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
@@ -2731,29 +3443,29 @@
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>UNIT_840192883(2도움), UNIT_848265695(1도움), 콩콩콩룔_851236496(1도움)</t>
+          <t>UNIT_840228251(1도움), UNIT_840192883(1도움), UNIT_848135455(1도움), Voor_845239231(1도움), Voor_845009676(1도움)</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>2026-09-29 10:56:21</t>
+          <t>2026-09-30 17:03:54</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>오스트리아</t>
+          <t>UNIT</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>ShangHaiPortFC</t>
+          <t>Voor</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>7_1</t>
+          <t>5_1</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
@@ -2763,14 +3475,14 @@
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>오스트리아_864182152(2도움), 오스트리아_864140057(1도움), 오스트리아_851236636(4도움), ShangHaiPortFC_848031432(1도움)</t>
+          <t>UNIT_848180930(1도움), UNIT_840192883(1도움), UNIT_848265695(3도움), Voor_852233700(1도움)</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-09-29 10:47:10</t>
+          <t>2026-09-30 16:46:35</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -2780,61 +3492,61 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>셀래스틴</t>
+          <t>Voor</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>3_2</t>
+          <t>2_3</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>승</t>
+          <t>패</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>UNIT_848180930(1도움), UNIT_863250723(1도움), UNIT_840192883(1도움), 셀래스틴_846001551(1도움)</t>
+          <t>UNIT_840228251(1도움), UNIT_840192883(1도움), Voor_845009676(1도움), Voor_846184943(1도움), Voor_852233700(1도움)</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>2026-09-29 10:45:30</t>
+          <t>2026-09-30 14:01:02</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>오스트리아</t>
+          <t>UNIT</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>ShangHaiPortFC</t>
+          <t>셀래스틴</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>5_1</t>
+          <t>2_5</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>승</t>
+          <t>패</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>오스트리아_851221671(1도움), 오스트리아_863223671(1도움), 오스트리아_863240709(1도움), 오스트리아_864140057(1도움), 오스트리아_851216275(1도움), ShangHaiPortFC_827143001(1도움)</t>
+          <t>UNIT_867166676(2도움), 셀래스틴_848194765(1도움), 셀래스틴_848231866(1도움), 셀래스틴_852241461(1도움)</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-09-29 10:35:32</t>
+          <t>2026-09-30 13:49:10</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -2849,24 +3561,24 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>1_3</t>
+          <t>5_3</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>패</t>
+          <t>승</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>UNIT_867166676(1도움), 셀래스틴_848231866(2도움), 셀래스틴_852241461(1도움)</t>
+          <t>UNIT_840210736(2도움), UNIT_867166676(1도움), UNIT_848135455(1도움), UNIT_840192883(1도움), 셀래스틴_863200458(1도움), 셀래스틴_852241461(2도움)</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>2026-09-29 10:18:25</t>
+          <t>2026-09-30 13:33:10</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -2881,61 +3593,61 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>2_1</t>
+          <t>1_5</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>승</t>
+          <t>패</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>UNIT_839013383(1도움), UNIT_840192883(1도움), 셀래스틴_846001551(1도움)</t>
+          <t>UNIT_840192883(1도움), 셀래스틴_863200458(1도움), 셀래스틴_852259694(1도움), 셀래스틴_861005680(1도움)</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2026-09-29 09:24:43</t>
+          <t>2026-09-30 13:24:44</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>오스트리아</t>
+          <t>Gucci와퍼</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>셀래스틴</t>
+          <t>비주류중독</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>2_3</t>
+          <t>4_3</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>패</t>
+          <t>승</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>오스트리아_864199266(1도움), 오스트리아_863240709(1도움), 셀래스틴_846001551(1도움), 셀래스틴_848194765(2도움)</t>
+          <t>Gucci와퍼_852168473(3도움), Gucci와퍼_852028765(1도움), 비주류중독_840052241(1도움), 비주류중독_862180283(1도움)</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>2026-09-29 09:13:08</t>
+          <t>2026-09-30 13:21:00</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>오스트리아</t>
+          <t>UNIT</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
@@ -2945,61 +3657,61 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>1_1</t>
+          <t>2_0</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>무</t>
+          <t>승</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>오스트리아_851221671(1도움), 셀래스틴_848231866(1도움)</t>
+          <t>UNIT_840192883(1도움), UNIT_840228251(1도움)</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2026-09-29 09:02:47</t>
+          <t>2026-09-30 13:12:24</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>오스트리아</t>
+          <t>Gucci와퍼</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>셀래스틴</t>
+          <t>비주류중독</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>3_1</t>
+          <t>2_3</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>승</t>
+          <t>패</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>오스트리아_864140057(1도움), 오스트리아_864182152(1도움), 오스트리아_851236636(1도움), 셀래스틴_846001551(1도움)</t>
+          <t>Gucci와퍼_852010264(1도움), 비주류중독_834239977(1도움), 비주류중독_848006975(1도움)</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>2026-09-29 08:51:25</t>
+          <t>2026-09-30 13:10:05</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>오스트리아</t>
+          <t>UNIT</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
@@ -3009,47 +3721,783 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>0_2</t>
+          <t>4_3</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>패</t>
+          <t>승</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>셀래스틴_863200458(1도움), 셀래스틴_852241461(1도움)</t>
+          <t>UNIT_867166676(1도움), UNIT_840192883(2도움), UNIT_840225782(1도움), 셀래스틴_848194765(1도움), 셀래스틴_863200458(1도움)</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
+          <t>2026-09-30 12:57:48</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>UNIT</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>셀래스틴</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>3_1</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>승</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>UNIT_863250723(1도움), UNIT_840228251(2도움), 셀래스틴_852241461(1도움)</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>2026-09-30 12:35:39</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>셀래스틴</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>비주류중독</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>2_3</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>패</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>셀래스틴_848231866(1도움), 셀래스틴_852259694(1도움), 비주류중독_839247699(1도움), 비주류중독_834239977(2도움)</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>2026-09-30 12:24:21</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>셀래스틴</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>비주류중독</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>2_0</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>승</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>셀래스틴_852259694(1도움), 셀래스틴_848194765(1도움)</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>2026-09-30 12:00:21</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>UNIT</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>셀래스틴</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>2_3</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>패</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>UNIT_840225782(1도움), UNIT_867166676(1도움), 셀래스틴_848013038(1도움), 셀래스틴_852241461(2도움)</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>2026-09-30 09:47:20</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>방덕</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>Voor</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>3_4</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>패</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>방덕_867001040(1도움), 방덕_848231478(2도움), Voor_845009676(1도움), Voor_845239231(1도움), Voor_835183277(1도움), Voor_848216150(1도움)</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>2026-09-30 09:35:39</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>방덕</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>Voor</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>1_6</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>패</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>Voor_852233700(2도움), Voor_856256079(1도움), Voor_845009676(2도움), Voor_835183277(1도움)</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>2026-09-30 08:27:58</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>Legend독수리</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>syma</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>3_2</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>승</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>Legend독수리_861215732(1도움), Legend독수리_852209658(1도움), syma_852274967(1도움), syma_863228092(1도움)</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>2026-09-30 08:16:55</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>Legend독수리</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>syma</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>1_6</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>패</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>Legend독수리_861215732(1도움), syma_866231913(2도움), syma_863222665(4도움)</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>2026-09-30 08:04:48</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>Legend독수리</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>syma</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>2_2</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>무</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>Legend독수리_848224425(1도움), Legend독수리_826236703(1도움), syma_856233848(1도움)</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>2026-09-30 07:53:20</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>Legend독수리</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>syma</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>1_2</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>패</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>Legend독수리_861081644(1도움), syma_846001845(2도움)</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>2026-09-29 14:16:03</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>개포동덕배</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>Gucci차붐</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>7_2</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>승</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>개포동덕배_848206113(1도움), 개포동덕배_845208722(3도움), 개포동덕배_856202126(1도움), 개포동덕배_863212622(2도움), Gucci차붐_853272733(1도움), Gucci차붐_864176403(1도움)</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>2026-09-29 14:04:54</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>개포동덕배</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>Gucci차붐</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>4_2</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>승</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>개포동덕배_856202126(1도움), 개포동덕배_863234396(1도움), 개포동덕배_856275298(1도움), 개포동덕배_848206113(1도움), Gucci차붐_864084333(1도움), Gucci차붐_864247686(1도움)</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>2026-09-29 11:20:02</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>UNIT</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>콩콩콩룔</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>1_3</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>패</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>UNIT_867166676(1도움), 콩콩콩룔_867220502(1도움), 콩콩콩룔_848189505(2도움)</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>2026-09-29 11:08:25</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>UNIT</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>콩콩콩룔</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>3_2</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>승</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>UNIT_840192883(2도움), UNIT_848265695(1도움), 콩콩콩룔_851236496(1도움)</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>2026-09-29 10:56:21</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>오스트리아</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>ShangHaiPortFC</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>7_1</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>승</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>오스트리아_864182152(2도움), 오스트리아_864140057(1도움), 오스트리아_851236636(4도움), ShangHaiPortFC_848031432(1도움)</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>2026-09-29 10:47:10</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>UNIT</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>셀래스틴</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>3_2</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>승</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>UNIT_848180930(1도움), UNIT_863250723(1도움), UNIT_840192883(1도움), 셀래스틴_846001551(1도움)</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>2026-09-29 10:45:30</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>오스트리아</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>ShangHaiPortFC</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>5_1</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>승</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>오스트리아_851221671(1도움), 오스트리아_863223671(1도움), 오스트리아_863240709(1도움), 오스트리아_864140057(1도움), 오스트리아_851216275(1도움), ShangHaiPortFC_827143001(1도움)</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>2026-09-29 10:35:32</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>UNIT</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>셀래스틴</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>1_3</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>패</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>UNIT_867166676(1도움), 셀래스틴_848231866(2도움), 셀래스틴_852241461(1도움)</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>2026-09-29 10:18:25</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>UNIT</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>셀래스틴</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>2_1</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>승</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>UNIT_839013383(1도움), UNIT_840192883(1도움), 셀래스틴_846001551(1도움)</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>2026-09-29 09:24:43</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>오스트리아</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>셀래스틴</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>2_3</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>패</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>오스트리아_864199266(1도움), 오스트리아_863240709(1도움), 셀래스틴_846001551(1도움), 셀래스틴_848194765(2도움)</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>2026-09-29 09:13:08</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>오스트리아</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>셀래스틴</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>1_1</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>무</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>오스트리아_851221671(1도움), 셀래스틴_848231866(1도움)</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>2026-09-29 09:02:47</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>오스트리아</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>셀래스틴</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>3_1</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>승</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>오스트리아_864140057(1도움), 오스트리아_864182152(1도움), 오스트리아_851236636(1도움), 셀래스틴_846001551(1도움)</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>2026-09-29 08:51:25</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>오스트리아</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>셀래스틴</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>0_2</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>패</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>셀래스틴_863200458(1도움), 셀래스틴_852241461(1도움)</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
           <t>2026-09-29 04:33:11</t>
         </is>
       </c>
-      <c r="B41" t="inlineStr">
+      <c r="B64" t="inlineStr">
         <is>
           <t>여수가스</t>
         </is>
       </c>
-      <c r="C41" t="inlineStr">
+      <c r="C64" t="inlineStr">
         <is>
           <t>오스트리아</t>
         </is>
       </c>
-      <c r="D41" t="inlineStr">
+      <c r="D64" t="inlineStr">
         <is>
           <t>2_3</t>
         </is>
       </c>
-      <c r="E41" t="inlineStr">
-        <is>
-          <t>패</t>
-        </is>
-      </c>
-      <c r="F41" t="inlineStr">
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>패</t>
+        </is>
+      </c>
+      <c r="F64" t="inlineStr">
         <is>
           <t>여수가스_852216393(1도움), 여수가스_861162895(1도움), 오스트리아_864140057(1도움), 오스트리아_851257075(1도움)</t>
         </is>

</xml_diff>

<commit_message>
Update: Dashboard HTML (06:07:07)
</commit_message>
<xml_diff>
--- a/API데이터_경기_득점_및_도움_기록.xlsx
+++ b/API데이터_경기_득점_및_도움_기록.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F12"/>
+  <dimension ref="A1:F56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -452,54 +452,54 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-10-07 13:51:44</t>
+          <t>2026-10-09 13:36:17</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>앙쿠</t>
+          <t>검정소</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>셀래스틴</t>
+          <t>콩콩콩룔</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>6_2</t>
+          <t>3_3</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>승</t>
+          <t>무</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>앙쿠_848176580(1골), 앙쿠_861049369(3골), 앙쿠_851194765(2골), 셀래스틴_848194765(1골), 셀래스틴_861005680(1골)</t>
+          <t>검정소_868192181(3골), 콩콩콩룔_866223710(3골)</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-10-07 13:39:26</t>
+          <t>2026-10-09 13:33:58</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>UNIT</t>
+          <t>셀래스틴</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>셀래스틴</t>
+          <t>syma</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>4_2</t>
+          <t>2_0</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -509,29 +509,29 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>UNIT_867166676(3골), UNIT_848180930(1골), 셀래스틴_863233419(1골), 셀래스틴_861005680(1골)</t>
+          <t>셀래스틴_852241461(2골)</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-10-07 13:28:13</t>
+          <t>2026-10-09 13:25:18</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>앙쿠</t>
+          <t>검정소</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>UNIT</t>
+          <t>콩콩콩룔</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>2_1</t>
+          <t>10_4</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -541,51 +541,51 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>앙쿠_866266039(1골), 앙쿠_861049369(1골), UNIT_863250723(1골)</t>
+          <t>검정소_868192181(5골), 검정소_100214100(5골), 콩콩콩룔_866223710(1골), 콩콩콩룔_867223848(2골), 콩콩콩룔_848189505(1골)</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-10-07 13:16:19</t>
+          <t>2026-10-09 13:23:55</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>앙쿠</t>
+          <t>셀래스틴</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>셀래스틴</t>
+          <t>syma</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>2_3</t>
+          <t>3_2</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>패</t>
+          <t>승</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>앙쿠_861049369(1골), 앙쿠_848176580(1골), 셀래스틴_861005680(2골), 셀래스틴_848231866(1골)</t>
+          <t>셀래스틴_863233419(2골), 셀래스틴_848194765(1골), syma_861000041(1골), syma_839191695(1골)</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-10-07 13:05:29</t>
+          <t>2026-10-09 05:08:26</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>UNIT</t>
+          <t>ZD장인지참치</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -595,39 +595,39 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>1_3</t>
+          <t>5_1</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>패</t>
+          <t>승</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>UNIT_867166676(1골), 셀래스틴_861005680(2골), 셀래스틴_852241461(1골)</t>
+          <t>ZD장인지참치_840191208(2골), ZD장인지참치_848199503(1골), ZD장인지참치_839200104(2골), 셀래스틴_861005680(1골)</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-10-07 12:50:50</t>
+          <t>2026-10-09 04:53:33</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>앙쿠</t>
+          <t>ZD장인지참치</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>UNIT</t>
+          <t>셀래스틴</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>2_5</t>
+          <t>3_6</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -637,29 +637,29 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>앙쿠_851194765(1골), 앙쿠_861049369(1골), UNIT_848180930(3골), UNIT_867166676(2골)</t>
+          <t>ZD장인지참치_848199503(1골), ZD장인지참치_839200104(1골), ZD장인지참치_840191208(1골), 셀래스틴_861005680(1골), 셀래스틴_848230938(1골), 셀래스틴_863233419(1골), 셀래스틴_852241461(3골)</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-10-07 12:30:57</t>
+          <t>2026-10-09 04:42:24</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>UNIT</t>
+          <t>ZD장인지참치</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>ZD장인지참치</t>
+          <t>셀래스틴</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>2_1</t>
+          <t>4_2</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -669,19 +669,19 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>UNIT_867166676(2골), ZD장인지참치_840191208(1골)</t>
+          <t>ZD장인지참치_839200104(2골), ZD장인지참치_840256630(2골), 셀래스틴_861005680(2골)</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-10-07 12:14:34</t>
+          <t>2026-10-09 04:31:15</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>앙쿠</t>
+          <t>ZD장인지참치</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -691,29 +691,29 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>3_0</t>
+          <t>3_4</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>승</t>
+          <t>패</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>앙쿠_861049369(1골), 앙쿠_848176580(1골), 앙쿠_866266039(1골)</t>
+          <t>ZD장인지참치_851240740(1골), ZD장인지참치_839200104(1골), ZD장인지참치_840191208(1골), 셀래스틴_852241461(2골), 셀래스틴_863233419(1골), 셀래스틴_863200458(1골)</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-10-07 12:04:29</t>
+          <t>2026-10-09 04:19:11</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>앙쿠</t>
+          <t>ZD장인지참치</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -723,7 +723,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>3_1</t>
+          <t>2_1</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -733,29 +733,29 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>앙쿠_861049369(2골), 앙쿠_866266039(1골), 셀래스틴_852241461(1골)</t>
+          <t>ZD장인지참치_840191208(1골), ZD장인지참치_839200104(1골), 셀래스틴_852241461(1골)</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-10-07 11:33:41</t>
+          <t>2026-10-09 04:04:37</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>겐지간지</t>
+          <t>UNIT</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>용신</t>
+          <t>셀래스틴</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>0_3</t>
+          <t>0_0</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -763,39 +763,1439 @@
           <t>패</t>
         </is>
       </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>용신_825212188(3골)</t>
-        </is>
-      </c>
+      <c r="F11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
+          <t>2026-10-09 03:48:59</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>UNIT</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>셀래스틴</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>1_0</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>승</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>UNIT_863250723(1골)</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2026-10-09 02:36:22</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>syma</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>용신</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>1_2</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>패</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>syma_867192629(1골), 용신_866200104(1골), 용신_804264453(1골)</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-10-09 02:26:03</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>syma</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>용신</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>2_3</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>패</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>syma_848192638(1골), syma_845224574(1골), 용신_101173731(2골), 용신_866200104(1골)</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>2026-10-08 17:16:26</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>UNIT</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Voor</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>5_4</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>승</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>UNIT_848180930(3골), UNIT_840192883(2골), Voor_858025420(1골), Voor_852233700(2골), Voor_845009676(1골)</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-10-08 17:00:32</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>UNIT</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Voor</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>2_1</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>승</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>UNIT_867166676(1골), UNIT_848180930(1골), Voor_845009676(1골)</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2026-10-08 16:48:25</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>UNIT</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Voor</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>0_2</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>패</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>Voor_845009676(2골)</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>2026-10-08 16:33:10</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>검정소</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Voor</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>5_3</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>승</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>검정소_868192181(4골), 검정소_100214100(1골), Voor_858025420(1골), Voor_861000027(1골), Voor_845009676(1골)</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>2026-10-08 16:21:30</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>검정소</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Voor</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>2_3</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>패</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>검정소_868192181(2골), Voor_845009676(2골), Voor_852233700(1골)</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>2026-10-08 16:05:27</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>UNIT</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>검정소</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>3_4</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>패</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>UNIT_867166676(2골), UNIT_848180930(1골), 검정소_861214098(1골), 검정소_868192181(1골), 검정소_100214100(2골)</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>2026-10-08 15:53:08</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>UNIT</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>검정소</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>3_1</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>승</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>UNIT_867166676(1골), UNIT_848180930(2골), 검정소_868192181(1골)</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>2026-10-08 15:41:21</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>UNIT</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>검정소</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>2_2</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>패</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>UNIT_848180930(2골), 검정소_868192181(1골), 검정소_867241096(1골)</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>2026-10-08 14:34:46</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>호야국2인</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>UNIT</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>1_3</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>패</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>호야국2인_846192505(1골), UNIT_848180930(1골), UNIT_867166676(2골)</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>2026-10-08 14:19:20</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>UNIT</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>셀래스틴</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>3_3</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>무</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>UNIT_848180930(2골), UNIT_867166676(1골), 셀래스틴_861005680(2골), 셀래스틴_848231866(1골)</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>2026-10-08 14:05:46</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>호야국2인</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>셀래스틴</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>1_0</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>승</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>호야국2인_848232293(1골)</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>2026-10-08 13:50:45</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Gucci차붐</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>ZD장인지참치</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>3_3</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>무</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>Gucci차붐_840191208(3골), ZD장인지참치_861182521(1골), ZD장인지참치_840191208(1골), ZD장인지참치_839200104(1골)</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>2026-10-08 13:27:59</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Gucci차붐</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>셀래스틴</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>3_6</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>패</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>Gucci차붐_853227659(1골), Gucci차붐_864084333(1골), Gucci차붐_864176403(1골), 셀래스틴_861005680(2골), 셀래스틴_848194765(2골), 셀래스틴_852241461(1골), 셀래스틴_863233419(1골)</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>2026-10-08 13:15:09</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Gucci차붐</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>셀래스틴</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>4_5</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>패</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>Gucci차붐_864247686(1골), Gucci차붐_853272992(2골), Gucci차붐_853227659(1골), 셀래스틴_861005680(2골), 셀래스틴_845167680(1골), 셀래스틴_852241461(2골)</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>2026-10-08 12:47:28</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>개포동덕배</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Voor</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>5_1</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>승</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>개포동덕배_845190048(2골), 개포동덕배_856202126(1골), 개포동덕배_845208722(2골), Voor_861000027(1골)</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>2026-10-08 12:46:17</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>셀래스틴</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>용신</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>0_5</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>패</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>용신_877177003(1골), 용신_826251421(1골), 용신_866200104(3골)</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>2026-10-08 12:33:33</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>셀래스틴</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>용신</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>1_1</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>무</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>셀래스틴_861005680(1골), 용신_826251421(1골)</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>2026-10-08 12:27:12</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>개포동덕배</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>은안</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>6_1</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>승</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>개포동덕배_845208722(2골), 개포동덕배_845190048(3골), 개포동덕배_848206113(1골), 은안_856246420(1골)</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>2026-10-08 12:25:05</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>경남FC가즈아</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>syma</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>1_3</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>패</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>경남FC가즈아_225238224(1골), syma_867192629(1골), syma_845224574(1골), syma_866235522(1골)</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>2026-10-08 12:16:35</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>개포동덕배</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>은안</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>7_1</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>승</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>개포동덕배_856202126(4골), 개포동덕배_848206113(1골), 개포동덕배_845190048(2골), 은안_866241236(1골)</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>2026-10-08 12:13:50</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>경남FC가즈아</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>syma</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>1_1</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>무</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>경남FC가즈아_277205156(1골), syma_867192629(1골)</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>2026-10-08 12:11:09</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>앙쿠</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>ZD장인지참치</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>2_4</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>패</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>앙쿠_848176580(2골), ZD장인지참치_840191208(1골), ZD장인지참치_851240740(1골), ZD장인지참치_848199503(1골), ZD장인지참치_839200104(1골)</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>2026-10-08 11:59:25</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>앙쿠</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>ZD장인지참치</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>0_0</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>패</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr"/>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>2026-10-08 11:58:38</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>앙쿠</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>ZD장인지참치</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>2_4</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>패</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>앙쿠_848176580(1골), 앙쿠_845246191(1골), ZD장인지참치_839200104(4골)</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>2026-10-08 11:26:36</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>경남FC가즈아</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>셀래스틴</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>2_6</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>패</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>경남FC가즈아_225238224(1골), 경남FC가즈아_805267825(1골), 셀래스틴_861005680(5골), 셀래스틴_848230938(1골)</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>2026-10-08 11:13:33</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>경남FC가즈아</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>셀래스틴</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>3_3</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>무</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>경남FC가즈아_805267825(3골), 셀래스틴_863233419(1골), 셀래스틴_852241461(1골), 셀래스틴_848230938(1골)</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>2026-10-08 11:00:38</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>ZD장인지참치</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>용신</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>5_2</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>승</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>ZD장인지참치_839200104(4골), ZD장인지참치_840191208(1골), 용신_101173731(1골), 용신_863245367(1골)</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>2026-10-08 10:49:29</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>ZD장인지참치</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>용신</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>2_1</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>승</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>ZD장인지참치_840191208(1골), ZD장인지참치_840247263(1골), 용신_863245367(1골)</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>2026-10-07 14:25:42</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>UNIT</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>셀래스틴</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>1_0</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>승</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>UNIT_840192883(1골)</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>2026-10-07 14:14:55</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>앙쿠</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>UNIT</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>1_4</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>패</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>앙쿠_861049369(1골), UNIT_863250723(1골), UNIT_848180930(1골), UNIT_840228251(1골), UNIT_867166676(1골)</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>2026-10-07 14:03:01</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>앙쿠</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>셀래스틴</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>3_2</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>승</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>앙쿠_861049369(1골), 앙쿠_848176580(1골), 앙쿠_863232488(1골), 셀래스틴_863233419(1골), 셀래스틴_848231866(1골)</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>2026-10-07 13:51:44</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>앙쿠</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>셀래스틴</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>6_2</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>승</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>앙쿠_861049369(3골), 앙쿠_851194765(2골), 앙쿠_848176580(1골), 셀래스틴_848194765(1골), 셀래스틴_861005680(1골)</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>2026-10-07 13:39:26</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>UNIT</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>셀래스틴</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>4_2</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>승</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>UNIT_867166676(3골), UNIT_848180930(1골), 셀래스틴_863233419(1골), 셀래스틴_861005680(1골)</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>2026-10-07 13:28:13</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>앙쿠</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>UNIT</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>2_1</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>승</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>앙쿠_866266039(1골), 앙쿠_861049369(1골), UNIT_863250723(1골)</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>2026-10-07 13:16:19</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>앙쿠</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>셀래스틴</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>2_3</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>패</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>앙쿠_861049369(1골), 앙쿠_848176580(1골), 셀래스틴_861005680(2골), 셀래스틴_848231866(1골)</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>2026-10-07 13:05:29</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>UNIT</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>셀래스틴</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>1_3</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>패</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>UNIT_867166676(1골), 셀래스틴_861005680(2골), 셀래스틴_852241461(1골)</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>2026-10-07 12:50:50</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>앙쿠</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>UNIT</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>2_5</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>패</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>앙쿠_861049369(1골), 앙쿠_851194765(1골), UNIT_867166676(2골), UNIT_848180930(3골)</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>2026-10-07 12:30:57</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>UNIT</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>ZD장인지참치</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>2_1</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>승</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>UNIT_867166676(2골), ZD장인지참치_840191208(1골)</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>2026-10-07 12:14:34</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>앙쿠</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>셀래스틴</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>3_0</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>승</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>앙쿠_848176580(1골), 앙쿠_866266039(1골), 앙쿠_861049369(1골)</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>2026-10-07 12:04:29</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>앙쿠</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>셀래스틴</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>3_1</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>승</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>앙쿠_861049369(2골), 앙쿠_866266039(1골), 셀래스틴_852241461(1골)</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>2026-10-07 11:33:41</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>겐지간지</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>용신</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>0_3</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>패</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>용신_825212188(3골)</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
           <t>2026-10-07 11:21:15</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr">
+      <c r="B56" t="inlineStr">
         <is>
           <t>겐지간지</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr">
+      <c r="C56" t="inlineStr">
         <is>
           <t>용신</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr">
+      <c r="D56" t="inlineStr">
         <is>
           <t>1_4</t>
         </is>
       </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>패</t>
-        </is>
-      </c>
-      <c r="F12" t="inlineStr">
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>패</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
         <is>
           <t>겐지간지_845158023(1골), 용신_866200104(1골), 용신_825212188(3골)</t>
         </is>
@@ -812,7 +2212,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F12"/>
+  <dimension ref="A1:F56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -850,54 +2250,54 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-10-07 13:51:44</t>
+          <t>2026-10-09 13:36:17</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>앙쿠</t>
+          <t>검정소</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>셀래스틴</t>
+          <t>콩콩콩룔</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>6_2</t>
+          <t>3_3</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>승</t>
+          <t>무</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>앙쿠_848176580(1도움), 앙쿠_861049369(1도움), 앙쿠_851194765(3도움), 셀래스틴_852241461(1도움)</t>
+          <t>검정소_100214100(1도움), 검정소_861005003(2도움), 콩콩콩룔_848189505(1도움), 콩콩콩룔_867220502(2도움)</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-10-07 13:39:26</t>
+          <t>2026-10-09 13:33:58</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>UNIT</t>
+          <t>셀래스틴</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>셀래스틴</t>
+          <t>syma</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>4_2</t>
+          <t>2_0</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -907,29 +2307,29 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>UNIT_840192883(2도움), UNIT_840210736(1도움), UNIT_840228251(1도움)</t>
+          <t>셀래스틴_861005680(1도움), 셀래스틴_848231866(1도움)</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-10-07 13:28:13</t>
+          <t>2026-10-09 13:25:18</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>앙쿠</t>
+          <t>검정소</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>UNIT</t>
+          <t>콩콩콩룔</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>2_1</t>
+          <t>10_4</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -939,51 +2339,51 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>앙쿠_846193747(1도움)</t>
+          <t>검정소_861005003(3도움), 검정소_868192181(2도움), 검정소_861214098(2도움), 검정소_851241721(1도움), 검정소_100214100(1도움), 콩콩콩룔_861006235(1도움), 콩콩콩룔_867220502(1도움), 콩콩콩룔_867223848(1도움)</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-10-07 13:16:19</t>
+          <t>2026-10-09 13:23:55</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>앙쿠</t>
+          <t>셀래스틴</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>셀래스틴</t>
+          <t>syma</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>2_3</t>
+          <t>3_2</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>패</t>
+          <t>승</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>앙쿠_861049369(1도움), 앙쿠_851194765(1도움), 셀래스틴_852241461(2도움), 셀래스틴_863233419(1도움)</t>
+          <t>셀래스틴_848194765(1도움), 셀래스틴_852241461(1도움), 셀래스틴_848230938(1도움), syma_863251854(1도움), syma_866264388(1도움)</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-10-07 13:05:29</t>
+          <t>2026-10-09 05:08:26</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>UNIT</t>
+          <t>ZD장인지참치</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -993,39 +2393,39 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>1_3</t>
+          <t>5_1</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>패</t>
+          <t>승</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>UNIT_840210736(1도움), 셀래스틴_852259694(1도움), 셀래스틴_848230938(1도움)</t>
+          <t>ZD장인지참치_840256630(1도움), ZD장인지참치_848199503(1도움), ZD장인지참치_839200104(1도움), ZD장인지참치_851240740(2도움), 셀래스틴_852241461(1도움)</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-10-07 12:50:50</t>
+          <t>2026-10-09 04:53:33</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>앙쿠</t>
+          <t>ZD장인지참치</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>UNIT</t>
+          <t>셀래스틴</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>2_5</t>
+          <t>3_6</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -1035,29 +2435,29 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>앙쿠_848176580(1도움), UNIT_863250723(1도움), UNIT_840228251(1도움), UNIT_840210736(2도움), UNIT_840192883(1도움)</t>
+          <t>ZD장인지참치_861182521(1도움), ZD장인지참치_840191208(1도움), ZD장인지참치_851240740(1도움), 셀래스틴_861005680(2도움), 셀래스틴_848231866(1도움), 셀래스틴_848194765(2도움), 셀래스틴_863200458(1도움)</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-10-07 12:30:57</t>
+          <t>2026-10-09 04:42:24</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>UNIT</t>
+          <t>ZD장인지참치</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>ZD장인지참치</t>
+          <t>셀래스틴</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>2_1</t>
+          <t>4_2</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -1067,19 +2467,19 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>UNIT_840210736(1도움), ZD장인지참치_840256630(1도움)</t>
+          <t>ZD장인지참치_839200104(1도움), ZD장인지참치_848199503(1도움), ZD장인지참치_851240740(1도움), 셀래스틴_848013038(1도움), 셀래스틴_852259694(1도움)</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-10-07 12:14:34</t>
+          <t>2026-10-09 04:31:15</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>앙쿠</t>
+          <t>ZD장인지참치</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -1089,29 +2489,29 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>3_0</t>
+          <t>3_4</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>승</t>
+          <t>패</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>앙쿠_851194765(2도움), 앙쿠_846186345(1도움)</t>
+          <t>ZD장인지참치_848199503(1도움), ZD장인지참치_840191208(2도움), 셀래스틴_852241461(1도움), 셀래스틴_863233419(1도움), 셀래스틴_861005680(1도움), 셀래스틴_863200458(1도움)</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-10-07 12:04:29</t>
+          <t>2026-10-09 04:19:11</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>앙쿠</t>
+          <t>ZD장인지참치</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -1121,7 +2521,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>3_1</t>
+          <t>2_1</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -1131,29 +2531,29 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>앙쿠_851194765(1도움), 앙쿠_846186345(1도움), 앙쿠_848176580(1도움), 셀래스틴_863200458(1도움)</t>
+          <t>ZD장인지참치_840191208(1도움), ZD장인지참치_861182521(1도움), 셀래스틴_848231866(1도움)</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-10-07 11:33:41</t>
+          <t>2026-10-09 04:04:37</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>겐지간지</t>
+          <t>UNIT</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>용신</t>
+          <t>셀래스틴</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>0_3</t>
+          <t>0_0</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -1161,39 +2561,1439 @@
           <t>패</t>
         </is>
       </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>용신_101173731(1도움), 용신_866200104(1도움)</t>
-        </is>
-      </c>
+      <c r="F11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
+          <t>2026-10-09 03:48:59</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>UNIT</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>셀래스틴</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>1_0</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>승</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>UNIT_840192883(1도움)</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2026-10-09 02:36:22</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>syma</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>용신</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>1_2</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>패</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>syma_845224574(1도움), 용신_826251421(2도움)</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-10-09 02:26:03</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>syma</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>용신</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>2_3</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>패</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>syma_867192629(1도움), syma_851224415(1도움), 용신_877177003(1도움), 용신_101173731(1도움), 용신_826251421(1도움)</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>2026-10-08 17:16:26</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>UNIT</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Voor</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>5_4</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>승</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>UNIT_840225782(1도움), UNIT_848265695(1도움), UNIT_863250723(1도움), UNIT_840228251(1도움), Voor_856256079(1도움), Voor_861045674(1도움), Voor_852233700(1도움), Voor_845009676(1도움)</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-10-08 17:00:32</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>UNIT</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Voor</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>2_1</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>승</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>UNIT_863250723(1도움), UNIT_840228251(1도움), Voor_852233700(1도움)</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2026-10-08 16:48:25</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>UNIT</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Voor</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>0_2</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>패</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>Voor_852233700(1도움)</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>2026-10-08 16:33:10</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>검정소</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Voor</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>5_3</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>승</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>검정소_861005003(2도움), 검정소_851241721(1도움), 검정소_100214100(1도움), Voor_852233700(2도움)</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>2026-10-08 16:21:30</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>검정소</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Voor</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>2_3</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>패</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>검정소_861005003(2도움), Voor_861000027(1도움), Voor_845247090(1도움), Voor_852233700(1도움)</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>2026-10-08 16:05:27</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>UNIT</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>검정소</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>3_4</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>패</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>UNIT_840192883(3도움), 검정소_867241096(1도움), 검정소_851247229(1도움), 검정소_861005003(1도움)</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>2026-10-08 15:53:08</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>UNIT</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>검정소</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>3_1</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>승</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>UNIT_848265695(1도움), UNIT_867166676(1도움), 검정소_861214098(1도움)</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>2026-10-08 15:41:21</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>UNIT</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>검정소</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>2_2</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>패</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>UNIT_840192883(1도움), UNIT_840228251(1도움), 검정소_861214098(1도움)</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>2026-10-08 14:34:46</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>호야국2인</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>UNIT</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>1_3</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>패</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>호야국2인_848216435(1도움), UNIT_840225782(1도움), UNIT_840210736(1도움), UNIT_840192883(1도움)</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>2026-10-08 14:19:20</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>UNIT</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>셀래스틴</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>3_3</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>무</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>UNIT_840228251(1도움), UNIT_840210736(1도움), UNIT_840192883(1도움), 셀래스틴_852259694(1도움), 셀래스틴_852241461(1도움), 셀래스틴_863200458(1도움)</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>2026-10-08 14:05:46</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>호야국2인</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>셀래스틴</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>1_0</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>승</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>호야국2인_848216435(1도움)</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>2026-10-08 13:50:45</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Gucci차붐</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>ZD장인지참치</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>3_3</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>무</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>Gucci차붐_867208128(2도움), Gucci차붐_877256630(1도움), ZD장인지참치_840191208(1도움), ZD장인지참치_851240740(1도움), ZD장인지참치_839200104(1도움)</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>2026-10-08 13:27:59</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Gucci차붐</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>셀래스틴</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>3_6</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>패</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>Gucci차붐_853227659(1도움), Gucci차붐_864247686(1도움), 셀래스틴_848230938(2도움), 셀래스틴_861005680(1도움), 셀래스틴_852241461(1도움), 셀래스틴_863233419(2도움)</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>2026-10-08 13:15:09</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Gucci차붐</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>셀래스틴</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>4_5</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>패</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>Gucci차붐_864176403(1도움), Gucci차붐_851221671(2도움), 셀래스틴_863200458(1도움), 셀래스틴_852259694(1도움), 셀래스틴_848194765(2도움), 셀래스틴_852241461(1도움)</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>2026-10-08 12:47:28</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>개포동덕배</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Voor</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>5_1</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>승</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>개포동덕배_848206113(1도움), 개포동덕배_856202126(1도움), 개포동덕배_856212622(1도움), 개포동덕배_852225375(1도움), 개포동덕배_863234396(1도움)</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>2026-10-08 12:46:17</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>셀래스틴</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>용신</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>0_5</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>패</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>용신_877177003(1도움), 용신_101173731(2도움), 용신_863245367(1도움), 용신_856243576(1도움)</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>2026-10-08 12:33:33</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>셀래스틴</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>용신</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>1_1</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>무</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>셀래스틴_863233419(1도움), 용신_101173731(1도움)</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>2026-10-08 12:27:12</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>개포동덕배</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>은안</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>6_1</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>승</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>개포동덕배_845208722(2도움), 개포동덕배_856202126(4도움), 은안_866241236(1도움)</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>2026-10-08 12:25:05</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>경남FC가즈아</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>syma</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>1_3</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>패</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>경남FC가즈아_518251161(1도움), syma_861001668(1도움), syma_867192629(1도움)</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>2026-10-08 12:16:35</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>개포동덕배</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>은안</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>7_1</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>승</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>개포동덕배_845208722(3도움), 개포동덕배_856202126(1도움), 개포동덕배_845190048(1도움), 개포동덕배_856275298(2도움), 은안_877143001(1도움)</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>2026-10-08 12:13:50</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>경남FC가즈아</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>syma</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>1_1</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>무</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>경남FC가즈아_805267825(1도움), syma_861001668(1도움)</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>2026-10-08 12:11:09</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>앙쿠</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>ZD장인지참치</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>2_4</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>패</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>앙쿠_851194765(1도움), 앙쿠_845246191(1도움), ZD장인지참치_852213331(1도움), ZD장인지참치_840256630(1도움), ZD장인지참치_848199503(1도움), ZD장인지참치_839200104(1도움)</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>2026-10-08 11:59:25</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>앙쿠</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>ZD장인지참치</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>0_0</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>패</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr"/>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>2026-10-08 11:58:38</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>앙쿠</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>ZD장인지참치</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>2_4</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>패</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>앙쿠_848176580(1도움), 앙쿠_851194765(1도움), ZD장인지참치_840191208(2도움), ZD장인지참치_861182521(1도움), ZD장인지참치_848199503(1도움)</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>2026-10-08 11:26:36</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>경남FC가즈아</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>셀래스틴</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>2_6</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>패</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>경남FC가즈아_805207730(1도움), 경남FC가즈아_853221467(1도움), 셀래스틴_863200458(1도움), 셀래스틴_852241461(3도움), 셀래스틴_852259694(1도움), 셀래스틴_848194765(1도움)</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>2026-10-08 11:13:33</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>경남FC가즈아</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>셀래스틴</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>3_3</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>무</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>경남FC가즈아_225238224(1도움), 경남FC가즈아_853221467(2도움), 셀래스틴_861005680(1도움), 셀래스틴_848230938(1도움), 셀래스틴_848194765(1도움)</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>2026-10-08 11:00:38</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>ZD장인지참치</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>용신</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>5_2</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>승</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>ZD장인지참치_861182521(2도움), ZD장인지참치_839200104(1도움), ZD장인지참치_840256630(1도움), ZD장인지참치_840191208(1도움), 용신_101173731(1도움)</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>2026-10-08 10:49:29</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>ZD장인지참치</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>용신</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>2_1</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>승</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>ZD장인지참치_861182521(1도움), 용신_101173731(1도움)</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>2026-10-07 14:25:42</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>UNIT</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>셀래스틴</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>1_0</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>승</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>UNIT_840228251(1도움)</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>2026-10-07 14:14:55</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>앙쿠</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>UNIT</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>1_4</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>패</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>앙쿠_848176580(1도움), UNIT_840228251(1도움), UNIT_867166676(1도움)</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>2026-10-07 14:03:01</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>앙쿠</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>셀래스틴</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>3_2</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>승</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>앙쿠_851194765(2도움), 앙쿠_846186345(1도움), 셀래스틴_852241461(1도움)</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>2026-10-07 13:51:44</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>앙쿠</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>셀래스틴</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>6_2</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>승</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>앙쿠_861049369(1도움), 앙쿠_851194765(3도움), 앙쿠_848176580(1도움), 셀래스틴_852241461(1도움)</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>2026-10-07 13:39:26</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>UNIT</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>셀래스틴</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>4_2</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>승</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>UNIT_840192883(2도움), UNIT_840228251(1도움), UNIT_840210736(1도움)</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>2026-10-07 13:28:13</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>앙쿠</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>UNIT</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>2_1</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>승</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>앙쿠_846193747(1도움)</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>2026-10-07 13:16:19</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>앙쿠</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>셀래스틴</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>2_3</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>패</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>앙쿠_851194765(1도움), 앙쿠_861049369(1도움), 셀래스틴_852241461(2도움), 셀래스틴_863233419(1도움)</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>2026-10-07 13:05:29</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>UNIT</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>셀래스틴</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>1_3</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>패</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>UNIT_840210736(1도움), 셀래스틴_852259694(1도움), 셀래스틴_848230938(1도움)</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>2026-10-07 12:50:50</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>앙쿠</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>UNIT</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>2_5</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>패</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>앙쿠_848176580(1도움), UNIT_840210736(2도움), UNIT_840192883(1도움), UNIT_863250723(1도움), UNIT_840228251(1도움)</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>2026-10-07 12:30:57</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>UNIT</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>ZD장인지참치</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>2_1</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>승</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>UNIT_840210736(1도움), ZD장인지참치_840256630(1도움)</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>2026-10-07 12:14:34</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>앙쿠</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>셀래스틴</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>3_0</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>승</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>앙쿠_846186345(1도움), 앙쿠_851194765(2도움)</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>2026-10-07 12:04:29</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>앙쿠</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>셀래스틴</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>3_1</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>승</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>앙쿠_846186345(1도움), 앙쿠_851194765(1도움), 앙쿠_848176580(1도움), 셀래스틴_863200458(1도움)</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>2026-10-07 11:33:41</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>겐지간지</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>용신</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>0_3</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>패</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>용신_101173731(1도움), 용신_866200104(1도움)</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
           <t>2026-10-07 11:21:15</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr">
+      <c r="B56" t="inlineStr">
         <is>
           <t>겐지간지</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr">
+      <c r="C56" t="inlineStr">
         <is>
           <t>용신</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr">
+      <c r="D56" t="inlineStr">
         <is>
           <t>1_4</t>
         </is>
       </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>패</t>
-        </is>
-      </c>
-      <c r="F12" t="inlineStr">
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>패</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
         <is>
           <t>겐지간지_852231443(1도움), 용신_866200104(1도움), 용신_291213648(2도움)</t>
         </is>

</xml_diff>

<commit_message>
Update: Dashboard HTML (10:08:25)
</commit_message>
<xml_diff>
--- a/API데이터_경기_득점_및_도움_기록.xlsx
+++ b/API데이터_경기_득점_및_도움_기록.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F114"/>
+  <dimension ref="A1:F128"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2960,7 +2960,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>2026-10-11 07:47:05</t>
+          <t>2026-10-11 07:59:52</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
@@ -2975,7 +2975,7 @@
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>2_5</t>
+          <t>2_3</t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
@@ -2985,14 +2985,14 @@
       </c>
       <c r="F81" t="inlineStr">
         <is>
-          <t>A지냐크_877031432(1골), A지냐크_861167134(1골), 셀래스틴_863233419(1골), 셀래스틴_861005680(2골), 셀래스틴_852241461(2골)</t>
+          <t>A지냐크_861167134(2골), 셀래스틴_861005680(1골), 셀래스틴_863233419(2골)</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>2026-10-11 07:59:52</t>
+          <t>2026-10-11 08:33:57</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
@@ -3002,29 +3002,29 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>셀래스틴</t>
+          <t>ShangHaiPortFC</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>2_3</t>
+          <t>7_2</t>
         </is>
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>패</t>
+          <t>승</t>
         </is>
       </c>
       <c r="F82" t="inlineStr">
         <is>
-          <t>A지냐크_861167134(2골), 셀래스틴_861005680(1골), 셀래스틴_863233419(2골)</t>
+          <t>A지냐크_834271400(3골), A지냐크_877031432(3골), A지냐크_863241496(1골), ShangHaiPortFC_848031432(2골)</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>2026-10-11 08:33:57</t>
+          <t>2026-10-11 08:45:05</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
@@ -3039,39 +3039,39 @@
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>7_2</t>
+          <t>1_5</t>
         </is>
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>승</t>
+          <t>패</t>
         </is>
       </c>
       <c r="F83" t="inlineStr">
         <is>
-          <t>A지냐크_834271400(3골), A지냐크_877031432(3골), A지냐크_863241496(1골), ShangHaiPortFC_848031432(2골)</t>
+          <t>A지냐크_863241496(1골), ShangHaiPortFC_848031432(3골), ShangHaiPortFC_864191910(2골)</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>2026-10-11 08:45:05</t>
+          <t>2026-10-11 10:08:39</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>A지냐크</t>
+          <t>ShangHaiPortFC</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>ShangHaiPortFC</t>
+          <t>용신</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>1_5</t>
+          <t>2_6</t>
         </is>
       </c>
       <c r="E84" t="inlineStr">
@@ -3081,14 +3081,14 @@
       </c>
       <c r="F84" t="inlineStr">
         <is>
-          <t>A지냐크_863241496(1골), ShangHaiPortFC_848031432(3골), ShangHaiPortFC_864191910(2골)</t>
+          <t>ShangHaiPortFC_848031432(2골), 용신_863245367(1골), 용신_866200104(1골), 용신_826251421(2골), 용신_101173731(2골)</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>2026-10-11 10:08:39</t>
+          <t>2026-10-11 10:48:32</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
@@ -3103,56 +3103,56 @@
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>2_6</t>
+          <t>3_2</t>
         </is>
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>패</t>
+          <t>승</t>
         </is>
       </c>
       <c r="F85" t="inlineStr">
         <is>
-          <t>ShangHaiPortFC_848031432(2골), 용신_863245367(1골), 용신_866200104(1골), 용신_826251421(2골), 용신_101173731(2골)</t>
+          <t>ShangHaiPortFC_861051412(1골), ShangHaiPortFC_845231138(1골), ShangHaiPortFC_256164959(1골), 용신_866200104(2골)</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>2026-10-11 10:48:32</t>
+          <t>2026-10-11 11:11:43</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>ShangHaiPortFC</t>
+          <t>여수가스</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>용신</t>
+          <t>셀래스틴</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>3_2</t>
+          <t>4_6</t>
         </is>
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>승</t>
+          <t>패</t>
         </is>
       </c>
       <c r="F86" t="inlineStr">
         <is>
-          <t>ShangHaiPortFC_861051412(1골), ShangHaiPortFC_845231138(1골), ShangHaiPortFC_256164959(1골), 용신_866200104(2골)</t>
+          <t>여수가스_846001551(1골), 여수가스_861215732(3골), 셀래스틴_852241461(3골), 셀래스틴_863233419(1골), 셀래스틴_861005680(2골)</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>2026-10-11 11:11:43</t>
+          <t>2026-10-11 11:23:07</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
@@ -3167,29 +3167,29 @@
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>4_6</t>
+          <t>2_1</t>
         </is>
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>패</t>
+          <t>승</t>
         </is>
       </c>
       <c r="F87" t="inlineStr">
         <is>
-          <t>여수가스_846001551(1골), 여수가스_861215732(3골), 셀래스틴_852241461(3골), 셀래스틴_863233419(1골), 셀래스틴_861005680(2골)</t>
+          <t>여수가스_861215732(1골), 여수가스_846001551(1골), 셀래스틴_863233419(1골)</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>2026-10-11 11:23:07</t>
+          <t>2026-10-11 12:05:40</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>여수가스</t>
+          <t>앙쿠</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
@@ -3199,24 +3199,24 @@
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>2_1</t>
+          <t>1_2</t>
         </is>
       </c>
       <c r="E88" t="inlineStr">
         <is>
-          <t>승</t>
+          <t>패</t>
         </is>
       </c>
       <c r="F88" t="inlineStr">
         <is>
-          <t>여수가스_861215732(1골), 여수가스_846001551(1골), 셀래스틴_863233419(1골)</t>
+          <t>앙쿠_848176580(1골), 셀래스틴_861005680(1골), 셀래스틴_852241461(1골)</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>2026-10-11 12:05:40</t>
+          <t>2026-10-11 12:16:11</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
@@ -3231,7 +3231,7 @@
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>1_2</t>
+          <t>0_2</t>
         </is>
       </c>
       <c r="E89" t="inlineStr">
@@ -3241,14 +3241,14 @@
       </c>
       <c r="F89" t="inlineStr">
         <is>
-          <t>앙쿠_848176580(1골), 셀래스틴_861005680(1골), 셀래스틴_852241461(1골)</t>
+          <t>셀래스틴_852241461(1골), 셀래스틴_863233419(1골)</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>2026-10-11 12:16:11</t>
+          <t>2026-10-11 12:25:49</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
@@ -3263,56 +3263,56 @@
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>0_2</t>
+          <t>1_1</t>
         </is>
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t>패</t>
+          <t>무</t>
         </is>
       </c>
       <c r="F90" t="inlineStr">
         <is>
-          <t>셀래스틴_852241461(1골), 셀래스틴_863233419(1골)</t>
+          <t>앙쿠_861049369(1골), 셀래스틴_852241461(1골)</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>2026-10-11 12:25:49</t>
+          <t>2026-10-11 17:54:01</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>앙쿠</t>
+          <t>UNIT</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>셀래스틴</t>
+          <t>Voor</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>1_1</t>
+          <t>0_4</t>
         </is>
       </c>
       <c r="E91" t="inlineStr">
         <is>
-          <t>무</t>
+          <t>패</t>
         </is>
       </c>
       <c r="F91" t="inlineStr">
         <is>
-          <t>앙쿠_861049369(1골), 셀래스틴_852241461(1골)</t>
+          <t>Voor_852233700(1골), Voor_845247090(1골), Voor_868007512(2골)</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>2026-10-11 17:43:20</t>
+          <t>2026-10-11 18:05:57</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
@@ -3327,24 +3327,24 @@
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>4_4</t>
+          <t>4_2</t>
         </is>
       </c>
       <c r="E92" t="inlineStr">
         <is>
-          <t>패</t>
+          <t>승</t>
         </is>
       </c>
       <c r="F92" t="inlineStr">
         <is>
-          <t>UNIT_848180930(2골), UNIT_867166676(2골), Voor_868007512(3골), Voor_845247090(1골)</t>
+          <t>UNIT_867166676(2골), UNIT_848180930(2골), Voor_868007512(1골), Voor_861000027(1골)</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>2026-10-11 17:54:01</t>
+          <t>2026-10-11 18:23:54</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
@@ -3359,7 +3359,7 @@
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>0_4</t>
+          <t>3_3</t>
         </is>
       </c>
       <c r="E93" t="inlineStr">
@@ -3369,14 +3369,14 @@
       </c>
       <c r="F93" t="inlineStr">
         <is>
-          <t>Voor_852233700(1골), Voor_845247090(1골), Voor_868007512(2골)</t>
+          <t>UNIT_867166676(1골), UNIT_848180930(1골), UNIT_851236403(1골), Voor_852233700(1골), Voor_861000027(1골), Voor_868007512(1골)</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>2026-10-11 18:05:57</t>
+          <t>2026-10-11 18:36:25</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
@@ -3391,24 +3391,24 @@
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>4_2</t>
+          <t>3_4</t>
         </is>
       </c>
       <c r="E94" t="inlineStr">
         <is>
-          <t>승</t>
+          <t>패</t>
         </is>
       </c>
       <c r="F94" t="inlineStr">
         <is>
-          <t>UNIT_867166676(2골), UNIT_848180930(2골), Voor_868007512(1골), Voor_861000027(1골)</t>
+          <t>UNIT_867166676(1골), UNIT_848180930(2골), Voor_868007512(2골), Voor_835183277(2골)</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>2026-10-11 18:23:54</t>
+          <t>2026-10-11 18:53:58</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
@@ -3433,14 +3433,14 @@
       </c>
       <c r="F95" t="inlineStr">
         <is>
-          <t>UNIT_867166676(1골), UNIT_848180930(1골), UNIT_851236403(1골), Voor_852233700(1골), Voor_861000027(1골), Voor_868007512(1골)</t>
+          <t>UNIT_848180930(2골), UNIT_840192883(1골), Voor_861045674(1골), Voor_868007512(1골), Voor_852233700(1골)</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>2026-10-11 18:36:25</t>
+          <t>2026-10-12 10:04:39</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
@@ -3450,76 +3450,76 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>Voor</t>
+          <t>셀래스틴</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>3_4</t>
+          <t>2_1</t>
         </is>
       </c>
       <c r="E96" t="inlineStr">
         <is>
-          <t>패</t>
+          <t>승</t>
         </is>
       </c>
       <c r="F96" t="inlineStr">
         <is>
-          <t>UNIT_867166676(1골), UNIT_848180930(2골), Voor_868007512(2골), Voor_835183277(2골)</t>
+          <t>UNIT_840228251(1골), UNIT_839013383(1골), 셀래스틴_848231866(1골)</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>2026-10-11 18:53:58</t>
+          <t>2026-10-12 12:06:47</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>UNIT</t>
+          <t>0708ManUtd</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>Voor</t>
+          <t>콩콩콩룔</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>3_3</t>
+          <t>3_0</t>
         </is>
       </c>
       <c r="E97" t="inlineStr">
         <is>
-          <t>패</t>
+          <t>승</t>
         </is>
       </c>
       <c r="F97" t="inlineStr">
         <is>
-          <t>UNIT_848180930(2골), UNIT_840192883(1골), Voor_861045674(1골), Voor_868007512(1골), Voor_852233700(1골)</t>
+          <t>0708ManUtd_868037576(2골), 0708ManUtd_868001397(1골)</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>2026-10-12 10:04:39</t>
+          <t>2026-10-12 12:12:43</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>UNIT</t>
+          <t>A지냐크</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>셀래스틴</t>
+          <t>Gucci와퍼</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>2_1</t>
+          <t>4_1</t>
         </is>
       </c>
       <c r="E98" t="inlineStr">
@@ -3529,14 +3529,14 @@
       </c>
       <c r="F98" t="inlineStr">
         <is>
-          <t>UNIT_840228251(1골), UNIT_839013383(1골), 셀래스틴_848231866(1골)</t>
+          <t>A지냐크_877031432(4골), Gucci와퍼_864200104(1골)</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>2026-10-12 12:06:47</t>
+          <t>2026-10-12 12:17:19</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
@@ -3561,14 +3561,14 @@
       </c>
       <c r="F99" t="inlineStr">
         <is>
-          <t>0708ManUtd_868037576(2골), 0708ManUtd_868001397(1골)</t>
+          <t>0708ManUtd_868037576(1골), 0708ManUtd_834239053(2골)</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>2026-10-12 12:12:43</t>
+          <t>2026-10-12 12:30:45</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
@@ -3583,24 +3583,24 @@
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>4_1</t>
+          <t>4_5</t>
         </is>
       </c>
       <c r="E100" t="inlineStr">
         <is>
-          <t>승</t>
+          <t>패</t>
         </is>
       </c>
       <c r="F100" t="inlineStr">
         <is>
-          <t>A지냐크_877031432(4골), Gucci와퍼_864200104(1골)</t>
+          <t>A지냐크_877031432(4골), Gucci와퍼_852010264(2골), Gucci와퍼_851210697(2골), Gucci와퍼_864200104(1골)</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>2026-10-12 12:17:19</t>
+          <t>2026-10-12 12:39:42</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
@@ -3610,12 +3610,12 @@
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>콩콩콩룔</t>
+          <t>용신</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>3_0</t>
+          <t>3_1</t>
         </is>
       </c>
       <c r="E101" t="inlineStr">
@@ -3625,14 +3625,14 @@
       </c>
       <c r="F101" t="inlineStr">
         <is>
-          <t>0708ManUtd_868037576(1골), 0708ManUtd_834239053(2골)</t>
+          <t>0708ManUtd_868037576(2골), 0708ManUtd_868001397(1골), 용신_866200104(1골)</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>2026-10-12 12:30:45</t>
+          <t>2026-10-12 12:45:19</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
@@ -3647,7 +3647,7 @@
       </c>
       <c r="D102" t="inlineStr">
         <is>
-          <t>4_5</t>
+          <t>3_4</t>
         </is>
       </c>
       <c r="E102" t="inlineStr">
@@ -3657,14 +3657,14 @@
       </c>
       <c r="F102" t="inlineStr">
         <is>
-          <t>A지냐크_877031432(4골), Gucci와퍼_852010264(2골), Gucci와퍼_851210697(2골), Gucci와퍼_864200104(1골)</t>
+          <t>A지냐크_861167134(2골), A지냐크_877031432(1골), Gucci와퍼_852168473(1골), Gucci와퍼_864200104(3골)</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>2026-10-12 12:39:42</t>
+          <t>2026-10-12 12:50:47</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
@@ -3679,39 +3679,39 @@
       </c>
       <c r="D103" t="inlineStr">
         <is>
-          <t>3_1</t>
+          <t>3_3</t>
         </is>
       </c>
       <c r="E103" t="inlineStr">
         <is>
-          <t>승</t>
+          <t>무</t>
         </is>
       </c>
       <c r="F103" t="inlineStr">
         <is>
-          <t>0708ManUtd_868037576(2골), 0708ManUtd_868001397(1골), 용신_866200104(1골)</t>
+          <t>0708ManUtd_835183277(1골), 0708ManUtd_868001397(1골), 0708ManUtd_868037576(1골), 용신_101173731(1골), 용신_866200104(2골)</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>2026-10-12 12:45:19</t>
+          <t>2026-10-12 13:04:34</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>A지냐크</t>
+          <t>0708ManUtd</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>Gucci와퍼</t>
+          <t>UNIT</t>
         </is>
       </c>
       <c r="D104" t="inlineStr">
         <is>
-          <t>3_4</t>
+          <t>2_4</t>
         </is>
       </c>
       <c r="E104" t="inlineStr">
@@ -3721,14 +3721,14 @@
       </c>
       <c r="F104" t="inlineStr">
         <is>
-          <t>A지냐크_861167134(2골), A지냐크_877031432(1골), Gucci와퍼_852168473(1골), Gucci와퍼_864200104(3골)</t>
+          <t>0708ManUtd_851226161(1골), 0708ManUtd_868001397(1골), UNIT_867166676(2골), UNIT_848180930(2골)</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>2026-10-12 12:50:47</t>
+          <t>2026-10-12 13:17:50</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
@@ -3738,29 +3738,29 @@
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>용신</t>
+          <t>A지냐크</t>
         </is>
       </c>
       <c r="D105" t="inlineStr">
         <is>
-          <t>3_3</t>
+          <t>7_0</t>
         </is>
       </c>
       <c r="E105" t="inlineStr">
         <is>
-          <t>무</t>
+          <t>승</t>
         </is>
       </c>
       <c r="F105" t="inlineStr">
         <is>
-          <t>0708ManUtd_835183277(1골), 0708ManUtd_868001397(1골), 0708ManUtd_868037576(1골), 용신_101173731(1골), 용신_866200104(2골)</t>
+          <t>0708ManUtd_835183277(1골), 0708ManUtd_861005661(2골), 0708ManUtd_868001397(2골), 0708ManUtd_851226161(1골), 0708ManUtd_868037576(1골)</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>2026-10-12 13:04:34</t>
+          <t>2026-10-12 13:29:18</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
@@ -3770,29 +3770,29 @@
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>UNIT</t>
+          <t>A지냐크</t>
         </is>
       </c>
       <c r="D106" t="inlineStr">
         <is>
-          <t>2_4</t>
+          <t>5_3</t>
         </is>
       </c>
       <c r="E106" t="inlineStr">
         <is>
-          <t>패</t>
+          <t>승</t>
         </is>
       </c>
       <c r="F106" t="inlineStr">
         <is>
-          <t>0708ManUtd_851226161(1골), 0708ManUtd_868001397(1골), UNIT_867166676(2골), UNIT_848180930(2골)</t>
+          <t>0708ManUtd_868001397(2골), 0708ManUtd_834239053(1골), 0708ManUtd_851226161(1골), 0708ManUtd_868037576(1골), A지냐크_861167134(2골), A지냐크_877031432(1골)</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>2026-10-12 13:17:50</t>
+          <t>2026-10-12 13:44:20</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
@@ -3802,12 +3802,12 @@
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>A지냐크</t>
+          <t>셀래스틴</t>
         </is>
       </c>
       <c r="D107" t="inlineStr">
         <is>
-          <t>7_0</t>
+          <t>2_1</t>
         </is>
       </c>
       <c r="E107" t="inlineStr">
@@ -3817,51 +3817,51 @@
       </c>
       <c r="F107" t="inlineStr">
         <is>
-          <t>0708ManUtd_835183277(1골), 0708ManUtd_861005661(2골), 0708ManUtd_868001397(2골), 0708ManUtd_851226161(1골), 0708ManUtd_868037576(1골)</t>
+          <t>0708ManUtd_868001397(2골), 셀래스틴_861005680(1골)</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>2026-10-12 13:29:18</t>
+          <t>2026-10-13 10:11:17</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>0708ManUtd</t>
+          <t>UNIT</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>A지냐크</t>
+          <t>셀래스틴</t>
         </is>
       </c>
       <c r="D108" t="inlineStr">
         <is>
-          <t>5_3</t>
+          <t>5_0</t>
         </is>
       </c>
       <c r="E108" t="inlineStr">
         <is>
-          <t>승</t>
+          <t>패</t>
         </is>
       </c>
       <c r="F108" t="inlineStr">
         <is>
-          <t>0708ManUtd_868001397(2골), 0708ManUtd_834239053(1골), 0708ManUtd_851226161(1골), 0708ManUtd_868037576(1골), A지냐크_861167134(2골), A지냐크_877031432(1골)</t>
+          <t>UNIT_848180930(1골), UNIT_867166676(4골)</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>2026-10-12 13:44:20</t>
+          <t>2026-10-13 10:23:58</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>0708ManUtd</t>
+          <t>UNIT</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
@@ -3871,7 +3871,7 @@
       </c>
       <c r="D109" t="inlineStr">
         <is>
-          <t>2_1</t>
+          <t>6_0</t>
         </is>
       </c>
       <c r="E109" t="inlineStr">
@@ -3881,29 +3881,29 @@
       </c>
       <c r="F109" t="inlineStr">
         <is>
-          <t>0708ManUtd_868001397(2골), 셀래스틴_861005680(1골)</t>
+          <t>UNIT_867135455(1골), UNIT_848180930(2골), UNIT_867166676(2골), UNIT_840228251(1골)</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>2026-10-13 10:11:17</t>
+          <t>2026-10-13 13:02:46</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>UNIT</t>
+          <t>콩콩콩룔</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>셀래스틴</t>
+          <t>비주류중독</t>
         </is>
       </c>
       <c r="D110" t="inlineStr">
         <is>
-          <t>5_0</t>
+          <t>0_0</t>
         </is>
       </c>
       <c r="E110" t="inlineStr">
@@ -3911,48 +3911,44 @@
           <t>패</t>
         </is>
       </c>
-      <c r="F110" t="inlineStr">
-        <is>
-          <t>UNIT_848180930(1골), UNIT_867166676(4골)</t>
-        </is>
-      </c>
+      <c r="F110" t="inlineStr"/>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>2026-10-13 10:23:58</t>
+          <t>2026-10-13 13:15:38</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>UNIT</t>
+          <t>콩콩콩룔</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>셀래스틴</t>
+          <t>비주류중독</t>
         </is>
       </c>
       <c r="D111" t="inlineStr">
         <is>
-          <t>6_0</t>
+          <t>0_2</t>
         </is>
       </c>
       <c r="E111" t="inlineStr">
         <is>
-          <t>승</t>
+          <t>패</t>
         </is>
       </c>
       <c r="F111" t="inlineStr">
         <is>
-          <t>UNIT_867135455(1골), UNIT_848180930(2골), UNIT_867166676(2골), UNIT_840228251(1골)</t>
+          <t>비주류중독_840052241(1골), 비주류중독_848006975(1골)</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>2026-10-13 13:02:46</t>
+          <t>2026-10-13 13:27:17</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
@@ -3967,7 +3963,7 @@
       </c>
       <c r="D112" t="inlineStr">
         <is>
-          <t>0_0</t>
+          <t>4_5</t>
         </is>
       </c>
       <c r="E112" t="inlineStr">
@@ -3975,69 +3971,521 @@
           <t>패</t>
         </is>
       </c>
-      <c r="F112" t="inlineStr"/>
+      <c r="F112" t="inlineStr">
+        <is>
+          <t>콩콩콩룔_866223710(1골), 콩콩콩룔_867223848(3골), 비주류중독_839247699(1골), 비주류중독_834239977(1골), 비주류중독_848006975(1골), 비주류중독_840052241(2골)</t>
+        </is>
+      </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>2026-10-13 13:15:38</t>
+          <t>2026-10-13 16:14:32</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>콩콩콩룔</t>
+          <t>UNIT</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>비주류중독</t>
+          <t>Voor</t>
         </is>
       </c>
       <c r="D113" t="inlineStr">
         <is>
-          <t>0_2</t>
+          <t>3_2</t>
         </is>
       </c>
       <c r="E113" t="inlineStr">
         <is>
-          <t>패</t>
+          <t>승</t>
         </is>
       </c>
       <c r="F113" t="inlineStr">
         <is>
-          <t>비주류중독_840052241(1골), 비주류중독_848006975(1골)</t>
+          <t>UNIT_840228251(1골), UNIT_867166676(2골), Voor_868007512(1골), Voor_835183277(1골)</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>2026-10-13 13:27:17</t>
+          <t>2026-10-13 16:26:07</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>콩콩콩룔</t>
+          <t>UNIT</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>비주류중독</t>
+          <t>Voor</t>
         </is>
       </c>
       <c r="D114" t="inlineStr">
         <is>
-          <t>4_5</t>
+          <t>3_None</t>
         </is>
       </c>
       <c r="E114" t="inlineStr">
         <is>
-          <t>패</t>
+          <t>승</t>
         </is>
       </c>
       <c r="F114" t="inlineStr">
         <is>
-          <t>콩콩콩룔_866223710(1골), 콩콩콩룔_867223848(3골), 비주류중독_839247699(1골), 비주류중독_834239977(1골), 비주류중독_848006975(1골), 비주류중독_840052241(2골)</t>
+          <t>UNIT_848180930(2골), UNIT_867166676(1골)</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>2026-10-13 16:38:10</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>UNIT</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>Voor</t>
+        </is>
+      </c>
+      <c r="D115" t="inlineStr">
+        <is>
+          <t>5_4</t>
+        </is>
+      </c>
+      <c r="E115" t="inlineStr">
+        <is>
+          <t>승</t>
+        </is>
+      </c>
+      <c r="F115" t="inlineStr">
+        <is>
+          <t>UNIT_867166676(1골), UNIT_848180930(4골), Voor_845201024(1골), Voor_868007512(1골), Voor_852233700(2골)</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>2026-10-13 16:51:42</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>UNIT</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>Voor</t>
+        </is>
+      </c>
+      <c r="D116" t="inlineStr">
+        <is>
+          <t>4_2</t>
+        </is>
+      </c>
+      <c r="E116" t="inlineStr">
+        <is>
+          <t>승</t>
+        </is>
+      </c>
+      <c r="F116" t="inlineStr">
+        <is>
+          <t>UNIT_848180930(2골), UNIT_867166676(2골), Voor_852233700(1골), Voor_835183277(1골)</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>2026-10-13 17:10:24</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>UNIT</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>Voor</t>
+        </is>
+      </c>
+      <c r="D117" t="inlineStr">
+        <is>
+          <t>6_6</t>
+        </is>
+      </c>
+      <c r="E117" t="inlineStr">
+        <is>
+          <t>승</t>
+        </is>
+      </c>
+      <c r="F117" t="inlineStr">
+        <is>
+          <t>UNIT_848180930(1골), UNIT_840192883(1골), UNIT_840228251(1골), UNIT_867166676(3골), Voor_845247090(3골), Voor_868007512(2골), Voor_852233700(1골)</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>2026-10-14 10:54:40</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>UNIT</t>
+        </is>
+      </c>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>셀래스틴</t>
+        </is>
+      </c>
+      <c r="D118" t="inlineStr">
+        <is>
+          <t>3_2</t>
+        </is>
+      </c>
+      <c r="E118" t="inlineStr">
+        <is>
+          <t>승</t>
+        </is>
+      </c>
+      <c r="F118" t="inlineStr">
+        <is>
+          <t>UNIT_848180930(2골), UNIT_867166676(1골), 셀래스틴_846199564(1골), 셀래스틴_848230938(1골)</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>2026-10-14 11:06:43</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>UNIT</t>
+        </is>
+      </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>셀래스틴</t>
+        </is>
+      </c>
+      <c r="D119" t="inlineStr">
+        <is>
+          <t>5_2</t>
+        </is>
+      </c>
+      <c r="E119" t="inlineStr">
+        <is>
+          <t>승</t>
+        </is>
+      </c>
+      <c r="F119" t="inlineStr">
+        <is>
+          <t>UNIT_848180930(2골), UNIT_867166676(3골), 셀래스틴_852241461(2골)</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>2026-10-14 11:18:07</t>
+        </is>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>UNIT</t>
+        </is>
+      </c>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>셀래스틴</t>
+        </is>
+      </c>
+      <c r="D120" t="inlineStr">
+        <is>
+          <t>3_4</t>
+        </is>
+      </c>
+      <c r="E120" t="inlineStr">
+        <is>
+          <t>패</t>
+        </is>
+      </c>
+      <c r="F120" t="inlineStr">
+        <is>
+          <t>UNIT_848180930(3골), 셀래스틴_848194765(1골), 셀래스틴_861005680(3골)</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>2026-10-14 11:48:16</t>
+        </is>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>은안</t>
+        </is>
+      </c>
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>아들러</t>
+        </is>
+      </c>
+      <c r="D121" t="inlineStr">
+        <is>
+          <t>3_1</t>
+        </is>
+      </c>
+      <c r="E121" t="inlineStr">
+        <is>
+          <t>승</t>
+        </is>
+      </c>
+      <c r="F121" t="inlineStr">
+        <is>
+          <t>은안_866241236(1골), 은안_856246420(1골), 은안_852237692(1골), 아들러_866251377(1골)</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>2026-10-14 12:02:04</t>
+        </is>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>은안</t>
+        </is>
+      </c>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>아들러</t>
+        </is>
+      </c>
+      <c r="D122" t="inlineStr">
+        <is>
+          <t>2_2</t>
+        </is>
+      </c>
+      <c r="E122" t="inlineStr">
+        <is>
+          <t>무</t>
+        </is>
+      </c>
+      <c r="F122" t="inlineStr">
+        <is>
+          <t>은안_866241236(2골), 아들러_866251377(1골), 아들러_840191208(1골)</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>2026-10-14 13:23:01</t>
+        </is>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>0708ManUtd</t>
+        </is>
+      </c>
+      <c r="C123" t="inlineStr">
+        <is>
+          <t>개포동덕배</t>
+        </is>
+      </c>
+      <c r="D123" t="inlineStr">
+        <is>
+          <t>3_5</t>
+        </is>
+      </c>
+      <c r="E123" t="inlineStr">
+        <is>
+          <t>패</t>
+        </is>
+      </c>
+      <c r="F123" t="inlineStr">
+        <is>
+          <t>0708ManUtd_868037576(1골), 0708ManUtd_848238794(1골), 0708ManUtd_868001397(1골), 개포동덕배_848206113(1골), 개포동덕배_845190048(3골), 개포동덕배_856202126(1골)</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>2026-10-14 13:34:28</t>
+        </is>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>0708ManUtd</t>
+        </is>
+      </c>
+      <c r="C124" t="inlineStr">
+        <is>
+          <t>개포동덕배</t>
+        </is>
+      </c>
+      <c r="D124" t="inlineStr">
+        <is>
+          <t>1_4</t>
+        </is>
+      </c>
+      <c r="E124" t="inlineStr">
+        <is>
+          <t>패</t>
+        </is>
+      </c>
+      <c r="F124" t="inlineStr">
+        <is>
+          <t>0708ManUtd_868037576(1골), 개포동덕배_845190048(4골)</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>2026-10-15 10:12:26</t>
+        </is>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>오스트리아</t>
+        </is>
+      </c>
+      <c r="C125" t="inlineStr">
+        <is>
+          <t>Gucci와퍼</t>
+        </is>
+      </c>
+      <c r="D125" t="inlineStr">
+        <is>
+          <t>2_1</t>
+        </is>
+      </c>
+      <c r="E125" t="inlineStr">
+        <is>
+          <t>승</t>
+        </is>
+      </c>
+      <c r="F125" t="inlineStr">
+        <is>
+          <t>오스트리아_864199266(1골), 오스트리아_291223790(1골), Gucci와퍼_852168473(1골)</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>2026-10-15 10:23:39</t>
+        </is>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>오스트리아</t>
+        </is>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>Gucci와퍼</t>
+        </is>
+      </c>
+      <c r="D126" t="inlineStr">
+        <is>
+          <t>2_0</t>
+        </is>
+      </c>
+      <c r="E126" t="inlineStr">
+        <is>
+          <t>승</t>
+        </is>
+      </c>
+      <c r="F126" t="inlineStr">
+        <is>
+          <t>오스트리아_864191566(1골), 오스트리아_864199266(1골)</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>2026-10-15 13:04:31</t>
+        </is>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>호야국2인</t>
+        </is>
+      </c>
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>셀래스틴</t>
+        </is>
+      </c>
+      <c r="D127" t="inlineStr">
+        <is>
+          <t>1_2</t>
+        </is>
+      </c>
+      <c r="E127" t="inlineStr">
+        <is>
+          <t>패</t>
+        </is>
+      </c>
+      <c r="F127" t="inlineStr">
+        <is>
+          <t>호야국2인_846192505(1골), 셀래스틴_861005680(1골), 셀래스틴_863233419(1골)</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>2026-10-15 13:14:57</t>
+        </is>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>호야국2인</t>
+        </is>
+      </c>
+      <c r="C128" t="inlineStr">
+        <is>
+          <t>셀래스틴</t>
+        </is>
+      </c>
+      <c r="D128" t="inlineStr">
+        <is>
+          <t>3_3</t>
+        </is>
+      </c>
+      <c r="E128" t="inlineStr">
+        <is>
+          <t>무</t>
+        </is>
+      </c>
+      <c r="F128" t="inlineStr">
+        <is>
+          <t>호야국2인_845198219(1골), 호야국2인_851216409(1골), 호야국2인_848227236(1골), 셀래스틴_861005680(2골), 셀래스틴_863233419(1골)</t>
         </is>
       </c>
     </row>
@@ -4052,7 +4500,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F114"/>
+  <dimension ref="A1:F128"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6598,7 +7046,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>2026-10-11 07:47:05</t>
+          <t>2026-10-11 07:59:52</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
@@ -6613,7 +7061,7 @@
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>2_5</t>
+          <t>2_3</t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
@@ -6623,14 +7071,14 @@
       </c>
       <c r="F81" t="inlineStr">
         <is>
-          <t>A지냐크_877001668(1도움), 셀래스틴_863233419(2도움), 셀래스틴_861005680(1도움), 셀래스틴_852259694(1도움), 셀래스틴_852241461(1도움)</t>
+          <t>A지냐크_834271400(1도움), A지냐크_855213648(1도움), 셀래스틴_848013038(1도움)</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>2026-10-11 07:59:52</t>
+          <t>2026-10-11 08:33:57</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
@@ -6640,29 +7088,29 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>셀래스틴</t>
+          <t>ShangHaiPortFC</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>2_3</t>
+          <t>7_2</t>
         </is>
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>패</t>
+          <t>승</t>
         </is>
       </c>
       <c r="F82" t="inlineStr">
         <is>
-          <t>A지냐크_834271400(1도움), A지냐크_855213648(1도움), 셀래스틴_848013038(1도움)</t>
+          <t>A지냐크_877226851(1도움), A지냐크_877031432(2도움), A지냐크_863241496(3도움), ShangHaiPortFC_861051412(2도움)</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>2026-10-11 08:33:57</t>
+          <t>2026-10-11 08:45:05</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
@@ -6677,39 +7125,39 @@
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>7_2</t>
+          <t>1_5</t>
         </is>
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>승</t>
+          <t>패</t>
         </is>
       </c>
       <c r="F83" t="inlineStr">
         <is>
-          <t>A지냐크_877226851(1도움), A지냐크_877031432(2도움), A지냐크_863241496(3도움), ShangHaiPortFC_861051412(2도움)</t>
+          <t>ShangHaiPortFC_861051412(2도움), ShangHaiPortFC_827143001(2도움)</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>2026-10-11 08:45:05</t>
+          <t>2026-10-11 10:08:39</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>A지냐크</t>
+          <t>ShangHaiPortFC</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>ShangHaiPortFC</t>
+          <t>용신</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>1_5</t>
+          <t>2_6</t>
         </is>
       </c>
       <c r="E84" t="inlineStr">
@@ -6719,14 +7167,14 @@
       </c>
       <c r="F84" t="inlineStr">
         <is>
-          <t>ShangHaiPortFC_861051412(2도움), ShangHaiPortFC_827143001(2도움)</t>
+          <t>용신_863245367(1도움), 용신_866200104(1도움), 용신_826251421(1도움), 용신_877216267(1도움), 용신_291213648(1도움)</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>2026-10-11 10:08:39</t>
+          <t>2026-10-11 10:48:32</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
@@ -6741,56 +7189,56 @@
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>2_6</t>
+          <t>3_2</t>
         </is>
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>패</t>
+          <t>승</t>
         </is>
       </c>
       <c r="F85" t="inlineStr">
         <is>
-          <t>용신_863245367(1도움), 용신_866200104(1도움), 용신_826251421(1도움), 용신_877216267(1도움), 용신_291213648(1도움)</t>
+          <t>ShangHaiPortFC_827143001(1도움), ShangHaiPortFC_864191910(1도움), 용신_863245367(1도움), 용신_101173731(1도움)</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>2026-10-11 10:48:32</t>
+          <t>2026-10-11 11:11:43</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>ShangHaiPortFC</t>
+          <t>여수가스</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>용신</t>
+          <t>셀래스틴</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>3_2</t>
+          <t>4_6</t>
         </is>
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>승</t>
+          <t>패</t>
         </is>
       </c>
       <c r="F86" t="inlineStr">
         <is>
-          <t>ShangHaiPortFC_827143001(1도움), ShangHaiPortFC_864191910(1도움), 용신_863245367(1도움), 용신_101173731(1도움)</t>
+          <t>여수가스_828231747(1도움), 여수가스_861215732(1도움), 여수가스_861162895(2도움), 셀래스틴_852241461(1도움), 셀래스틴_863233419(1도움), 셀래스틴_861005680(1도움), 셀래스틴_848194765(1도움), 셀래스틴_848231866(1도움), 셀래스틴_852259694(1도움)</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>2026-10-11 11:11:43</t>
+          <t>2026-10-11 11:23:07</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
@@ -6805,29 +7253,29 @@
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>4_6</t>
+          <t>2_1</t>
         </is>
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>패</t>
+          <t>승</t>
         </is>
       </c>
       <c r="F87" t="inlineStr">
         <is>
-          <t>여수가스_828231747(1도움), 여수가스_861215732(1도움), 여수가스_861162895(2도움), 셀래스틴_852241461(1도움), 셀래스틴_863233419(1도움), 셀래스틴_861005680(1도움), 셀래스틴_848194765(1도움), 셀래스틴_848231866(1도움), 셀래스틴_852259694(1도움)</t>
+          <t>여수가스_861215732(1도움), 여수가스_828231747(1도움), 셀래스틴_848231866(1도움)</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>2026-10-11 11:23:07</t>
+          <t>2026-10-11 12:05:40</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>여수가스</t>
+          <t>앙쿠</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
@@ -6837,24 +7285,24 @@
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>2_1</t>
+          <t>1_2</t>
         </is>
       </c>
       <c r="E88" t="inlineStr">
         <is>
-          <t>승</t>
+          <t>패</t>
         </is>
       </c>
       <c r="F88" t="inlineStr">
         <is>
-          <t>여수가스_861215732(1도움), 여수가스_828231747(1도움), 셀래스틴_848231866(1도움)</t>
+          <t>앙쿠_861049369(1도움), 셀래스틴_848194765(1도움), 셀래스틴_861005680(1도움)</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>2026-10-11 12:05:40</t>
+          <t>2026-10-11 12:16:11</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
@@ -6869,7 +7317,7 @@
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>1_2</t>
+          <t>0_2</t>
         </is>
       </c>
       <c r="E89" t="inlineStr">
@@ -6879,14 +7327,14 @@
       </c>
       <c r="F89" t="inlineStr">
         <is>
-          <t>앙쿠_861049369(1도움), 셀래스틴_848194765(1도움), 셀래스틴_861005680(1도움)</t>
+          <t>셀래스틴_852259694(2도움)</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>2026-10-11 12:16:11</t>
+          <t>2026-10-11 12:25:49</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
@@ -6901,56 +7349,56 @@
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>0_2</t>
+          <t>1_1</t>
         </is>
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t>패</t>
+          <t>무</t>
         </is>
       </c>
       <c r="F90" t="inlineStr">
         <is>
-          <t>셀래스틴_852259694(2도움)</t>
+          <t>앙쿠_851194765(1도움), 셀래스틴_848231866(1도움)</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>2026-10-11 12:25:49</t>
+          <t>2026-10-11 17:54:01</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>앙쿠</t>
+          <t>UNIT</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>셀래스틴</t>
+          <t>Voor</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>1_1</t>
+          <t>0_4</t>
         </is>
       </c>
       <c r="E91" t="inlineStr">
         <is>
-          <t>무</t>
+          <t>패</t>
         </is>
       </c>
       <c r="F91" t="inlineStr">
         <is>
-          <t>앙쿠_851194765(1도움), 셀래스틴_848231866(1도움)</t>
+          <t>Voor_861000027(1도움), Voor_852233700(1도움), Voor_868007512(1도움), Voor_856256079(1도움)</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>2026-10-11 17:43:20</t>
+          <t>2026-10-11 18:05:57</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
@@ -6965,24 +7413,24 @@
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>4_4</t>
+          <t>4_2</t>
         </is>
       </c>
       <c r="E92" t="inlineStr">
         <is>
-          <t>패</t>
+          <t>승</t>
         </is>
       </c>
       <c r="F92" t="inlineStr">
         <is>
-          <t>UNIT_840192883(1도움), UNIT_848180930(1도움), UNIT_840228251(2도움), Voor_856256079(1도움), Voor_835183277(2도움)</t>
+          <t>UNIT_840192883(1도움), UNIT_840210736(1도움), UNIT_848265695(1도움), UNIT_840228251(1도움), Voor_856256079(1도움), Voor_852001201(1도움)</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>2026-10-11 17:54:01</t>
+          <t>2026-10-11 18:23:54</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
@@ -6997,7 +7445,7 @@
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>0_4</t>
+          <t>3_3</t>
         </is>
       </c>
       <c r="E93" t="inlineStr">
@@ -7007,14 +7455,14 @@
       </c>
       <c r="F93" t="inlineStr">
         <is>
-          <t>Voor_861000027(1도움), Voor_852233700(1도움), Voor_868007512(1도움), Voor_856256079(1도움)</t>
+          <t>UNIT_840228251(1도움), UNIT_840210736(1도움), UNIT_829274967(1도움), Voor_835183277(1도움), Voor_868007512(1도움)</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>2026-10-11 18:05:57</t>
+          <t>2026-10-11 18:36:25</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
@@ -7029,24 +7477,24 @@
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>4_2</t>
+          <t>3_4</t>
         </is>
       </c>
       <c r="E94" t="inlineStr">
         <is>
-          <t>승</t>
+          <t>패</t>
         </is>
       </c>
       <c r="F94" t="inlineStr">
         <is>
-          <t>UNIT_840192883(1도움), UNIT_840210736(1도움), UNIT_848265695(1도움), UNIT_840228251(1도움), Voor_856256079(1도움), Voor_852001201(1도움)</t>
+          <t>UNIT_840228251(1도움), UNIT_840210736(1도움), UNIT_840192883(1도움), Voor_868007512(1도움), Voor_852233700(1도움), Voor_845247090(1도움), Voor_848216150(1도움)</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>2026-10-11 18:23:54</t>
+          <t>2026-10-11 18:53:58</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
@@ -7071,14 +7519,14 @@
       </c>
       <c r="F95" t="inlineStr">
         <is>
-          <t>UNIT_840228251(1도움), UNIT_840210736(1도움), UNIT_829274967(1도움), Voor_835183277(1도움), Voor_868007512(1도움)</t>
+          <t>UNIT_840216150(1도움), UNIT_840228251(2도움), Voor_835183277(1도움), Voor_852001201(1도움), Voor_845239231(1도움)</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>2026-10-11 18:36:25</t>
+          <t>2026-10-12 10:04:39</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
@@ -7088,76 +7536,76 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>Voor</t>
+          <t>셀래스틴</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>3_4</t>
+          <t>2_1</t>
         </is>
       </c>
       <c r="E96" t="inlineStr">
         <is>
-          <t>패</t>
+          <t>승</t>
         </is>
       </c>
       <c r="F96" t="inlineStr">
         <is>
-          <t>UNIT_840228251(1도움), UNIT_840210736(1도움), UNIT_840192883(1도움), Voor_868007512(1도움), Voor_852233700(1도움), Voor_845247090(1도움), Voor_848216150(1도움)</t>
+          <t>UNIT_848180930(1도움), 셀래스틴_863200458(1도움)</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>2026-10-11 18:53:58</t>
+          <t>2026-10-12 12:06:47</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>UNIT</t>
+          <t>0708ManUtd</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>Voor</t>
+          <t>콩콩콩룔</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>3_3</t>
+          <t>3_0</t>
         </is>
       </c>
       <c r="E97" t="inlineStr">
         <is>
-          <t>패</t>
+          <t>승</t>
         </is>
       </c>
       <c r="F97" t="inlineStr">
         <is>
-          <t>UNIT_840216150(1도움), UNIT_840228251(2도움), Voor_835183277(1도움), Voor_852001201(1도움), Voor_845239231(1도움)</t>
+          <t>0708ManUtd_868001397(1도움), 0708ManUtd_848238794(2도움)</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>2026-10-12 10:04:39</t>
+          <t>2026-10-12 12:12:43</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>UNIT</t>
+          <t>A지냐크</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>셀래스틴</t>
+          <t>Gucci와퍼</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>2_1</t>
+          <t>4_1</t>
         </is>
       </c>
       <c r="E98" t="inlineStr">
@@ -7167,14 +7615,14 @@
       </c>
       <c r="F98" t="inlineStr">
         <is>
-          <t>UNIT_848180930(1도움), 셀래스틴_863200458(1도움)</t>
+          <t>A지냐크_861167134(2도움), A지냐크_863241496(2도움), Gucci와퍼_852010264(1도움)</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>2026-10-12 12:06:47</t>
+          <t>2026-10-12 12:17:19</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
@@ -7199,14 +7647,14 @@
       </c>
       <c r="F99" t="inlineStr">
         <is>
-          <t>0708ManUtd_868001397(1도움), 0708ManUtd_848238794(2도움)</t>
+          <t>0708ManUtd_868037576(1도움), 0708ManUtd_851226161(1도움), 0708ManUtd_868001397(1도움)</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>2026-10-12 12:12:43</t>
+          <t>2026-10-12 12:30:45</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
@@ -7221,24 +7669,24 @@
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>4_1</t>
+          <t>4_5</t>
         </is>
       </c>
       <c r="E100" t="inlineStr">
         <is>
-          <t>승</t>
+          <t>패</t>
         </is>
       </c>
       <c r="F100" t="inlineStr">
         <is>
-          <t>A지냐크_861167134(2도움), A지냐크_863241496(2도움), Gucci와퍼_852010264(1도움)</t>
+          <t>A지냐크_861167134(1도움), A지냐크_877226851(1도움), A지냐크_863241496(1도움), A지냐크_840204970(1도움), Gucci와퍼_852168473(2도움), Gucci와퍼_840208574(1도움), Gucci와퍼_852208128(1도움)</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>2026-10-12 12:17:19</t>
+          <t>2026-10-12 12:39:42</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
@@ -7248,12 +7696,12 @@
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>콩콩콩룔</t>
+          <t>용신</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>3_0</t>
+          <t>3_1</t>
         </is>
       </c>
       <c r="E101" t="inlineStr">
@@ -7263,14 +7711,14 @@
       </c>
       <c r="F101" t="inlineStr">
         <is>
-          <t>0708ManUtd_868037576(1도움), 0708ManUtd_851226161(1도움), 0708ManUtd_868001397(1도움)</t>
+          <t>0708ManUtd_848238794(1도움), 0708ManUtd_851226161(1도움), 0708ManUtd_835183277(1도움), 용신_101173731(1도움)</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>2026-10-12 12:30:45</t>
+          <t>2026-10-12 12:45:19</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
@@ -7285,7 +7733,7 @@
       </c>
       <c r="D102" t="inlineStr">
         <is>
-          <t>4_5</t>
+          <t>3_4</t>
         </is>
       </c>
       <c r="E102" t="inlineStr">
@@ -7295,14 +7743,14 @@
       </c>
       <c r="F102" t="inlineStr">
         <is>
-          <t>A지냐크_861167134(1도움), A지냐크_877226851(1도움), A지냐크_863241496(1도움), A지냐크_840204970(1도움), Gucci와퍼_852168473(2도움), Gucci와퍼_840208574(1도움), Gucci와퍼_852208128(1도움)</t>
+          <t>A지냐크_861167134(1도움), A지냐크_840204970(1도움), A지냐크_877031432(1도움), Gucci와퍼_852168473(2도움), Gucci와퍼_851210697(1도움), Gucci와퍼_864200104(1도움)</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>2026-10-12 12:39:42</t>
+          <t>2026-10-12 12:50:47</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
@@ -7317,39 +7765,39 @@
       </c>
       <c r="D103" t="inlineStr">
         <is>
-          <t>3_1</t>
+          <t>3_3</t>
         </is>
       </c>
       <c r="E103" t="inlineStr">
         <is>
-          <t>승</t>
+          <t>무</t>
         </is>
       </c>
       <c r="F103" t="inlineStr">
         <is>
-          <t>0708ManUtd_848238794(1도움), 0708ManUtd_851226161(1도움), 0708ManUtd_835183277(1도움), 용신_101173731(1도움)</t>
+          <t>0708ManUtd_868037576(1도움), 0708ManUtd_851226161(2도움), 용신_101173731(1도움), 용신_826251421(2도움)</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>2026-10-12 12:45:19</t>
+          <t>2026-10-12 13:04:34</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>A지냐크</t>
+          <t>0708ManUtd</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>Gucci와퍼</t>
+          <t>UNIT</t>
         </is>
       </c>
       <c r="D104" t="inlineStr">
         <is>
-          <t>3_4</t>
+          <t>2_4</t>
         </is>
       </c>
       <c r="E104" t="inlineStr">
@@ -7359,14 +7807,14 @@
       </c>
       <c r="F104" t="inlineStr">
         <is>
-          <t>A지냐크_861167134(1도움), A지냐크_840204970(1도움), A지냐크_877031432(1도움), Gucci와퍼_852168473(2도움), Gucci와퍼_851210697(1도움), Gucci와퍼_864200104(1도움)</t>
+          <t>0708ManUtd_848238794(2도움), UNIT_840210736(1도움), UNIT_840228251(2도움), UNIT_840225782(1도움)</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>2026-10-12 12:50:47</t>
+          <t>2026-10-12 13:17:50</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
@@ -7376,29 +7824,29 @@
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>용신</t>
+          <t>A지냐크</t>
         </is>
       </c>
       <c r="D105" t="inlineStr">
         <is>
-          <t>3_3</t>
+          <t>7_0</t>
         </is>
       </c>
       <c r="E105" t="inlineStr">
         <is>
-          <t>무</t>
+          <t>승</t>
         </is>
       </c>
       <c r="F105" t="inlineStr">
         <is>
-          <t>0708ManUtd_868037576(1도움), 0708ManUtd_851226161(2도움), 용신_101173731(1도움), 용신_826251421(2도움)</t>
+          <t>0708ManUtd_868001397(1도움), 0708ManUtd_827005589(1도움), 0708ManUtd_834239053(1도움), 0708ManUtd_868037576(2도움)</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>2026-10-12 13:04:34</t>
+          <t>2026-10-12 13:29:18</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
@@ -7408,29 +7856,29 @@
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>UNIT</t>
+          <t>A지냐크</t>
         </is>
       </c>
       <c r="D106" t="inlineStr">
         <is>
-          <t>2_4</t>
+          <t>5_3</t>
         </is>
       </c>
       <c r="E106" t="inlineStr">
         <is>
-          <t>패</t>
+          <t>승</t>
         </is>
       </c>
       <c r="F106" t="inlineStr">
         <is>
-          <t>0708ManUtd_848238794(2도움), UNIT_840210736(1도움), UNIT_840228251(2도움), UNIT_840225782(1도움)</t>
+          <t>0708ManUtd_863239231(1도움), 0708ManUtd_851226161(3도움), 0708ManUtd_848238794(1도움), A지냐크_863241496(1도움), A지냐크_840204970(1도움), A지냐크_877031432(1도움)</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>2026-10-12 13:17:50</t>
+          <t>2026-10-12 13:44:20</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
@@ -7440,12 +7888,12 @@
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>A지냐크</t>
+          <t>셀래스틴</t>
         </is>
       </c>
       <c r="D107" t="inlineStr">
         <is>
-          <t>7_0</t>
+          <t>2_1</t>
         </is>
       </c>
       <c r="E107" t="inlineStr">
@@ -7455,51 +7903,51 @@
       </c>
       <c r="F107" t="inlineStr">
         <is>
-          <t>0708ManUtd_868001397(1도움), 0708ManUtd_827005589(1도움), 0708ManUtd_834239053(1도움), 0708ManUtd_868037576(2도움)</t>
+          <t>0708ManUtd_851226161(1도움), 셀래스틴_852241461(1도움)</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>2026-10-12 13:29:18</t>
+          <t>2026-10-13 10:11:17</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>0708ManUtd</t>
+          <t>UNIT</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>A지냐크</t>
+          <t>셀래스틴</t>
         </is>
       </c>
       <c r="D108" t="inlineStr">
         <is>
-          <t>5_3</t>
+          <t>5_0</t>
         </is>
       </c>
       <c r="E108" t="inlineStr">
         <is>
-          <t>승</t>
+          <t>패</t>
         </is>
       </c>
       <c r="F108" t="inlineStr">
         <is>
-          <t>0708ManUtd_863239231(1도움), 0708ManUtd_851226161(3도움), 0708ManUtd_848238794(1도움), A지냐크_863241496(1도움), A지냐크_840204970(1도움), A지냐크_877031432(1도움)</t>
+          <t>UNIT_840192883(1도움), UNIT_840228251(1도움), UNIT_848180930(1도움), UNIT_867135455(1도움)</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>2026-10-12 13:44:20</t>
+          <t>2026-10-13 10:23:58</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>0708ManUtd</t>
+          <t>UNIT</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
@@ -7509,7 +7957,7 @@
       </c>
       <c r="D109" t="inlineStr">
         <is>
-          <t>2_1</t>
+          <t>6_0</t>
         </is>
       </c>
       <c r="E109" t="inlineStr">
@@ -7519,29 +7967,29 @@
       </c>
       <c r="F109" t="inlineStr">
         <is>
-          <t>0708ManUtd_851226161(1도움), 셀래스틴_852241461(1도움)</t>
+          <t>UNIT_867135455(1도움), UNIT_840228251(2도움), UNIT_840225782(1도움), UNIT_851236403(1도움)</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>2026-10-13 10:11:17</t>
+          <t>2026-10-13 13:02:46</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>UNIT</t>
+          <t>콩콩콩룔</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>셀래스틴</t>
+          <t>비주류중독</t>
         </is>
       </c>
       <c r="D110" t="inlineStr">
         <is>
-          <t>5_0</t>
+          <t>0_0</t>
         </is>
       </c>
       <c r="E110" t="inlineStr">
@@ -7549,48 +7997,44 @@
           <t>패</t>
         </is>
       </c>
-      <c r="F110" t="inlineStr">
-        <is>
-          <t>UNIT_840192883(1도움), UNIT_840228251(1도움), UNIT_848180930(1도움), UNIT_867135455(1도움)</t>
-        </is>
-      </c>
+      <c r="F110" t="inlineStr"/>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>2026-10-13 10:23:58</t>
+          <t>2026-10-13 13:15:38</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>UNIT</t>
+          <t>콩콩콩룔</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>셀래스틴</t>
+          <t>비주류중독</t>
         </is>
       </c>
       <c r="D111" t="inlineStr">
         <is>
-          <t>6_0</t>
+          <t>0_2</t>
         </is>
       </c>
       <c r="E111" t="inlineStr">
         <is>
-          <t>승</t>
+          <t>패</t>
         </is>
       </c>
       <c r="F111" t="inlineStr">
         <is>
-          <t>UNIT_867135455(1도움), UNIT_840228251(2도움), UNIT_840225782(1도움), UNIT_851236403(1도움)</t>
+          <t>비주류중독_840052241(1도움), 비주류중독_848006975(1도움)</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>2026-10-13 13:02:46</t>
+          <t>2026-10-13 13:27:17</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
@@ -7605,7 +8049,7 @@
       </c>
       <c r="D112" t="inlineStr">
         <is>
-          <t>0_0</t>
+          <t>4_5</t>
         </is>
       </c>
       <c r="E112" t="inlineStr">
@@ -7613,69 +8057,521 @@
           <t>패</t>
         </is>
       </c>
-      <c r="F112" t="inlineStr"/>
+      <c r="F112" t="inlineStr">
+        <is>
+          <t>콩콩콩룔_848189505(1도움), 콩콩콩룔_866223710(2도움), 콩콩콩룔_867223848(1도움), 비주류중독_839247699(2도움), 비주류중독_848006975(2도움), 비주류중독_840052241(1도움)</t>
+        </is>
+      </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>2026-10-13 13:15:38</t>
+          <t>2026-10-13 16:14:32</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>콩콩콩룔</t>
+          <t>UNIT</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>비주류중독</t>
+          <t>Voor</t>
         </is>
       </c>
       <c r="D113" t="inlineStr">
         <is>
-          <t>0_2</t>
+          <t>3_2</t>
         </is>
       </c>
       <c r="E113" t="inlineStr">
         <is>
-          <t>패</t>
+          <t>승</t>
         </is>
       </c>
       <c r="F113" t="inlineStr">
         <is>
-          <t>비주류중독_840052241(1도움), 비주류중독_848006975(1도움)</t>
+          <t>UNIT_840192883(1도움), Voor_852233700(1도움), Voor_858025420(1도움)</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>2026-10-13 13:27:17</t>
+          <t>2026-10-13 16:26:07</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>콩콩콩룔</t>
+          <t>UNIT</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>비주류중독</t>
+          <t>Voor</t>
         </is>
       </c>
       <c r="D114" t="inlineStr">
         <is>
-          <t>4_5</t>
+          <t>3_None</t>
         </is>
       </c>
       <c r="E114" t="inlineStr">
         <is>
-          <t>패</t>
+          <t>승</t>
         </is>
       </c>
       <c r="F114" t="inlineStr">
         <is>
-          <t>콩콩콩룔_848189505(1도움), 콩콩콩룔_866223710(2도움), 콩콩콩룔_867223848(1도움), 비주류중독_839247699(2도움), 비주류중독_848006975(2도움), 비주류중독_840052241(1도움)</t>
+          <t>UNIT_867166676(1도움), UNIT_845210736(2도움)</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>2026-10-13 16:38:10</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>UNIT</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>Voor</t>
+        </is>
+      </c>
+      <c r="D115" t="inlineStr">
+        <is>
+          <t>5_4</t>
+        </is>
+      </c>
+      <c r="E115" t="inlineStr">
+        <is>
+          <t>승</t>
+        </is>
+      </c>
+      <c r="F115" t="inlineStr">
+        <is>
+          <t>UNIT_840228251(2도움), UNIT_840192883(1도움), UNIT_840225782(2도움), Voor_856256079(1도움), Voor_835183277(1도움), Voor_852233700(1도움)</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>2026-10-13 16:51:42</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>UNIT</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>Voor</t>
+        </is>
+      </c>
+      <c r="D116" t="inlineStr">
+        <is>
+          <t>4_2</t>
+        </is>
+      </c>
+      <c r="E116" t="inlineStr">
+        <is>
+          <t>승</t>
+        </is>
+      </c>
+      <c r="F116" t="inlineStr">
+        <is>
+          <t>UNIT_867166676(1도움), UNIT_840228251(1도움), UNIT_840192883(2도움), Voor_868007512(2도움)</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>2026-10-13 17:10:24</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>UNIT</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>Voor</t>
+        </is>
+      </c>
+      <c r="D117" t="inlineStr">
+        <is>
+          <t>6_6</t>
+        </is>
+      </c>
+      <c r="E117" t="inlineStr">
+        <is>
+          <t>승</t>
+        </is>
+      </c>
+      <c r="F117" t="inlineStr">
+        <is>
+          <t>UNIT_840192883(1도움), UNIT_845210736(1도움), UNIT_840228251(2도움), UNIT_867166676(1도움), Voor_868007512(2도움), Voor_852233700(2도움), Voor_861000027(1도움), Voor_856256079(1도움)</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>2026-10-14 10:54:40</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>UNIT</t>
+        </is>
+      </c>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>셀래스틴</t>
+        </is>
+      </c>
+      <c r="D118" t="inlineStr">
+        <is>
+          <t>3_2</t>
+        </is>
+      </c>
+      <c r="E118" t="inlineStr">
+        <is>
+          <t>승</t>
+        </is>
+      </c>
+      <c r="F118" t="inlineStr">
+        <is>
+          <t>UNIT_845210736(1도움), UNIT_840225782(1도움), UNIT_867135455(1도움), 셀래스틴_848231866(1도움), 셀래스틴_852241461(1도움)</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>2026-10-14 11:06:43</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>UNIT</t>
+        </is>
+      </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>셀래스틴</t>
+        </is>
+      </c>
+      <c r="D119" t="inlineStr">
+        <is>
+          <t>5_2</t>
+        </is>
+      </c>
+      <c r="E119" t="inlineStr">
+        <is>
+          <t>승</t>
+        </is>
+      </c>
+      <c r="F119" t="inlineStr">
+        <is>
+          <t>UNIT_840225782(1도움), UNIT_840192883(4도움), 셀래스틴_846199564(1도움), 셀래스틴_863233419(1도움)</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>2026-10-14 11:18:07</t>
+        </is>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>UNIT</t>
+        </is>
+      </c>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>셀래스틴</t>
+        </is>
+      </c>
+      <c r="D120" t="inlineStr">
+        <is>
+          <t>3_4</t>
+        </is>
+      </c>
+      <c r="E120" t="inlineStr">
+        <is>
+          <t>패</t>
+        </is>
+      </c>
+      <c r="F120" t="inlineStr">
+        <is>
+          <t>UNIT_840228251(1도움), UNIT_867166676(1도움), UNIT_840192883(1도움), 셀래스틴_848194765(1도움), 셀래스틴_848230938(1도움)</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>2026-10-14 11:48:16</t>
+        </is>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>은안</t>
+        </is>
+      </c>
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>아들러</t>
+        </is>
+      </c>
+      <c r="D121" t="inlineStr">
+        <is>
+          <t>3_1</t>
+        </is>
+      </c>
+      <c r="E121" t="inlineStr">
+        <is>
+          <t>승</t>
+        </is>
+      </c>
+      <c r="F121" t="inlineStr">
+        <is>
+          <t>은안_877143001(1도움), 은안_856246420(1도움)</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>2026-10-14 12:02:04</t>
+        </is>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>은안</t>
+        </is>
+      </c>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>아들러</t>
+        </is>
+      </c>
+      <c r="D122" t="inlineStr">
+        <is>
+          <t>2_2</t>
+        </is>
+      </c>
+      <c r="E122" t="inlineStr">
+        <is>
+          <t>무</t>
+        </is>
+      </c>
+      <c r="F122" t="inlineStr">
+        <is>
+          <t>은안_852237692(1도움), 아들러_840229752(1도움)</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>2026-10-14 13:23:01</t>
+        </is>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>0708ManUtd</t>
+        </is>
+      </c>
+      <c r="C123" t="inlineStr">
+        <is>
+          <t>개포동덕배</t>
+        </is>
+      </c>
+      <c r="D123" t="inlineStr">
+        <is>
+          <t>3_5</t>
+        </is>
+      </c>
+      <c r="E123" t="inlineStr">
+        <is>
+          <t>패</t>
+        </is>
+      </c>
+      <c r="F123" t="inlineStr">
+        <is>
+          <t>0708ManUtd_835183277(2도움), 0708ManUtd_851226161(1도움), 개포동덕배_848206113(1도움), 개포동덕배_845208722(2도움), 개포동덕배_856202126(1도움)</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>2026-10-14 13:34:28</t>
+        </is>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>0708ManUtd</t>
+        </is>
+      </c>
+      <c r="C124" t="inlineStr">
+        <is>
+          <t>개포동덕배</t>
+        </is>
+      </c>
+      <c r="D124" t="inlineStr">
+        <is>
+          <t>1_4</t>
+        </is>
+      </c>
+      <c r="E124" t="inlineStr">
+        <is>
+          <t>패</t>
+        </is>
+      </c>
+      <c r="F124" t="inlineStr">
+        <is>
+          <t>0708ManUtd_868001397(1도움), 개포동덕배_856202126(1도움), 개포동덕배_856275298(2도움), 개포동덕배_848206113(1도움)</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>2026-10-15 10:12:26</t>
+        </is>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>오스트리아</t>
+        </is>
+      </c>
+      <c r="C125" t="inlineStr">
+        <is>
+          <t>Gucci와퍼</t>
+        </is>
+      </c>
+      <c r="D125" t="inlineStr">
+        <is>
+          <t>2_1</t>
+        </is>
+      </c>
+      <c r="E125" t="inlineStr">
+        <is>
+          <t>승</t>
+        </is>
+      </c>
+      <c r="F125" t="inlineStr">
+        <is>
+          <t>오스트리아_864199266(1도움), 오스트리아_851216275(1도움), Gucci와퍼_851210697(1도움)</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>2026-10-15 10:23:39</t>
+        </is>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>오스트리아</t>
+        </is>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>Gucci와퍼</t>
+        </is>
+      </c>
+      <c r="D126" t="inlineStr">
+        <is>
+          <t>2_0</t>
+        </is>
+      </c>
+      <c r="E126" t="inlineStr">
+        <is>
+          <t>승</t>
+        </is>
+      </c>
+      <c r="F126" t="inlineStr">
+        <is>
+          <t>오스트리아_291223790(1도움), 오스트리아_291229071(1도움)</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>2026-10-15 13:04:31</t>
+        </is>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>호야국2인</t>
+        </is>
+      </c>
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>셀래스틴</t>
+        </is>
+      </c>
+      <c r="D127" t="inlineStr">
+        <is>
+          <t>1_2</t>
+        </is>
+      </c>
+      <c r="E127" t="inlineStr">
+        <is>
+          <t>패</t>
+        </is>
+      </c>
+      <c r="F127" t="inlineStr">
+        <is>
+          <t>호야국2인_848216435(1도움), 셀래스틴_852259694(1도움)</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>2026-10-15 13:14:57</t>
+        </is>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>호야국2인</t>
+        </is>
+      </c>
+      <c r="C128" t="inlineStr">
+        <is>
+          <t>셀래스틴</t>
+        </is>
+      </c>
+      <c r="D128" t="inlineStr">
+        <is>
+          <t>3_3</t>
+        </is>
+      </c>
+      <c r="E128" t="inlineStr">
+        <is>
+          <t>무</t>
+        </is>
+      </c>
+      <c r="F128" t="inlineStr">
+        <is>
+          <t>호야국2인_848216435(1도움), 호야국2인_848232293(2도움), 셀래스틴_863200458(1도움), 셀래스틴_852241461(2도움)</t>
         </is>
       </c>
     </row>

</xml_diff>